<commit_message>
Sign-off toolkit: module name of each pack in captions and workbook texts, upload column checks only for packs with uploads, walkthrough steps on screens of other packs, pack signatories, screen messages of single files and of form checks read, BRD-03 set and the configuration templates file 06 registered; BRD-01 set rebuilt with the added screen messages
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-01_New_Business/04_BIBS_TestPlan_BRD-01_New_Business_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-01_New_Business/04_BIBS_TestPlan_BRD-01_New_Business_v2.0.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Test Conditions'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Scenarios'!$A$4:$F$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Scenarios'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Cases'!$A$4:$S$479</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Test Cases'!$A$4:$S$480</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Test Cases'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Coverage'!$A$4:$J$219</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Coverage'!$4:$4</definedName>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="D24" s="12" t="n">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
     <row r="25">
@@ -1101,7 +1101,7 @@
     <row r="37">
       <c r="B37" s="19" t="inlineStr">
         <is>
-          <t>Source: FRS BRD-1 (FRS_BRD01_NEW_BUSINESS.md). 93 FRs, 122 BRD IDs, 237 test conditions, 10 scenarios, 475 test cases (206 positive, 269 negative), 311 with an automation reference.</t>
+          <t>Source: FRS BRD-1 (FRS_BRD01_NEW_BUSINESS.md). 93 FRs, 122 BRD IDs, 237 test conditions, 10 scenarios, 476 test cases (206 positive, 270 negative), 311 with an automation reference.</t>
         </is>
       </c>
     </row>
@@ -15738,7 +15738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S479"/>
+  <dimension ref="A1:S480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -51116,16 +51116,17 @@
 MSG-NB-101: "A quotation is approved by someone other than its maker" (QUOTATION_FOUR_EYES)
 MSG-NB-102: "Select the client and the product" (QUOTATION_INCOMPLETE)
 MSG-NB-103: "Select the product" (QUOTATION_INCOMPLETE)
-MSG-NB-104: "Quotation &lt;quotation no&gt; is &lt;status&gt;" (QUOTATION_NOT_EDITABLE)
+MSG-NB-104: "Quotation &lt;quotation no&gt; is &lt;&gt;" (QUOTATION_NOT_EDITABLE)
 MSG-NB-105: "The premium cannot be computed: give each item a sum insured (and a rate when the product has no default rate)" (QUOTATION_NOT_RATED)
 MSG-NB-106: "Add at least one risk item" (QUOTATION_NO_ITEMS)
 MSG-NB-107: "The period end must be after the period start" (QUOTATION_PERIOD_INVALID)
 MSG-NB-108: "The product of a quotation cannot change" (QUOTATION_PRODUCT_FIXED)
-MSG-NB-109: "The validity date cannot be in the past" (QUOTATION_VALIDITY_PAST)
-MSG-NB-110: "Version &lt;version no&gt; was submitted and is read-only" (QUOTATION_VERSION_FROZEN)
-MSG-NB-111: "The quotation is priced on version &lt;scheme version&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: save the quotation again to re-price it" (RATE_SCHEME_NOT_CURRENT)
-MSG-NB-112: "Unknown rating basis &lt;value&gt;" (RATING_BASIS_INVALID)
-MSG-NB-113: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-109: "Choose the market segment on the Client step before you submit the quotation" (QUOTATION_SEGMENT_REQUIRED)
+MSG-NB-110: "The validity date cannot be in the past" (QUOTATION_VALIDITY_PAST)
+MSG-NB-111: "Version &lt;version no&gt; was submitted and is read-only" (QUOTATION_VERSION_FROZEN)
+MSG-NB-112: "The quotation is priced on version &lt;scheme version&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: save the quotation again to re-price it" (RATE_SCHEME_NOT_CURRENT)
+MSG-NB-113: "Unknown rating basis &lt;value&gt;" (RATING_BASIS_INVALID)
+MSG-NB-114: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M444" s="12" t="inlineStr">
@@ -51201,8 +51202,8 @@
       <c r="L445" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-115: "Enter the item rate between 0 and 100"
-MSG-NB-116: "Explain why the scheme rate cannot be used"</t>
+MSG-NB-116: "Enter the item rate between 0 and 100"
+MSG-NB-117: "Explain why the scheme rate cannot be used"</t>
         </is>
       </c>
       <c r="M445" s="12" t="inlineStr">
@@ -51278,19 +51279,19 @@
       <c r="L446" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-123: "Select the client or prospect"
-MSG-NB-124: "Select the product"
-MSG-NB-125: "The period end must be after the period start"
-MSG-NB-126: "Attach the mandatory documents: &lt;missing&gt;" (MISSING_DOCUMENTS)
-MSG-NB-127: "ProposalRequest not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-128: "A PRF is approved by someone other than its maker" (PRF_FOUR_EYES)
-MSG-NB-129: "Complete the PRF header" (PRF_INCOMPLETE)
-MSG-NB-130: "Describe the risk (sections or risk items) before submitting" (PRF_INCOMPLETE)
-MSG-NB-131: "PRF &lt;prf no&gt; cannot be changed while &lt;status&gt;" (PRF_NOT_EDITABLE)
-MSG-NB-132: "No TSU rule applies to this package risk: quote it directly as a package quotation" (PRF_NOT_NEEDED)
-MSG-NB-133: "The period end must be after the period start" (PRF_PERIOD_INVALID)
-MSG-NB-134: "The product of a PRF cannot change" (PRF_PRODUCT_FIXED)
-MSG-NB-135: "Product &lt;code&gt; is not offered to segment &lt;market segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-124: "Select the client or prospect"
+MSG-NB-125: "Select the product"
+MSG-NB-126: "The period end must be after the period start"
+MSG-NB-127: "Attach the mandatory documents: &lt;missing&gt;" (MISSING_DOCUMENTS)
+MSG-NB-128: "ProposalRequest not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-129: "A PRF is approved by someone other than its maker" (PRF_FOUR_EYES)
+MSG-NB-130: "Complete the PRF header" (PRF_INCOMPLETE)
+MSG-NB-131: "Describe the risk (sections or risk items) before submitting" (PRF_INCOMPLETE)
+MSG-NB-132: "PRF &lt;prf no&gt; cannot be changed while &lt;&gt;" (PRF_NOT_EDITABLE)
+MSG-NB-133: "No TSU rule applies to this package risk: quote it directly as a package quotation" (PRF_NOT_NEEDED)
+MSG-NB-134: "The period end must be after the period start" (PRF_PERIOD_INVALID)
+MSG-NB-135: "The product of a PRF cannot change" (PRF_PRODUCT_FIXED)
+MSG-NB-136: "Product &lt;code&gt; is not offered to segment &lt;market segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M446" s="12" t="inlineStr">
@@ -51366,26 +51367,27 @@
       <c r="L447" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-145: "Attach the client's acceptance e-mail first" (ACCEPTANCE_EMAIL_REQUIRED)
-MSG-NB-146: "The proposal covers risk groups &lt;offered&gt; only" (ACCEPTANCE_GROUP_UNKNOWN)
-MSG-NB-147: "&lt;name&gt; has no placement e-mail address" (INSURER_NO_EMAIL)
-MSG-NB-148: "Insurer response not found: &lt;response id&gt;" (NOT_FOUND)
-MSG-NB-149: "Record the client's acceptance of the proposal first" (PROPOSAL_NOT_ACCEPTED)
-MSG-NB-150: "No terms of &lt;chosen insurer&gt; are recorded" (PROPOSAL_TERMS_MISSING)
-MSG-NB-151: "The proposal slip is approved by another TSU officer" (PS_FOUR_EYES)
-MSG-NB-152: "Choose the insurer (or flag the recommended one) for the proposal slip" (PS_INSURER_REQUIRED)
-MSG-NB-153: "No proposal slip has been prepared yet" (PS_NOT_PREPARED)
-MSG-NB-154: "&lt;insurer name&gt; has not quoted terms" (PS_TERMS_MISSING)
-MSG-NB-155: "The chosen terms are gone" (PS_TERMS_MISSING)
-MSG-NB-156: "Insurers are selected before the quotation slip is submitted" (QS_CLOSED)
-MSG-NB-157: "The quotation slip is approved by another TSU officer" (QS_FOUR_EYES)
-MSG-NB-158: "No quotation slip has been prepared yet" (QS_NOT_PREPARED)
-MSG-NB-159: "Select at least one insurer of the panel for the quotation slip" (QS_NO_INSURER)
-MSG-NB-160: "Insurer terms are keyed in after the quotation slip is sent" (RESPONSES_CLOSED)
-MSG-NB-161: "Only received terms can be recommended" (RESPONSE_NOT_RECEIVED)
-MSG-NB-162: "Enter the premium quoted by &lt;insurer name&gt;" (RESPONSE_PREMIUM_REQUIRED)
-MSG-NB-163: "No insurer terms have been received" (TERMS_NONE)
-MSG-NB-164: "&lt;pending&gt; insurer(s) have not answered: close the request to proceed" (TERMS_PENDING)</t>
+MSG-NB-140: "Enter the premium quoted"
+MSG-NB-147: "Attach the client's acceptance e-mail first" (ACCEPTANCE_EMAIL_REQUIRED)
+MSG-NB-148: "The proposal covers risk groups &lt;offered&gt; only" (ACCEPTANCE_GROUP_UNKNOWN)
+MSG-NB-149: "&lt;name&gt; has no placement e-mail address" (INSURER_NO_EMAIL)
+MSG-NB-150: "Insurer response not found: &lt;response id&gt;" (NOT_FOUND)
+MSG-NB-151: "Record the client's acceptance of the proposal first" (PROPOSAL_NOT_ACCEPTED)
+MSG-NB-152: "No terms of &lt;chosen insurer&gt; are recorded" (PROPOSAL_TERMS_MISSING)
+MSG-NB-153: "The proposal slip is approved by another TSU officer" (PS_FOUR_EYES)
+MSG-NB-154: "Choose the insurer (or flag the recommended one) for the proposal slip" (PS_INSURER_REQUIRED)
+MSG-NB-155: "No proposal slip has been prepared yet" (PS_NOT_PREPARED)
+MSG-NB-156: "&lt;insurer name&gt; has not quoted terms" (PS_TERMS_MISSING)
+MSG-NB-157: "The chosen terms are gone" (PS_TERMS_MISSING)
+MSG-NB-158: "Insurers are selected before the quotation slip is submitted" (QS_CLOSED)
+MSG-NB-159: "The quotation slip is approved by another TSU officer" (QS_FOUR_EYES)
+MSG-NB-160: "No quotation slip has been prepared yet" (QS_NOT_PREPARED)
+MSG-NB-161: "Select at least one insurer of the panel for the quotation slip" (QS_NO_INSURER)
+MSG-NB-162: "Insurer terms are keyed in after the quotation slip is sent" (RESPONSES_CLOSED)
+MSG-NB-163: "Only received terms can be recommended" (RESPONSE_NOT_RECEIVED)
+MSG-NB-164: "Enter the premium quoted by &lt;insurer name&gt;" (RESPONSE_PREMIUM_REQUIRED)
+MSG-NB-165: "No insurer terms have been received" (TERMS_NONE)
+MSG-NB-166: "&lt;pending&gt; insurer(s) have not answered: close the request to proceed" (TERMS_PENDING)</t>
         </is>
       </c>
       <c r="M447" s="12" t="inlineStr">
@@ -51461,12 +51463,12 @@
       <c r="L448" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-167: "Account &lt;arn&gt; is &lt;status&gt;" (ACCOUNT_NOT_ACTIVE)
-MSG-NB-168: "Product &lt;product code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
-MSG-NB-169: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
-MSG-NB-170: "Account &lt;arn&gt; is not tagged Free First Year" (FFY_NOT_TAGGED)
-MSG-NB-171: "Enter the Free First Year start" (FFY_START_REQUIRED)
-MSG-NB-172: "The payment gate of &lt;arn&gt; is passed" (PAYMENT_ARRANGEMENT_LOCKED)</t>
+MSG-NB-169: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_ACTIVE)
+MSG-NB-170: "Product &lt;product code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
+MSG-NB-171: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
+MSG-NB-172: "Account &lt;arn&gt; is not tagged Free First Year" (FFY_NOT_TAGGED)
+MSG-NB-173: "Enter the Free First Year start" (FFY_START_REQUIRED)
+MSG-NB-174: "The payment gate of &lt;arn&gt; is passed" (PAYMENT_ARRANGEMENT_LOCKED)</t>
         </is>
       </c>
       <c r="M448" s="12" t="inlineStr">
@@ -51542,17 +51544,17 @@
       <c r="L449" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-175: "Account &lt;arn&gt; is &lt;status&gt;" (ACCOUNT_NOT_EDITABLE)
-MSG-NB-176: "Account &lt;arn&gt; is &lt;status&gt;, not &lt;status&gt;" (ACCOUNT_STATUS_INVALID)
-MSG-NB-177: "The ARN must read ARN-yyyy-nnnnnn (or ARN-yyyy-nnnnnn-nn)" (ARN_INVALID)
-MSG-NB-178: "An account already has ARN &lt;given&gt;" (ARN_IN_USE)
-MSG-NB-179: "Account not found: &lt;arn&gt;" (NOT_FOUND)
-MSG-NB-180: "Account not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-181: "Account &lt;arn&gt; is set up with insurer &lt;insurer code&gt;" (PLACEMENT_INSURER_MISMATCH)
-MSG-NB-182: "Attach the issued policy (policy copy or e-policy) before direct booking" (POLICY_DOCUMENT_REQUIRED)
-MSG-NB-183: "Account &lt;arn&gt; needs &lt;term years&gt; policy number(s), one per year" (POLICY_NUMBERS_MISMATCH)
-MSG-NB-184: "TSU clearance is given before the account is validated" (TSU_CLEARANCE_CLOSED)
-MSG-NB-185: "TSU must clear the account first: &lt;reason&gt;" (TSU_CLEARANCE_REQUIRED)</t>
+MSG-NB-177: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
+MSG-NB-178: "Account &lt;arn&gt; is &lt;&gt;, not &lt;status&gt;" (ACCOUNT_STATUS_INVALID)
+MSG-NB-179: "The ARN must read ARN-yyyy-nnnnnn (or ARN-yyyy-nnnnnn-nn)" (ARN_INVALID)
+MSG-NB-180: "An account already has ARN &lt;given&gt;" (ARN_IN_USE)
+MSG-NB-181: "Account not found: &lt;arn&gt;" (NOT_FOUND)
+MSG-NB-182: "Account not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-183: "Account &lt;arn&gt; is set up with insurer &lt;insurer code&gt;" (PLACEMENT_INSURER_MISMATCH)
+MSG-NB-184: "Attach the issued policy (policy copy or e-policy) before direct booking" (POLICY_DOCUMENT_REQUIRED)
+MSG-NB-185: "Account &lt;arn&gt; needs &lt;term years&gt; policy number(s), one per year" (POLICY_NUMBERS_MISMATCH)
+MSG-NB-186: "TSU clearance is given before the account is validated" (TSU_CLEARANCE_CLOSED)
+MSG-NB-187: "TSU must clear the account first: &lt;reason&gt;" (TSU_CLEARANCE_REQUIRED)</t>
         </is>
       </c>
       <c r="M449" s="12" t="inlineStr">
@@ -51628,24 +51630,28 @@
       <c r="L450" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-188: "Duplicate risks: &lt;list&gt;"
-MSG-NB-189: "Not ready to submit: &lt;list&gt;"
-MSG-NB-190: "These risks are already on account &lt;list&gt; — open the existing account instead of creating a new one."
-MSG-NB-191: "Select the client" (ACCOUNT_CLIENT_REQUIRED)
-MSG-NB-192: "Complete the mandatory fields of &lt;product code&gt;: &lt;check&gt;" (ACCOUNT_INCOMPLETE)
-MSG-NB-193: "The period end must be after the period start" (ACCOUNT_PERIOD_INVALID)
-MSG-NB-194: "Select the product" (ACCOUNT_PRODUCT_REQUIRED)
-MSG-NB-195: "Only a renewal account names the policy it renews (&lt;renewal of ref&gt;)" (ACCOUNT_RENEWAL_OF_NOT_RENEWAL)
-MSG-NB-196: "A multi-year account needs a term of at least 2 years" (ACCOUNT_TERM_INVALID)
-MSG-NB-197: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
-MSG-NB-198: "Duplicate of existing account &lt;arns&gt;: &lt;details&gt;" (DUPLICATE_ACCOUNT)
-MSG-NB-199: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
-MSG-NB-200: "Upload the mandatory documents: &lt;check&gt;" (MISSING_DOCUMENTS)
-MSG-NB-201: "Product &lt;code&gt; carries no mortgagee" (MORTGAGE_NOT_APPLICABLE)
-MSG-NB-202: "Product &lt;code&gt; allows a term of up to &lt;max term years&gt; year(s)" (MULTI_YEAR_NOT_ALLOWED)
-MSG-NB-203: "Compute the premium (sum insured and rate of every item) first" (PREMIUM_NOT_RATED)
-MSG-NB-204: "Account &lt;arn&gt; is priced on version &lt;priced&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: update the account to re-price it or request a rate exception" (RATE_SCHEME_NOT_CURRENT)
-MSG-NB-205: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-189: "Choose the client and product to save the draft."
+MSG-NB-191: "Duplicate risks: &lt;list&gt;"
+MSG-NB-192: "Not ready to submit: &lt;list&gt;"
+MSG-NB-193: "The draft is not saved yet: click Save Draft to check it before submission."
+MSG-NB-194: "The draft was not saved: correct what the message above describes, then save the draft again."
+MSG-NB-195: "The draft was not saved: its risks are already on the account shown above. Change the risk items, or open the existing account instead."
+MSG-NB-196: "These risks are already on account &lt;list&gt; — open the existing account instead of creating a new one."
+MSG-NB-197: "Select the client" (ACCOUNT_CLIENT_REQUIRED)
+MSG-NB-198: "Complete the mandatory fields of &lt;product code&gt;: &lt;check&gt;" (ACCOUNT_INCOMPLETE)
+MSG-NB-199: "The period end must be after the period start" (ACCOUNT_PERIOD_INVALID)
+MSG-NB-200: "Select the product" (ACCOUNT_PRODUCT_REQUIRED)
+MSG-NB-201: "Only a renewal account names the policy it renews (&lt;renewal of ref&gt;)" (ACCOUNT_RENEWAL_OF_NOT_RENEWAL)
+MSG-NB-202: "A multi-year account needs a term of at least 2 years" (ACCOUNT_TERM_INVALID)
+MSG-NB-203: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
+MSG-NB-204: "Duplicate of existing account &lt;arns&gt;: &lt;details&gt;" (DUPLICATE_ACCOUNT)
+MSG-NB-205: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
+MSG-NB-206: "Upload the mandatory documents: &lt;check&gt;" (MISSING_DOCUMENTS)
+MSG-NB-207: "Product &lt;code&gt; carries no mortgagee" (MORTGAGE_NOT_APPLICABLE)
+MSG-NB-208: "Product &lt;code&gt; allows a term of up to &lt;max term years&gt; year(s)" (MULTI_YEAR_NOT_ALLOWED)
+MSG-NB-209: "Compute the premium (sum insured and rate of every item) first" (PREMIUM_NOT_RATED)
+MSG-NB-210: "Account &lt;arn&gt; is priced on version &lt;priced&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: update the account to re-price it or request a rate exception" (RATE_SCHEME_NOT_CURRENT)
+MSG-NB-211: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M450" s="12" t="inlineStr">
@@ -51721,9 +51727,9 @@
       <c r="L451" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-210: "Account &lt;arn&gt; is &lt;status&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
-MSG-NB-211: "Account &lt;arn&gt; is not paid directly to the insurer" (GATE_NOT_DIRECT_PAYMENT)
-MSG-NB-212: "Account &lt;arn&gt; must be paid: match its payment from a payment report" (GATE_REQUIRES_PAYMENT)</t>
+MSG-NB-216: "Account &lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
+MSG-NB-217: "Account &lt;arn&gt; is not paid directly to the insurer" (GATE_NOT_DIRECT_PAYMENT)
+MSG-NB-218: "Account &lt;arn&gt; must be paid: match its payment from a payment report" (GATE_REQUIRES_PAYMENT)</t>
         </is>
       </c>
       <c r="M451" s="12" t="inlineStr">
@@ -51799,15 +51805,15 @@
       <c r="L452" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-215: "Record Hold Cover Confirmation"
-MSG-NB-216: "Record Hold Cover Decline"
-MSG-NB-217: "The hold cover of &lt;arn&gt; is &lt;status&gt;" (HOLD_COVER_CLOSED)
-MSG-NB-218: "The hold cover cannot expire before it starts (&lt;start date&gt;)" (HOLD_COVER_DATES)
-MSG-NB-219: "Account &lt;arn&gt; has no open hold cover" (HOLD_COVER_NONE)
-MSG-NB-220: "A hold cover is requested while the account is being placed, not &lt;status&gt;" (HOLD_COVER_NOT_ALLOWED)
-MSG-NB-221: "Account &lt;arn&gt; already has a hold cover requested or confirmed" (HOLD_COVER_OPEN)
-MSG-NB-222: "Enter the insurer's reference" (HOLD_COVER_REFERENCE)
-MSG-NB-223: "Choose the insurer on the account first" (INSURER_NOT_SET)</t>
+MSG-NB-221: "Record Hold Cover Confirmation"
+MSG-NB-222: "Record Hold Cover Decline"
+MSG-NB-223: "The hold cover of &lt;arn&gt; is &lt;status&gt;" (HOLD_COVER_CLOSED)
+MSG-NB-224: "The hold cover cannot expire before it starts (&lt;start date&gt;)" (HOLD_COVER_DATES)
+MSG-NB-225: "Account &lt;arn&gt; has no open hold cover" (HOLD_COVER_NONE)
+MSG-NB-226: "A hold cover is requested while the account is being placed, not &lt;&gt;" (HOLD_COVER_NOT_ALLOWED)
+MSG-NB-227: "Account &lt;arn&gt; already has a hold cover requested or confirmed" (HOLD_COVER_OPEN)
+MSG-NB-228: "Enter the insurer's reference" (HOLD_COVER_REFERENCE)
+MSG-NB-229: "Choose the insurer on the account first" (INSURER_NOT_SET)</t>
         </is>
       </c>
       <c r="M452" s="12" t="inlineStr">
@@ -51883,20 +51889,20 @@
       <c r="L453" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-232: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
-MSG-NB-233: "Missing documents: &lt;missing&gt;" (DOCUMENTS_MISSING)
-MSG-NB-234: "Choose the insurer and branch on the account before placement" (INSURER_NOT_SET)
-MSG-NB-235: "Placement slip file not found: &lt;format&gt;" (NOT_FOUND)
-MSG-NB-236: "PlacementSlip not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-237: "The account is &lt;status&gt;; a slip needs Ready for placement" (NOT_READY_FOR_PLACEMENT)
-MSG-NB-238: "The payment or client confirmation is not recorded" (PAYMENT_NOT_CONFIRMED)
-MSG-NB-239: "&lt;name&gt; is set up for &lt;placement channel&gt; placements; only e-mail is available: set the insurer to e-mail placement" (PLACEMENT_CHANNEL_PARKED)
-MSG-NB-240: "Select at least one account" (PLACEMENT_NO_ACCOUNTS)
-MSG-NB-241: "Select the accounts to place" (SLIP_NO_ACCOUNTS)
-MSG-NB-242: "Placement prerequisites not met - &lt;problems&gt;" (SLIP_PREREQUISITES_UNMET)
-MSG-NB-243: "Slip &lt;display no&gt; was already replaced" (SLIP_SUPERSEDED)
-MSG-NB-244: "Slip &lt;slip no&gt; v&lt;version no&gt; was replaced by a new version" (SLIP_SUPERSEDED)
-MSG-NB-245: "TSU clearance is required (&lt;rule&gt;) and not given" (TSU_NOT_CLEARED)</t>
+MSG-NB-238: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
+MSG-NB-239: "Missing documents: &lt;missing&gt;" (DOCUMENTS_MISSING)
+MSG-NB-240: "Choose the insurer and branch on the account before placement" (INSURER_NOT_SET)
+MSG-NB-241: "Placement slip file not found: &lt;format&gt;" (NOT_FOUND)
+MSG-NB-242: "PlacementSlip not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-243: "The account is &lt;&gt;; a slip needs Ready for placement" (NOT_READY_FOR_PLACEMENT)
+MSG-NB-244: "The payment or client confirmation is not recorded" (PAYMENT_NOT_CONFIRMED)
+MSG-NB-245: "&lt;name&gt; is set up for &lt;placement channel&gt; placements; only e-mail is available: set the insurer to e-mail placement" (PLACEMENT_CHANNEL_PARKED)
+MSG-NB-246: "Select at least one account" (PLACEMENT_NO_ACCOUNTS)
+MSG-NB-247: "Select the accounts to place" (SLIP_NO_ACCOUNTS)
+MSG-NB-248: "Placement prerequisites not met - &lt;problems&gt;" (SLIP_PREREQUISITES_UNMET)
+MSG-NB-249: "Slip &lt;display no&gt; was already replaced" (SLIP_SUPERSEDED)
+MSG-NB-250: "Slip &lt;slip no&gt; v&lt;version no&gt; was replaced by a new version" (SLIP_SUPERSEDED)
+MSG-NB-251: "TSU clearance is required (&lt;rule&gt;) and not given" (TSU_NOT_CLEARED)</t>
         </is>
       </c>
       <c r="M453" s="12" t="inlineStr">
@@ -51972,10 +51978,10 @@
       <c r="L454" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-249: "Choose the billing file format XLSX or ODS" (BILLING_FORMAT)
-MSG-NB-250: "No CBG Fire account awaiting payment is left to bill" (BILLING_NOTHING_TO_BILL)
-MSG-NB-251: "Not CBG Fire accounts awaiting payment, or already billed: &lt;wanted&gt;" (BILLING_NOT_CANDIDATE)
-MSG-NB-252: "BillingBatch not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-255: "Choose the billing file format XLSX or ODS" (BILLING_FORMAT)
+MSG-NB-256: "No CBG Fire account awaiting payment is left to bill" (BILLING_NOTHING_TO_BILL)
+MSG-NB-257: "Not CBG Fire accounts awaiting payment, or already billed: &lt;wanted&gt;" (BILLING_NOT_CANDIDATE)
+MSG-NB-258: "BillingBatch not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M454" s="12" t="inlineStr">
@@ -52051,19 +52057,19 @@
       <c r="L455" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-254: "&lt;arn&gt; is &lt;status&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
-MSG-NB-255: "Billing batch &lt;batch no&gt; is closed" (BILLING_BATCH_CLOSED)
-MSG-NB-256: "BillingBatch not found: &lt;batch id&gt;" (NOT_FOUND)
-MSG-NB-257: "Payment report line not found: &lt;line id&gt;" (NOT_FOUND)
-MSG-NB-258: "PaymentReport not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-259: "Row &lt;row no&gt; is already matched to &lt;arn&gt;" (PAYMENT_LINE_MATCHED)
-MSG-NB-260: "Choose the CLPC billing batch the report answers" (PAYMENT_REPORT_BATCH_REQUIRED)
-MSG-NB-261: "Payment report &lt;report no&gt; is &lt;status&gt;" (PAYMENT_REPORT_CLOSED)
-MSG-NB-262: "The payment report has no rows" (PAYMENT_REPORT_EMPTY)
-MSG-NB-263: "The CLPC report needs a 'PN No.' or 'Loan Application No.' column" (PAYMENT_REPORT_LAYOUT)
-MSG-NB-264: "The payment report needs an 'ARN' or 'Reference' column" (PAYMENT_REPORT_LAYOUT)
-MSG-NB-265: "Row &lt;row no&gt;: '&lt;value&gt;' is not a date (yyyy-mm-dd)" (PAYMENT_REPORT_VALUE)
-MSG-NB-266: "Row &lt;row no&gt;: '&lt;value&gt;' is not an amount" (PAYMENT_REPORT_VALUE)</t>
+MSG-NB-260: "&lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
+MSG-NB-261: "Billing batch &lt;batch no&gt; is closed" (BILLING_BATCH_CLOSED)
+MSG-NB-262: "BillingBatch not found: &lt;batch id&gt;" (NOT_FOUND)
+MSG-NB-263: "Payment report line not found: &lt;line id&gt;" (NOT_FOUND)
+MSG-NB-264: "PaymentReport not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-265: "Row &lt;row no&gt; is already matched to &lt;arn&gt;" (PAYMENT_LINE_MATCHED)
+MSG-NB-266: "Choose the CLPC billing batch the report answers" (PAYMENT_REPORT_BATCH_REQUIRED)
+MSG-NB-267: "Payment report &lt;report no&gt; is &lt;status&gt;" (PAYMENT_REPORT_CLOSED)
+MSG-NB-268: "The payment report has no rows" (PAYMENT_REPORT_EMPTY)
+MSG-NB-269: "The CLPC report needs a 'PN No.' or 'Loan Application No.' column" (PAYMENT_REPORT_LAYOUT)
+MSG-NB-270: "The payment report needs an 'ARN' or 'Reference' column" (PAYMENT_REPORT_LAYOUT)
+MSG-NB-271: "Row &lt;row no&gt;: '&lt;value&gt;' is not a date (yyyy-mm-dd)" (PAYMENT_REPORT_VALUE)
+MSG-NB-272: "Row &lt;row no&gt;: '&lt;value&gt;' is not an amount" (PAYMENT_REPORT_VALUE)</t>
         </is>
       </c>
       <c r="M455" s="12" t="inlineStr">
@@ -52139,14 +52145,14 @@
       <c r="L456" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-269: "No account found for &lt;file name&gt;: choose the account (ARN)" (EPOLICY_ACCOUNT_NOT_FOUND)
-MSG-NB-270: "Account &lt;arn&gt; is &lt;status&gt;; an e-policy is received once placed" (EPOLICY_ACCOUNT_STATUS)
-MSG-NB-271: "Upload between 1 and 50 e-policies at a time" (EPOLICY_FILE_COUNT)
-MSG-NB-272: "The e-policy &lt;file name&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)
-MSG-NB-273: "This upload is &lt;status&gt;" (EPOLICY_UPLOAD_CLOSED)
-MSG-NB-274: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-275: "E-policy upload file not found: &lt;item id&gt;" (NOT_FOUND)
-MSG-NB-276: "Epolicy not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-275: "No account found for &lt;file name&gt;: choose the account (ARN)" (EPOLICY_ACCOUNT_NOT_FOUND)
+MSG-NB-276: "Account &lt;arn&gt; is &lt;&gt;; an e-policy is received once placed" (EPOLICY_ACCOUNT_STATUS)
+MSG-NB-277: "Upload between 1 and 50 e-policies at a time" (EPOLICY_FILE_COUNT)
+MSG-NB-278: "The e-policy &lt;file name&gt; is already &lt;&gt;" (EPOLICY_REVIEWED)
+MSG-NB-279: "This upload is &lt;status&gt;" (EPOLICY_UPLOAD_CLOSED)
+MSG-NB-280: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-281: "E-policy upload file not found: &lt;item id&gt;" (NOT_FOUND)
+MSG-NB-282: "Epolicy not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M456" s="12" t="inlineStr">
@@ -52222,12 +52228,12 @@
       <c r="L457" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-277: "Check before confirming &lt;list&gt;"
-MSG-NB-279: "Enter one policy number per policy year."
-MSG-NB-283: "Rejected by &lt;user&gt;: &lt;reject reason&gt;"
-MSG-NB-284: "The policy numbers must be different."
-MSG-NB-285: "Confirm the policy data of &lt;arn&gt; before sending the e-policy" (EPOLICY_NOT_CONFIRMED)
-MSG-NB-286: "The e-policy &lt;file name&gt; of &lt;arn&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)</t>
+MSG-NB-283: "Check before confirming &lt;list&gt;"
+MSG-NB-285: "Enter one policy number per policy year."
+MSG-NB-289: "Rejected by &lt;user&gt;: &lt;reject reason&gt;"
+MSG-NB-290: "The policy numbers must be different."
+MSG-NB-291: "Confirm the policy data of &lt;arn&gt; before sending the e-policy" (EPOLICY_NOT_CONFIRMED)
+MSG-NB-292: "The e-policy &lt;file name&gt; of &lt;arn&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)</t>
         </is>
       </c>
       <c r="M457" s="12" t="inlineStr">
@@ -52303,10 +52309,10 @@
       <c r="L458" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-289: "Account &lt;arn&gt; is &lt;status&gt;; it must be placed first" (IA_ACCOUNT_STATUS)
-MSG-NB-290: "Account &lt;arn&gt; has no mortgagee bank: no Insurance Advice" (IA_NOT_MORTGAGED)
-MSG-NB-291: "Select between 1 and 50 Insurance Advices" (IA_SELECTION)
-MSG-NB-292: "InsuranceAdvice not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-295: "Account &lt;arn&gt; is &lt;status&gt;; it must be placed first" (IA_ACCOUNT_STATUS)
+MSG-NB-296: "Account &lt;arn&gt; has no mortgagee bank: no Insurance Advice" (IA_NOT_MORTGAGED)
+MSG-NB-297: "Select between 1 and 50 Insurance Advices" (IA_SELECTION)
+MSG-NB-298: "InsuranceAdvice not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M458" s="12" t="inlineStr">
@@ -52382,8 +52388,8 @@
       <c r="L459" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-295: "Account &lt;arn&gt; has no contact e-mail: enter the recipient" (EPOLICY_NO_RECIPIENT)
-MSG-NB-296: "Select between 1 and 200 records" (ISSUANCE_SELECTION)</t>
+MSG-NB-301: "Account &lt;arn&gt; has no contact e-mail: enter the recipient" (EPOLICY_NO_RECIPIENT)
+MSG-NB-302: "Select between 1 and 200 records" (ISSUANCE_SELECTION)</t>
         </is>
       </c>
       <c r="M459" s="12" t="inlineStr">
@@ -52459,20 +52465,22 @@
       <c r="L460" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-299: "A negative endorsement reduces the sum insured (enter a minus)"
-MSG-NB-300: "A positive endorsement increases the sum insured"
-MSG-NB-301: "Choose the reason"
-MSG-NB-302: "Describe the cancellation"
-MSG-NB-303: "Describe the change"
-MSG-NB-304: "Enter a rate of zero or more, or leave it blank"
-MSG-NB-305: "Enter the cancellation date"
-MSG-NB-306: "Enter the change of the sum insured"
-MSG-NB-307: "Enter the effective date"
-MSG-NB-309: "No queued account to book" (BATCH_EMPTY)
-MSG-NB-310: "Select at least one account to book" (BATCH_EMPTY)
-MSG-NB-311: "The booking date &lt;booking date&gt; is in the future" (BOOKING_DATE_FUTURE)
-MSG-NB-312: "BookingQueue not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-313: "Account &lt;arn&gt; is no longer queued (&lt;status&gt;)" (QUEUE_ENTRY_CLOSED)</t>
+MSG-NB-305: "A negative endorsement reduces the sum insured (enter a minus)"
+MSG-NB-306: "A positive endorsement increases the sum insured"
+MSG-NB-307: "Choose the reason"
+MSG-NB-308: "Describe the cancellation"
+MSG-NB-309: "Describe the change"
+MSG-NB-310: "Enter a booking date that is not in the future"
+MSG-NB-311: "Enter a rate of zero or more, or leave it blank"
+MSG-NB-312: "Enter the cancellation date"
+MSG-NB-313: "Enter the change of the sum insured"
+MSG-NB-314: "Enter the effective date"
+MSG-NB-316: "The booking date cannot be in the future"
+MSG-NB-317: "No queued account to book" (BATCH_EMPTY)
+MSG-NB-318: "Select at least one account to book" (BATCH_EMPTY)
+MSG-NB-319: "The booking date &lt;booking date&gt; is in the future" (BOOKING_DATE_FUTURE)
+MSG-NB-320: "BookingQueue not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-321: "Account &lt;arn&gt; is no longer queued (&lt;status&gt;)" (QUEUE_ENTRY_CLOSED)</t>
         </is>
       </c>
       <c r="M460" s="12" t="inlineStr">
@@ -52548,24 +52556,25 @@
       <c r="L461" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-315: "Account &lt;arn&gt; has no insurer" (ACCOUNT_INSURER_MISSING)
-MSG-NB-316: "Account &lt;arn&gt; is &lt;status&gt;: only issued policies are booked" (ACCOUNT_NOT_BOOKABLE)
-MSG-NB-317: "Account &lt;arn&gt; has no period of cover" (ACCOUNT_PERIOD_MISSING)
-MSG-NB-318: "Billing number &lt;billing no&gt; of &lt;insurer code&gt; is already on invoice &lt;invoice no&gt;" (BILLING_NO_DUPLICATE)
-MSG-NB-319: "Enter the insurer billing number" (BILLING_NO_REQUIRED)
-MSG-NB-320: "The insurer billing number has at most 60 characters" (BILLING_NO_TOO_LONG)
-MSG-NB-321: "The company has no branch to book invoices" (BOOKING_BRANCH_MISSING)
-MSG-NB-322: "The booking date &lt;date&gt; is in the future" (BOOKING_DATE_FUTURE)
-MSG-NB-323: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (CLIENT_PARTY_MISSING)
-MSG-NB-324: "Enter the cost center of account &lt;arn&gt;" (COST_CENTER_REQUIRED)
-MSG-NB-325: "Account &lt;arn&gt; is already booked" (DUPLICATE_BOOKING)
-MSG-NB-326: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (INSURER_PARTY_MISSING)
-MSG-NB-327: "Each insurer appears once with a positive share" (INSURER_SHARES_INVALID)
-MSG-NB-328: "Insurer shares must add up to 100% and include the lead insurer &lt;insurer code&gt;" (INSURER_SHARES_INVALID)
-MSG-NB-329: "Invoice &lt;arn&gt;/&lt;transaction no&gt; is &lt;status&gt;" (INVOICE_ALREADY_BOOKED)
-MSG-NB-330: "No invoice" (INVOICE_NOT_FOUND)
-MSG-NB-331: "Policy year &lt;policy year&gt; of &lt;arn&gt; is not due for booking" (POLICY_YEAR_NOT_DUE)
-MSG-NB-332: "Account &lt;arn&gt; has no rated premium" (PREMIUM_NOT_RATED)</t>
+MSG-NB-323: "Enter a booking date that is not in the future"
+MSG-NB-324: "Account &lt;arn&gt; has no insurer" (ACCOUNT_INSURER_MISSING)
+MSG-NB-325: "Account &lt;arn&gt; is &lt;&gt;: only issued policies are booked" (ACCOUNT_NOT_BOOKABLE)
+MSG-NB-326: "Account &lt;arn&gt; has no period of cover" (ACCOUNT_PERIOD_MISSING)
+MSG-NB-327: "Billing number &lt;billing no&gt; of &lt;insurer code&gt; is already on invoice &lt;invoice no&gt;" (BILLING_NO_DUPLICATE)
+MSG-NB-328: "Enter the insurer billing number" (BILLING_NO_REQUIRED)
+MSG-NB-329: "The insurer billing number has at most 60 characters" (BILLING_NO_TOO_LONG)
+MSG-NB-330: "The company has no branch to book invoices" (BOOKING_BRANCH_MISSING)
+MSG-NB-331: "The booking date &lt;date&gt; is in the future" (BOOKING_DATE_FUTURE)
+MSG-NB-332: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (CLIENT_PARTY_MISSING)
+MSG-NB-333: "Enter the cost center of account &lt;arn&gt;" (COST_CENTER_REQUIRED)
+MSG-NB-334: "Account &lt;arn&gt; is already booked" (DUPLICATE_BOOKING)
+MSG-NB-335: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (INSURER_PARTY_MISSING)
+MSG-NB-336: "Each insurer appears once with a positive share" (INSURER_SHARES_INVALID)
+MSG-NB-337: "Insurer shares must add up to 100% and include the lead insurer &lt;insurer code&gt;" (INSURER_SHARES_INVALID)
+MSG-NB-338: "Invoice &lt;arn&gt;/&lt;transaction no&gt; is &lt;status&gt;" (INVOICE_ALREADY_BOOKED)
+MSG-NB-339: "No invoice" (INVOICE_NOT_FOUND)
+MSG-NB-340: "Policy year &lt;policy year&gt; of &lt;arn&gt; is not due for booking" (POLICY_YEAR_NOT_DUE)
+MSG-NB-341: "Account &lt;arn&gt; has no rated premium" (PREMIUM_NOT_RATED)</t>
         </is>
       </c>
       <c r="M461" s="12" t="inlineStr">
@@ -52641,15 +52650,15 @@
       <c r="L462" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-339: "Account &lt;arn&gt; is &lt;status&gt;: only booked accounts are endorsed" (ACCOUNT_NOT_BOOKED)
-MSG-NB-340: "A cancellation, and only a cancellation, has a kind" (CANCELLATION_KIND_REQUIRED)
-MSG-NB-341: "Enter the change of the sum insured or the premium" (ENDORSEMENT_CHANGE_REQUIRED)
-MSG-NB-342: "The effective date &lt;effective&gt; is not within a booked policy year of &lt;arn&gt;" (ENDORSEMENT_DATE_OUTSIDE_TERM)
-MSG-NB-343: "Enter the account, type, effective date and description" (ENDORSEMENT_INCOMPLETE)
-MSG-NB-344: "A negative endorsement or cancellation must return premium" (ENDORSEMENT_SIGN_MISMATCH)
-MSG-NB-345: "A positive endorsement must add premium" (ENDORSEMENT_SIGN_MISMATCH)
-MSG-NB-346: "The return premium exceeds the premium in force of policy year &lt;year&gt;" (RETURN_EXCEEDS_PREMIUM)
-MSG-NB-347: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
+MSG-NB-348: "Account &lt;arn&gt; is &lt;&gt;: only booked accounts are endorsed" (ACCOUNT_NOT_BOOKED)
+MSG-NB-349: "A cancellation, and only a cancellation, has a kind" (CANCELLATION_KIND_REQUIRED)
+MSG-NB-350: "Enter the change of the sum insured or the premium" (ENDORSEMENT_CHANGE_REQUIRED)
+MSG-NB-351: "The effective date &lt;effective&gt; is not within a booked policy year of &lt;arn&gt;" (ENDORSEMENT_DATE_OUTSIDE_TERM)
+MSG-NB-352: "Enter the account, type, effective date and description" (ENDORSEMENT_INCOMPLETE)
+MSG-NB-353: "A negative endorsement or cancellation must return premium" (ENDORSEMENT_SIGN_MISMATCH)
+MSG-NB-354: "A positive endorsement must add premium" (ENDORSEMENT_SIGN_MISMATCH)
+MSG-NB-355: "The return premium exceeds the premium in force of policy year &lt;year&gt;" (RETURN_EXCEEDS_PREMIUM)
+MSG-NB-356: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
         </is>
       </c>
       <c r="M462" s="12" t="inlineStr">
@@ -52725,14 +52734,15 @@
       <c r="L463" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-349: "E-mail: &lt;dispatch error&gt;"
-MSG-NB-351: "Service invoice &lt;si no&gt; has &lt;commission&gt; commission and &lt;vat&gt; VAT left to credit" (CREDIT_EXCEEDS_INVOICE)
-MSG-NB-352: "&lt;si no&gt; is itself a credit" (CREDIT_OF_CREDIT)
-MSG-NB-353: "Service invoice type not found: &lt;code&gt;" (NOT_FOUND)
-MSG-NB-354: "ServiceInvoice not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-355: "ServiceInvoice not found: &lt;si no&gt;" (NOT_FOUND)
-MSG-NB-356: "Service invoices of type &lt;type code&gt; are issued automatically with the early remittance incentive" (SERVICE_INVOICE_AUTOMATIC_ONLY)
-MSG-NB-357: "Service invoice type &lt;code&gt; is inactive" (SERVICE_INVOICE_TYPE_INACTIVE)</t>
+MSG-NB-358: "E-mail: &lt;dispatch error&gt;"
+MSG-NB-359: "Give the reason of the credit"
+MSG-NB-361: "Service invoice &lt;si no&gt; has &lt;commission&gt; commission and &lt;vat&gt; VAT left to credit" (CREDIT_EXCEEDS_INVOICE)
+MSG-NB-362: "&lt;si no&gt; is itself a credit" (CREDIT_OF_CREDIT)
+MSG-NB-363: "Service invoice type not found: &lt;code&gt;" (NOT_FOUND)
+MSG-NB-364: "ServiceInvoice not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-365: "ServiceInvoice not found: &lt;si no&gt;" (NOT_FOUND)
+MSG-NB-366: "Service invoices of type &lt;type code&gt; are issued automatically with the early remittance incentive" (SERVICE_INVOICE_AUTOMATIC_ONLY)
+MSG-NB-367: "Service invoice type &lt;code&gt; is inactive" (SERVICE_INVOICE_TYPE_INACTIVE)</t>
         </is>
       </c>
       <c r="M463" s="12" t="inlineStr">
@@ -52808,12 +52818,12 @@
       <c r="L464" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-360: "Service invoice type already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-361: "The period end must not be before the period start" (INCENTIVE_PERIOD_INVALID)
-MSG-NB-362: "Incentive rules are maintained in Product Maintenance &gt; Incentive Criteria" (INCENTIVE_RULES_FROZEN)
-MSG-NB-363: "AutoBookRule not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-364: "IncentiveRule not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-365: "ServiceInvoiceType not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-370: "Service invoice type already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-371: "The period end must not be before the period start" (INCENTIVE_PERIOD_INVALID)
+MSG-NB-372: "Incentive rules are maintained in Product Maintenance &gt; Incentive Criteria" (INCENTIVE_RULES_FROZEN)
+MSG-NB-373: "AutoBookRule not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-374: "IncentiveRule not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-375: "ServiceInvoiceType not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M464" s="12" t="inlineStr">
@@ -52889,31 +52899,31 @@
       <c r="L465" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-370: "Risk groups are numbers separated by ';'" (ACCEPTANCE_GROUP_INVALID)
-MSG-NB-371: "Account &lt;arn&gt; is &lt;status&gt;" (ACCOUNT_NOT_EDITABLE)
-MSG-NB-372: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
-MSG-NB-373: "Business Type must be NEW_BUSINESS or RENEWAL" (BULK_BUSINESS_TYPE_INVALID)
-MSG-NB-374: "Enter an individual's name as 'Last, First'" (BULK_CLIENT_NAME_FORMAT)
-MSG-NB-375: "Give the Client Code or the Client Name" (BULK_CLIENT_REQUIRED)
-MSG-NB-376: "This file was already uploaded as &lt;job no&gt; (&lt;file name&gt;)" (BULK_DUPLICATE_FILE)
-MSG-NB-377: "The file has no data rows" (BULK_FILE_EMPTY)
-MSG-NB-378: "The file has no header row" (BULK_FILE_EMPTY)
-MSG-NB-379: "The file has &lt;size&gt; rows; the maximum is &lt;max&gt;" (BULK_FILE_TOO_LARGE)
-MSG-NB-380: "Upload an Excel (.xlsx), OpenDocument (.ods), CSV (.csv) or text (.txt) file" (BULK_FILE_TYPE)
-MSG-NB-381: "The file cannot be read: &lt;message&gt;" (BULK_FILE_UNREADABLE)
-MSG-NB-382: "The file is not an OpenDocument spreadsheet" (BULK_FILE_UNREADABLE)
-MSG-NB-383: "Upload &lt;job no&gt; is already &lt;status&gt;" (BULK_JOB_CLOSED)
-MSG-NB-384: "Upload &lt;job no&gt; has not been committed yet" (BULK_JOB_NOT_COMPLETED)
-MSG-NB-385: "You are not allowed to use '&lt;title&gt;'" (BULK_NOT_PERMITTED)
-MSG-NB-386: "Choose the product of the upload" (BULK_PRODUCT_REQUIRED)
-MSG-NB-387: "The file does not follow the current template; missing column(s): &lt;missing&gt;" (BULK_TEMPLATE_MISMATCH)
-MSG-NB-388: "The fixed-width layout of this upload type has no fields" (BULK_TEXT_LAYOUT)
-MSG-NB-389: "The text file has no tab, pipe, semicolon or comma separated header line" (BULK_TEXT_LAYOUT)
-MSG-NB-390: "Action must be TAG or CANCEL" (FFY_ACTION_INVALID)
-MSG-NB-391: "No live account insures vehicle &lt;identifier&gt;" (FFY_VEHICLE_NOT_UNIQUE)
-MSG-NB-392: "Several accounts insure vehicle &lt;identifier&gt;: &lt;details&gt;" (FFY_VEHICLE_NOT_UNIQUE)
-MSG-NB-393: "Bulk upload type not found: &lt;code&gt;" (NOT_FOUND)
-MSG-NB-394: "BulkJob not found: &lt;job id&gt;" (NOT_FOUND)</t>
+MSG-NB-380: "Risk groups are numbers separated by ';'" (ACCEPTANCE_GROUP_INVALID)
+MSG-NB-381: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
+MSG-NB-382: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
+MSG-NB-383: "Business Type must be NEW_BUSINESS or RENEWAL" (BULK_BUSINESS_TYPE_INVALID)
+MSG-NB-384: "Enter an individual's name as 'Last, First'" (BULK_CLIENT_NAME_FORMAT)
+MSG-NB-385: "Give the Client Code or the Client Name" (BULK_CLIENT_REQUIRED)
+MSG-NB-386: "This file was already uploaded as &lt;job no&gt; (&lt;file name&gt;)" (BULK_DUPLICATE_FILE)
+MSG-NB-387: "The file has no data rows" (BULK_FILE_EMPTY)
+MSG-NB-388: "The file has no header row" (BULK_FILE_EMPTY)
+MSG-NB-389: "The file has &lt;size&gt; rows; the maximum is &lt;max&gt;" (BULK_FILE_TOO_LARGE)
+MSG-NB-390: "Upload an Excel (.xlsx), OpenDocument (.ods), CSV (.csv) or text (.txt) file" (BULK_FILE_TYPE)
+MSG-NB-391: "The file cannot be read: &lt;message&gt;" (BULK_FILE_UNREADABLE)
+MSG-NB-392: "The file is not an OpenDocument spreadsheet" (BULK_FILE_UNREADABLE)
+MSG-NB-393: "Upload &lt;job no&gt; is already &lt;status&gt;" (BULK_JOB_CLOSED)
+MSG-NB-394: "Upload &lt;job no&gt; has not been committed yet" (BULK_JOB_NOT_COMPLETED)
+MSG-NB-395: "You are not allowed to use '&lt;title&gt;'" (BULK_NOT_PERMITTED)
+MSG-NB-396: "Choose the product of the upload" (BULK_PRODUCT_REQUIRED)
+MSG-NB-397: "The file does not follow the current template; missing column(s): &lt;missing&gt;" (BULK_TEMPLATE_MISMATCH)
+MSG-NB-398: "The fixed-width layout of this upload type has no fields" (BULK_TEXT_LAYOUT)
+MSG-NB-399: "The text file has no tab, pipe, semicolon or comma separated header line" (BULK_TEXT_LAYOUT)
+MSG-NB-400: "Action must be TAG or CANCEL" (FFY_ACTION_INVALID)
+MSG-NB-401: "No live account insures vehicle &lt;identifier&gt;" (FFY_VEHICLE_NOT_UNIQUE)
+MSG-NB-402: "Several accounts insure vehicle &lt;identifier&gt;: &lt;details&gt;" (FFY_VEHICLE_NOT_UNIQUE)
+MSG-NB-403: "Bulk upload type not found: &lt;code&gt;" (NOT_FOUND)
+MSG-NB-404: "BulkJob not found: &lt;job id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M465" s="12" t="inlineStr">
@@ -52977,18 +52987,18 @@
       <c r="L466" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-396: "The file content does not match its .&lt;type&gt; type" (ATTACHMENT_CONTENT_MISMATCH)
-MSG-NB-397: "The file is empty" (ATTACHMENT_EMPTY)
-MSG-NB-398: "The file was rejected by the malware scan: &lt;detail&gt;" (ATTACHMENT_INFECTED)
-MSG-NB-399: "Stored file failed its checksum verification" (ATTACHMENT_INTEGRITY_FAILURE)
-MSG-NB-400: "The file exceeds the maximum size of &lt;to megabytes&gt; MB" (ATTACHMENT_TOO_LARGE)
-MSG-NB-401: "Only these file types are allowed: &lt;allowed extensions&gt;" (ATTACHMENT_TYPE_NOT_ALLOWED)
-MSG-NB-402: "Select between 1 and 50 documents" (DOCUMENT_FILE_COUNT)
-MSG-NB-403: "Upload between 1 and 50 files at a time" (DOCUMENT_FILE_COUNT)
-MSG-NB-404: "A reference is needed to nominate the file names" (DOCUMENT_REFERENCE_REQUIRED)
-MSG-NB-405: "Invalid entity type or id" (INVALID_ATTACHMENT_TARGET)
-MSG-NB-406: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-407: "Attachment content not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-406: "The file content does not match its .&lt;type&gt; type" (ATTACHMENT_CONTENT_MISMATCH)
+MSG-NB-407: "The file is empty" (ATTACHMENT_EMPTY)
+MSG-NB-408: "The file was rejected by the malware scan: &lt;detail&gt;" (ATTACHMENT_INFECTED)
+MSG-NB-409: "Stored file failed its checksum verification" (ATTACHMENT_INTEGRITY_FAILURE)
+MSG-NB-410: "The file exceeds the maximum size of &lt;to megabytes&gt; MB" (ATTACHMENT_TOO_LARGE)
+MSG-NB-411: "Only these file types are allowed: &lt;allowed extensions&gt;" (ATTACHMENT_TYPE_NOT_ALLOWED)
+MSG-NB-412: "Select between 1 and 50 documents" (DOCUMENT_FILE_COUNT)
+MSG-NB-413: "Upload between 1 and 50 files at a time" (DOCUMENT_FILE_COUNT)
+MSG-NB-414: "A reference is needed to nominate the file names" (DOCUMENT_REFERENCE_REQUIRED)
+MSG-NB-415: "Invalid entity type or id" (INVALID_ATTACHMENT_TARGET)
+MSG-NB-416: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-417: "Attachment content not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M466" s="12" t="inlineStr">
@@ -53052,16 +53062,16 @@
       <c r="L467" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-409: "&lt;entity type&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-410: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
-MSG-NB-411: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)
-MSG-NB-412: "Workflow not found: &lt;workflow code&gt;" (NOT_FOUND)
-MSG-NB-413: "Workflow stage not found: &lt;stage code&gt;" (NOT_FOUND)
-MSG-NB-414: "'&lt;label&gt;' must be done from the record screen" (WORKFLOW_ACTION_NOT_GENERIC)
-MSG-NB-415: "You are not allowed to '&lt;label&gt;'" (WORKFLOW_ACTION_NOT_PERMITTED)
-MSG-NB-416: "Select a reason for '&lt;label&gt;'" (WORKFLOW_REASON_REQUIRED)
-MSG-NB-417: "'&lt;action&gt;' is not allowed while &lt;reference&gt; is in stage &lt;name&gt;" (WORKFLOW_TRANSITION_NOT_ALLOWED)
-MSG-NB-418: "The item is closed" (WORK_CASE_CLOSED)</t>
+MSG-NB-419: "&lt;entity type&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-420: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
+MSG-NB-421: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)
+MSG-NB-422: "Workflow not found: &lt;workflow code&gt;" (NOT_FOUND)
+MSG-NB-423: "Workflow stage not found: &lt;stage code&gt;" (NOT_FOUND)
+MSG-NB-424: "'&lt;label&gt;' must be done from the record screen" (WORKFLOW_ACTION_NOT_GENERIC)
+MSG-NB-425: "You are not allowed to '&lt;label&gt;'" (WORKFLOW_ACTION_NOT_PERMITTED)
+MSG-NB-426: "Select a reason for '&lt;label&gt;'" (WORKFLOW_REASON_REQUIRED)
+MSG-NB-427: "'&lt;action&gt;' is not allowed while &lt;reference&gt; is in stage &lt;name&gt;" (WORKFLOW_TRANSITION_NOT_ALLOWED)
+MSG-NB-428: "The item is closed" (WORK_CASE_CLOSED)</t>
         </is>
       </c>
       <c r="M467" s="12" t="inlineStr">
@@ -53137,10 +53147,10 @@
       <c r="L468" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-421: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)
-MSG-NB-422: "&lt;assignee&gt; does not work this queue" (WORK_ASSIGNEE_NOT_ELIGIBLE)
-MSG-NB-423: "The item is closed" (WORK_CASE_CLOSED)
-MSG-NB-424: "This item is not in your queue" (WORK_CLAIM_NOT_ALLOWED)</t>
+MSG-NB-431: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)
+MSG-NB-432: "&lt;assignee&gt; does not work this queue" (WORK_ASSIGNEE_NOT_ELIGIBLE)
+MSG-NB-433: "The item is closed" (WORK_CASE_CLOSED)
+MSG-NB-434: "This item is not in your queue" (WORK_CLAIM_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M468" s="12" t="inlineStr">
@@ -53216,14 +53226,14 @@
       <c r="L469" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-427: "&lt;file name&gt; cannot be password protected. Send it as PDF, Excel or Word" (DOCUMENT_NOT_PROTECTABLE)
-MSG-NB-428: "Could not protect &lt;file name&gt;: &lt;message&gt;" (DOCUMENT_PROTECTION_FAILED)
-MSG-NB-429: "Invalid e-mail address: &lt;a&gt;" (EMAIL_ADDRESS_INVALID)
-MSG-NB-430: "Enter the &lt;field&gt;" (EMAIL_CONTENT_REQUIRED)
-MSG-NB-431: "Enter at least one recipient" (EMAIL_RECIPIENT_REQUIRED)
-MSG-NB-432: "Too many recipients" (EMAIL_TOO_MANY_RECIPIENTS)
-MSG-NB-433: "Only a failed message can be resent" (MESSAGE_NOT_FAILED)
-MSG-NB-434: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-437: "&lt;file name&gt; cannot be password protected. Send it as PDF, Excel or Word" (DOCUMENT_NOT_PROTECTABLE)
+MSG-NB-438: "Could not protect &lt;file name&gt;: &lt;message&gt;" (DOCUMENT_PROTECTION_FAILED)
+MSG-NB-439: "Invalid e-mail address: &lt;a&gt;" (EMAIL_ADDRESS_INVALID)
+MSG-NB-440: "Enter the &lt;field&gt;" (EMAIL_CONTENT_REQUIRED)
+MSG-NB-441: "Enter at least one recipient" (EMAIL_RECIPIENT_REQUIRED)
+MSG-NB-442: "Too many recipients" (EMAIL_TOO_MANY_RECIPIENTS)
+MSG-NB-443: "Only a failed message can be resent" (MESSAGE_NOT_FAILED)
+MSG-NB-444: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M469" s="12" t="inlineStr">
@@ -53299,12 +53309,17 @@
       <c r="L470" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-435: "&lt;type code&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-436: "The effective-to date is before the effective-from date" (LOV_EFFECTIVITY_INVALID)
-MSG-NB-437: "The list &lt;type code&gt; is maintained by the system" (LOV_NOT_MAINTAINABLE)
-MSG-NB-438: "'&lt;code&gt;' is not a valid value of &lt;type code&gt; on &lt;date&gt;" (LOV_VALUE_INVALID)
-MSG-NB-439: "LovType not found: &lt;type code&gt;" (NOT_FOUND)
-MSG-NB-440: "LovValue not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-446: "Enter a whole number"
+MSG-NB-447: "Enter the first valid date"
+MSG-NB-448: "Enter the label"
+MSG-NB-449: "Must not be before the first valid date"
+MSG-NB-450: "Use capital letters, digits and _ (up to 40)"
+MSG-NB-451: "&lt;type code&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-452: "The effective-to date is before the effective-from date" (LOV_EFFECTIVITY_INVALID)
+MSG-NB-453: "The list &lt;type code&gt; is maintained by the system" (LOV_NOT_MAINTAINABLE)
+MSG-NB-454: "'&lt;code&gt;' is not a valid value of &lt;type code&gt; on &lt;date&gt;" (LOV_VALUE_INVALID)
+MSG-NB-455: "LovType not found: &lt;type code&gt;" (NOT_FOUND)
+MSG-NB-456: "LovValue not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M470" s="12" t="inlineStr">
@@ -53380,13 +53395,13 @@
       <c r="L471" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-441: "Enter a whole number of bookings (0 or more)"
-MSG-NB-442: "Enter an amount of 0 or more"
-MSG-NB-443: "Enter the period"
-MSG-NB-444: "Enter the unit code or the officer username"
-MSG-NB-447: "The period end must not be before the start"
-MSG-NB-448: "Targets cannot be negative" (TARGET_NEGATIVE)
-MSG-NB-449: "The period end must not be before the period start" (TARGET_PERIOD_INVALID)</t>
+MSG-NB-457: "Enter a whole number of bookings (0 or more)"
+MSG-NB-458: "Enter an amount of 0 or more"
+MSG-NB-459: "Enter the period"
+MSG-NB-460: "Enter the unit code or the officer username"
+MSG-NB-463: "The period end must not be before the start"
+MSG-NB-464: "Targets cannot be negative" (TARGET_NEGATIVE)
+MSG-NB-465: "The period end must not be before the period start" (TARGET_PERIOD_INVALID)</t>
         </is>
       </c>
       <c r="M471" s="12" t="inlineStr">
@@ -53462,9 +53477,10 @@
       <c r="L472" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-450: "ReportVariant not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-451: "Report &lt;report code&gt; is not available to you" (REPORT_NOT_AVAILABLE)
-MSG-NB-452: "Only the user who saved a report variant may delete it" (VARIANT_NOT_OWNER)</t>
+MSG-NB-466: "Enter a name"
+MSG-NB-469: "ReportVariant not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-470: "Report &lt;report code&gt; is not available to you" (REPORT_NOT_AVAILABLE)
+MSG-NB-471: "Only the user who saved a report variant may delete it" (VARIANT_NOT_OWNER)</t>
         </is>
       </c>
       <c r="M472" s="12" t="inlineStr">
@@ -53540,13 +53556,13 @@
       <c r="L473" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-457: "This document cannot be produced in Word" (DOCUMENT_WORD_UNAVAILABLE)
-MSG-NB-458: "Document template not found: &lt;code&gt;" (NOT_FOUND)
-MSG-NB-459: "Document template not found: &lt;version no&gt;" (NOT_FOUND)
-MSG-NB-460: "Word copy of document not found: &lt;D&gt;" (NOT_FOUND)
-MSG-NB-461: "Enter the template text" (TEMPLATE_BODY_REQUIRED)
-MSG-NB-462: "The Word file needs the title in its first paragraph and the text below it" (TEMPLATE_WORD_INVALID)
-MSG-NB-463: "The file is not a Word (.docx) document" (TEMPLATE_WORD_INVALID)</t>
+MSG-NB-476: "This document cannot be produced in Word" (DOCUMENT_WORD_UNAVAILABLE)
+MSG-NB-477: "Document template not found: &lt;code&gt;" (NOT_FOUND)
+MSG-NB-478: "Document template not found: &lt;version no&gt;" (NOT_FOUND)
+MSG-NB-479: "Word copy of document not found: &lt;D&gt;" (NOT_FOUND)
+MSG-NB-480: "Enter the template text" (TEMPLATE_BODY_REQUIRED)
+MSG-NB-481: "The Word file needs the title in its first paragraph and the text below it" (TEMPLATE_WORD_INVALID)
+MSG-NB-482: "The file is not a Word (.docx) document" (TEMPLATE_WORD_INVALID)</t>
         </is>
       </c>
       <c r="M473" s="12" t="inlineStr">
@@ -53572,11 +53588,19 @@
         </is>
       </c>
       <c r="B474" s="12" t="inlineStr"/>
-      <c r="C474" s="12" t="inlineStr"/>
-      <c r="D474" s="12" t="inlineStr"/>
+      <c r="C474" s="12" t="inlineStr">
+        <is>
+          <t>FR-NB-137</t>
+        </is>
+      </c>
+      <c r="D474" s="12" t="inlineStr">
+        <is>
+          <t>BRNB.106, Data retention</t>
+        </is>
+      </c>
       <c r="E474" s="12" t="inlineStr">
         <is>
-          <t>Messages of Every screen (Common screen elements)</t>
+          <t>Messages of Data Retention (SCR-NB-43)</t>
         </is>
       </c>
       <c r="F474" s="12" t="inlineStr">
@@ -53586,15 +53610,19 @@
       </c>
       <c r="G474" s="12" t="inlineStr">
         <is>
-          <t>MKT_AO – Marketing AO (SIT/UAT user ao)</t>
+          <t>NB_APPROVER – New Business approver (SIT/UAT user approver)</t>
         </is>
       </c>
       <c r="H474" s="12" t="inlineStr">
         <is>
-          <t>Any New Business record</t>
-        </is>
-      </c>
-      <c r="I474" s="12" t="inlineStr"/>
+          <t>Setup &amp; Administration › Broking Setup › Data Retention</t>
+        </is>
+      </c>
+      <c r="I474" s="12" t="inlineStr">
+        <is>
+          <t>SCR-NB-43</t>
+        </is>
+      </c>
       <c r="J474" s="12" t="inlineStr">
         <is>
           <t>Seed data of the SIT environment.</t>
@@ -53602,23 +53630,19 @@
       </c>
       <c r="K474" s="12" t="inlineStr">
         <is>
-          <t>1. Sign in as ao.
-2. Open Any New Business record.
+          <t>1. Sign in as approver.
+2. Open Setup &amp; Administration › Broking Setup › Data Retention.
 3. For each message listed, create the condition described in the messages catalogue of the FRS (chapter 15) and run the action.</t>
         </is>
       </c>
       <c r="L474" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-466: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-NB-467: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-NB-468: "An unexpected error occurred. Quote reference &lt;reference&gt; to support." (INTERNAL_ERROR)
-MSG-NB-469: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-NB-470: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
-MSG-NB-471: "The request body is not valid JSON or has fields of the wrong type" (MALFORMED_REQUEST)
-MSG-NB-472: "No such endpoint: &lt;resource path&gt;" (NOT_FOUND)
-MSG-NB-473: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
-MSG-NB-474: "Invalid request" (VALIDATION_FAILED)</t>
+MSG-NB-484: "Between 0 and 50 years"
+MSG-NB-485: "Between 1 and 50 years"
+MSG-NB-486: "Enter a description"
+MSG-NB-487: "Enter at least one status"
+MSG-NB-490: "The &lt;record type&gt; module does not report retention candidates yet; the records will be counted once it does."</t>
         </is>
       </c>
       <c r="M474" s="12" t="inlineStr">
@@ -53644,19 +53668,11 @@
         </is>
       </c>
       <c r="B475" s="12" t="inlineStr"/>
-      <c r="C475" s="12" t="inlineStr">
-        <is>
-          <t>FR-NB-019</t>
-        </is>
-      </c>
-      <c r="D475" s="12" t="inlineStr">
-        <is>
-          <t>BRNB.039, BRNB.064, BRNB.024</t>
-        </is>
-      </c>
+      <c r="C475" s="12" t="inlineStr"/>
+      <c r="D475" s="12" t="inlineStr"/>
       <c r="E475" s="12" t="inlineStr">
         <is>
-          <t>Messages of Bulk upload wizard (SCR-NB-36): every upload type</t>
+          <t>Messages of Every screen (Common screen elements)</t>
         </is>
       </c>
       <c r="F475" s="12" t="inlineStr">
@@ -53671,14 +53687,10 @@
       </c>
       <c r="H475" s="12" t="inlineStr">
         <is>
-          <t>Client &amp; Policy › Bulk Processing › Bulk Uploads › Bulk Upload</t>
-        </is>
-      </c>
-      <c r="I475" s="12" t="inlineStr">
-        <is>
-          <t>SCR-NB-36</t>
-        </is>
-      </c>
+          <t>Any New Business record</t>
+        </is>
+      </c>
+      <c r="I475" s="12" t="inlineStr"/>
       <c r="J475" s="12" t="inlineStr">
         <is>
           <t>Seed data of the SIT environment.</t>
@@ -53687,15 +53699,22 @@
       <c r="K475" s="12" t="inlineStr">
         <is>
           <t>1. Sign in as ao.
-2. Open Client &amp; Policy › Bulk Processing › Bulk Uploads › Bulk Upload.
+2. Open Any New Business record.
 3. For each message listed, create the condition described in the messages catalogue of the FRS (chapter 15) and run the action.</t>
         </is>
       </c>
       <c r="L475" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-479: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
-MSG-NB-480: "&lt;Column&gt; is mandatory"</t>
+MSG-NB-493: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-NB-494: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-NB-495: "An unexpected error occurred. Quote reference &lt;reference&gt; to support." (INTERNAL_ERROR)
+MSG-NB-496: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-NB-497: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-NB-498: "The request body is not valid JSON or has fields of the wrong type" (MALFORMED_REQUEST)
+MSG-NB-499: "No such endpoint: &lt;resource path&gt;" (NOT_FOUND)
+MSG-NB-500: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
+MSG-NB-501: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
       </c>
       <c r="M475" s="12" t="inlineStr">
@@ -53733,7 +53752,7 @@
       </c>
       <c r="E476" s="12" t="inlineStr">
         <is>
-          <t>Messages of Bulk upload wizard (SCR-NB-36): Bulk quotation acceptance</t>
+          <t>Messages of Bulk upload wizard (SCR-NB-36): every upload type</t>
         </is>
       </c>
       <c r="F476" s="12" t="inlineStr">
@@ -53771,7 +53790,8 @@
       <c r="L476" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-481: "&lt;quotation no&gt; is &lt;status&gt;, not sent to the client"</t>
+MSG-NB-506: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
+MSG-NB-507: "&lt;Column&gt; is mandatory"</t>
         </is>
       </c>
       <c r="M476" s="12" t="inlineStr">
@@ -53809,7 +53829,7 @@
       </c>
       <c r="E477" s="12" t="inlineStr">
         <is>
-          <t>Messages of Bulk upload wizard (SCR-NB-36): Booking upload</t>
+          <t>Messages of Bulk upload wizard (SCR-NB-36): Bulk quotation acceptance</t>
         </is>
       </c>
       <c r="F477" s="12" t="inlineStr">
@@ -53847,8 +53867,7 @@
       <c r="L477" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-482: "Account &lt;arn&gt; belongs to another company"
-MSG-NB-485: "The booking date &lt;date&gt; is in the future"</t>
+MSG-NB-508: "&lt;quotation no&gt; is &lt;&gt;, not sent to the client"</t>
         </is>
       </c>
       <c r="M477" s="12" t="inlineStr">
@@ -53886,7 +53905,7 @@
       </c>
       <c r="E478" s="12" t="inlineStr">
         <is>
-          <t>Messages of Bulk upload wizard (SCR-NB-36): Bulk client creation and update</t>
+          <t>Messages of Bulk upload wizard (SCR-NB-36): Booking upload</t>
         </is>
       </c>
       <c r="F478" s="12" t="inlineStr">
@@ -53924,9 +53943,8 @@
       <c r="L478" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-483: "Client Type must be INDIVIDUAL or CORPORATE"
-MSG-NB-484: "Client code &lt;code&gt; does not exist"
-MSG-NB-486: "The row matches several clients: &lt;details&gt;"</t>
+MSG-NB-509: "Account &lt;arn&gt; belongs to another company"
+MSG-NB-512: "The booking date &lt;date&gt; is in the future"</t>
         </is>
       </c>
       <c r="M478" s="12" t="inlineStr">
@@ -53952,11 +53970,19 @@
         </is>
       </c>
       <c r="B479" s="12" t="inlineStr"/>
-      <c r="C479" s="12" t="inlineStr"/>
-      <c r="D479" s="12" t="inlineStr"/>
+      <c r="C479" s="12" t="inlineStr">
+        <is>
+          <t>FR-NB-019</t>
+        </is>
+      </c>
+      <c r="D479" s="12" t="inlineStr">
+        <is>
+          <t>BRNB.039, BRNB.064, BRNB.024</t>
+        </is>
+      </c>
       <c r="E479" s="12" t="inlineStr">
         <is>
-          <t>Messages of Several screens</t>
+          <t>Messages of Bulk upload wizard (SCR-NB-36): Bulk client creation and update</t>
         </is>
       </c>
       <c r="F479" s="12" t="inlineStr">
@@ -53971,10 +53997,14 @@
       </c>
       <c r="H479" s="12" t="inlineStr">
         <is>
-          <t>Any New Business record</t>
-        </is>
-      </c>
-      <c r="I479" s="12" t="inlineStr"/>
+          <t>Client &amp; Policy › Bulk Processing › Bulk Uploads › Bulk Upload</t>
+        </is>
+      </c>
+      <c r="I479" s="12" t="inlineStr">
+        <is>
+          <t>SCR-NB-36</t>
+        </is>
+      </c>
       <c r="J479" s="12" t="inlineStr">
         <is>
           <t>Seed data of the SIT environment.</t>
@@ -53983,25 +54013,16 @@
       <c r="K479" s="12" t="inlineStr">
         <is>
           <t>1. Sign in as ao.
-2. Open Any New Business record.
+2. Open Client &amp; Policy › Bulk Processing › Bulk Uploads › Bulk Upload.
 3. For each message listed, create the condition described in the messages catalogue of the FRS (chapter 15) and run the action.</t>
         </is>
       </c>
       <c r="L479" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-487: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
-MSG-NB-488: "Account not found: &lt;arn&gt;" (NOT_FOUND)
-MSG-NB-489: "Account not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-490: "Batch run not found: &lt;run no&gt;" (NOT_FOUND)
-MSG-NB-491: "Booked invoice not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-492: "Booked invoice not found: &lt;invoice no&gt;" (NOT_FOUND)
-MSG-NB-493: "Notification not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-494: "ProposalRequest not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-495: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-496: "Quotation not found: &lt;key&gt;" (NOT_FOUND)
-MSG-NB-497: "Quotation version not found: &lt;version no&gt;" (NOT_FOUND)
-MSG-NB-498: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)</t>
+MSG-NB-510: "Client Type must be INDIVIDUAL or CORPORATE"
+MSG-NB-511: "Client code &lt;code&gt; does not exist"
+MSG-NB-513: "The row matches several clients: &lt;details&gt;"</t>
         </is>
       </c>
       <c r="M479" s="12" t="inlineStr">
@@ -54020,12 +54041,87 @@
       <c r="R479" s="28" t="n"/>
       <c r="S479" s="12" t="n"/>
     </row>
+    <row r="480">
+      <c r="A480" s="12" t="inlineStr">
+        <is>
+          <t>TC-NB-MSG-44</t>
+        </is>
+      </c>
+      <c r="B480" s="12" t="inlineStr"/>
+      <c r="C480" s="12" t="inlineStr"/>
+      <c r="D480" s="12" t="inlineStr"/>
+      <c r="E480" s="12" t="inlineStr">
+        <is>
+          <t>Messages of Several screens</t>
+        </is>
+      </c>
+      <c r="F480" s="12" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="G480" s="12" t="inlineStr">
+        <is>
+          <t>MKT_AO – Marketing AO (SIT/UAT user ao)</t>
+        </is>
+      </c>
+      <c r="H480" s="12" t="inlineStr">
+        <is>
+          <t>Any New Business record</t>
+        </is>
+      </c>
+      <c r="I480" s="12" t="inlineStr"/>
+      <c r="J480" s="12" t="inlineStr">
+        <is>
+          <t>Seed data of the SIT environment.</t>
+        </is>
+      </c>
+      <c r="K480" s="12" t="inlineStr">
+        <is>
+          <t>1. Sign in as ao.
+2. Open Any New Business record.
+3. For each message listed, create the condition described in the messages catalogue of the FRS (chapter 15) and run the action.</t>
+        </is>
+      </c>
+      <c r="L480" s="12" t="inlineStr">
+        <is>
+          <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
+MSG-NB-514: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
+MSG-NB-515: "Account not found: &lt;arn&gt;" (NOT_FOUND)
+MSG-NB-516: "Account not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-517: "Batch run not found: &lt;run no&gt;" (NOT_FOUND)
+MSG-NB-518: "Booked invoice not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-519: "Booked invoice not found: &lt;invoice no&gt;" (NOT_FOUND)
+MSG-NB-520: "Notification not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-521: "ProposalRequest not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-522: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-523: "Quotation not found: &lt;key&gt;" (NOT_FOUND)
+MSG-NB-524: "Quotation version not found: &lt;version no&gt;" (NOT_FOUND)
+MSG-NB-525: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)</t>
+        </is>
+      </c>
+      <c r="M480" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N480" s="12" t="inlineStr"/>
+      <c r="O480" s="27" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+      <c r="P480" s="12" t="n"/>
+      <c r="Q480" s="12" t="n"/>
+      <c r="R480" s="28" t="n"/>
+      <c r="S480" s="12" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:S479"/>
+  <autoFilter ref="A4:S480"/>
   <mergeCells count="1">
     <mergeCell ref="A2:S2"/>
   </mergeCells>
-  <conditionalFormatting sqref="O5:O979">
+  <conditionalFormatting sqref="O5:O980">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
       <formula>"Pass"</formula>
     </cfRule>
@@ -54039,19 +54135,19 @@
       <formula>"N/A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:S979">
+  <conditionalFormatting sqref="A5:S980">
     <cfRule type="expression" priority="5" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="F5:F979" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="F5:F980" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'_lists'!$B$1:$B$9</formula1>
     </dataValidation>
-    <dataValidation sqref="M5:M979" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
+    <dataValidation sqref="M5:M980" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
       <formula1>'_lists'!$C$1:$C$3</formula1>
     </dataValidation>
-    <dataValidation sqref="O5:O979" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="O5:O980" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'_lists'!$D$1:$D$5</formula1>
     </dataValidation>
   </dataValidations>
@@ -58060,10 +58156,10 @@
         <v>2</v>
       </c>
       <c r="G97" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H97" s="12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I97" s="12" t="n">
         <v>3</v>
@@ -62126,10 +62222,10 @@
         <v>2</v>
       </c>
       <c r="G204" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H204" s="12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I204" s="12" t="n">
         <v>3</v>
@@ -62696,10 +62792,10 @@
         <v>2</v>
       </c>
       <c r="G219" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H219" s="12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I219" s="12" t="n">
         <v>3</v>
@@ -63704,7 +63800,7 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>TC-NB-SCR-36, TC-NB-MSG-29, TC-NB-MSG-39, TC-NB-MSG-40, TC-NB-MSG-41, TC-NB-MSG-42</t>
+          <t>TC-NB-SCR-36, TC-NB-MSG-29, TC-NB-MSG-40, TC-NB-MSG-41, TC-NB-MSG-42, TC-NB-MSG-43</t>
         </is>
       </c>
     </row>
@@ -63875,11 +63971,11 @@
         </is>
       </c>
       <c r="D47" s="12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E47" s="12" t="inlineStr">
         <is>
-          <t>TC-NB-137.1-01, TC-NB-137.2-01, TC-NB-137.2-02, TC-NB-SCR-43</t>
+          <t>TC-NB-137.1-01, TC-NB-137.2-01, TC-NB-137.2-02, TC-NB-SCR-43, TC-NB-MSG-38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BRD-01 sign-off pack v2.0 retaken after the screen and document corrections: 144 screenshots, walkthrough and quotation segment texts, messages of the new screen texts, the six files rebuilt
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-01_New_Business/04_BIBS_TestPlan_BRD-01_New_Business_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-01_New_Business/04_BIBS_TestPlan_BRD-01_New_Business_v2.0.xlsx
@@ -47253,7 +47253,7 @@
       <c r="L396" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-06 New Quotation and Edit Quotation of the FRS.
-Fields in this order: 1 Client or prospect (Look-up, mandatory Y); 2 Market segment (Drop-down, mandatory N); 3 Source channel (Drop-down, mandatory N); 4 Product (Drop-down, mandatory Y); 5 Insurer (Drop-down, mandatory N); 6 Insurer branch (LGT) (Drop-down, mandatory N); 7 Period from (Date, mandatory N); 8 Period to (Date, mandatory N); 9 Valid until (Date, mandatory N); 10 Rating basis (Drop-down, mandatory N); 11 Premium paid directly to the insurer (Check box, mandatory N (shown for products eligible for direct payment)); 12 Remarks (Text, mandatory N); 13 Vehicle: Plate no., Conduction sticker, Engine no., Chassis no. (Text, mandatory Cond.: plate no. or conduction sticker per vehicle; others per the product's field rules); 14 Vehicle: Make, Model, Year model, Body type, Colour, Seats (Text / Number / Drop-down, mandatory Cond.: per the product's field rules); 15 Location: Address, City, Province, Occupancy, Construction class (Text / Drop-down, mandatory Address Y for a location; others per the field rules); 16 Location: Insured items (description, sum insured) (Table, mandatory N); 17 Person: Name, Birth date, Relationship (Text / Date, mandatory Name Y for a person); 18 Description (Text, mandatory N); 19 Sum insured (Amount, mandatory Y to rate the premium); 20 Rate % (non-motor) (Number, mandatory N); 21 Excess BI limit, PD limit (motor) (Amount, mandatory N); 22 Item n: risk group (Number, mandatory N (shown with 2 or more items)); 23 Live premium (Display, mandatory -); 24 TSU routing notice (Banner, mandatory -); 25 Summary (Display, mandatory -).
+Fields in this order: 1 Client or prospect (Look-up, mandatory Y); 2 Market segment (Drop-down, mandatory Y at submission); 3 Source channel (Drop-down, mandatory N); 4 Product (Drop-down, mandatory Y); 5 Insurer (Drop-down, mandatory N); 6 Insurer branch (LGT) (Drop-down, mandatory N); 7 Period from (Date, mandatory N); 8 Period to (Date, mandatory N); 9 Valid until (Date, mandatory N); 10 Rating basis (Drop-down, mandatory N); 11 Premium paid directly to the insurer (Check box, mandatory N (shown for products eligible for direct payment)); 12 Remarks (Text, mandatory N); 13 Vehicle: Plate no., Conduction sticker, Engine no., Chassis no. (Text, mandatory Cond.: plate no. or conduction sticker per vehicle; others per the product's field rules); 14 Vehicle: Make, Model, Year model, Body type, Colour, Seats (Text / Number / Drop-down, mandatory Cond.: per the product's field rules); 15 Location: Address, City, Province, Occupancy, Construction class (Text / Drop-down, mandatory Address Y for a location; others per the field rules); 16 Location: Insured items (description, sum insured) (Table, mandatory N); 17 Person: Name, Birth date, Relationship (Text / Date, mandatory Name Y for a person); 18 Description (Text, mandatory N); 19 Sum insured (Amount, mandatory Y to rate the premium); 20 Rate % (non-motor) (Number, mandatory N); 21 Excess BI limit, PD limit (motor) (Amount, mandatory N); 22 Item n: risk group (Number, mandatory N (shown with 2 or more items)); 23 Live premium (Display, mandatory -); 24 TSU routing notice (Banner, mandatory -); 25 Summary (Display, mandatory -).
 Actions: Save Draft; Next / Back; Submit for Review.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -51116,16 +51116,17 @@
 MSG-NB-101: "A quotation is approved by someone other than its maker" (QUOTATION_FOUR_EYES)
 MSG-NB-102: "Select the client and the product" (QUOTATION_INCOMPLETE)
 MSG-NB-103: "Select the product" (QUOTATION_INCOMPLETE)
-MSG-NB-104: "Quotation &lt;quotation no&gt; is &lt;status&gt;" (QUOTATION_NOT_EDITABLE)
+MSG-NB-104: "Quotation &lt;quotation no&gt; is &lt;&gt;" (QUOTATION_NOT_EDITABLE)
 MSG-NB-105: "The premium cannot be computed: give each item a sum insured (and a rate when the product has no default rate)" (QUOTATION_NOT_RATED)
 MSG-NB-106: "Add at least one risk item" (QUOTATION_NO_ITEMS)
 MSG-NB-107: "The period end must be after the period start" (QUOTATION_PERIOD_INVALID)
 MSG-NB-108: "The product of a quotation cannot change" (QUOTATION_PRODUCT_FIXED)
-MSG-NB-109: "The validity date cannot be in the past" (QUOTATION_VALIDITY_PAST)
-MSG-NB-110: "Version &lt;version no&gt; was submitted and is read-only" (QUOTATION_VERSION_FROZEN)
-MSG-NB-111: "The quotation is priced on version &lt;scheme version&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: save the quotation again to re-price it" (RATE_SCHEME_NOT_CURRENT)
-MSG-NB-112: "Unknown rating basis &lt;value&gt;" (RATING_BASIS_INVALID)
-MSG-NB-113: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-109: "Choose the market segment on the Client step before you submit the quotation" (QUOTATION_SEGMENT_REQUIRED)
+MSG-NB-110: "The validity date cannot be in the past" (QUOTATION_VALIDITY_PAST)
+MSG-NB-111: "Version &lt;version no&gt; was submitted and is read-only" (QUOTATION_VERSION_FROZEN)
+MSG-NB-112: "The quotation is priced on version &lt;scheme version&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: save the quotation again to re-price it" (RATE_SCHEME_NOT_CURRENT)
+MSG-NB-113: "Unknown rating basis &lt;value&gt;" (RATING_BASIS_INVALID)
+MSG-NB-114: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M444" s="12" t="inlineStr">
@@ -51201,8 +51202,8 @@
       <c r="L445" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-115: "Enter the item rate between 0 and 100"
-MSG-NB-116: "Explain why the scheme rate cannot be used"</t>
+MSG-NB-116: "Enter the item rate between 0 and 100"
+MSG-NB-117: "Explain why the scheme rate cannot be used"</t>
         </is>
       </c>
       <c r="M445" s="12" t="inlineStr">
@@ -51278,19 +51279,19 @@
       <c r="L446" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-123: "Select the client or prospect"
-MSG-NB-124: "Select the product"
-MSG-NB-125: "The period end must be after the period start"
-MSG-NB-126: "Attach the mandatory documents: &lt;missing&gt;" (MISSING_DOCUMENTS)
-MSG-NB-127: "ProposalRequest not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-128: "A PRF is approved by someone other than its maker" (PRF_FOUR_EYES)
-MSG-NB-129: "Complete the PRF header" (PRF_INCOMPLETE)
-MSG-NB-130: "Describe the risk (sections or risk items) before submitting" (PRF_INCOMPLETE)
-MSG-NB-131: "PRF &lt;prf no&gt; cannot be changed while &lt;status&gt;" (PRF_NOT_EDITABLE)
-MSG-NB-132: "No TSU rule applies to this package risk: quote it directly as a package quotation" (PRF_NOT_NEEDED)
-MSG-NB-133: "The period end must be after the period start" (PRF_PERIOD_INVALID)
-MSG-NB-134: "The product of a PRF cannot change" (PRF_PRODUCT_FIXED)
-MSG-NB-135: "Product &lt;code&gt; is not offered to segment &lt;market segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-124: "Select the client or prospect"
+MSG-NB-125: "Select the product"
+MSG-NB-126: "The period end must be after the period start"
+MSG-NB-127: "Attach the mandatory documents: &lt;missing&gt;" (MISSING_DOCUMENTS)
+MSG-NB-128: "ProposalRequest not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-129: "A PRF is approved by someone other than its maker" (PRF_FOUR_EYES)
+MSG-NB-130: "Complete the PRF header" (PRF_INCOMPLETE)
+MSG-NB-131: "Describe the risk (sections or risk items) before submitting" (PRF_INCOMPLETE)
+MSG-NB-132: "PRF &lt;prf no&gt; cannot be changed while &lt;&gt;" (PRF_NOT_EDITABLE)
+MSG-NB-133: "No TSU rule applies to this package risk: quote it directly as a package quotation" (PRF_NOT_NEEDED)
+MSG-NB-134: "The period end must be after the period start" (PRF_PERIOD_INVALID)
+MSG-NB-135: "The product of a PRF cannot change" (PRF_PRODUCT_FIXED)
+MSG-NB-136: "Product &lt;code&gt; is not offered to segment &lt;market segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M446" s="12" t="inlineStr">
@@ -51366,26 +51367,26 @@
       <c r="L447" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-145: "Attach the client's acceptance e-mail first" (ACCEPTANCE_EMAIL_REQUIRED)
-MSG-NB-146: "The proposal covers risk groups &lt;offered&gt; only" (ACCEPTANCE_GROUP_UNKNOWN)
-MSG-NB-147: "&lt;name&gt; has no placement e-mail address" (INSURER_NO_EMAIL)
-MSG-NB-148: "Insurer response not found: &lt;response id&gt;" (NOT_FOUND)
-MSG-NB-149: "Record the client's acceptance of the proposal first" (PROPOSAL_NOT_ACCEPTED)
-MSG-NB-150: "No terms of &lt;chosen insurer&gt; are recorded" (PROPOSAL_TERMS_MISSING)
-MSG-NB-151: "The proposal slip is approved by another TSU officer" (PS_FOUR_EYES)
-MSG-NB-152: "Choose the insurer (or flag the recommended one) for the proposal slip" (PS_INSURER_REQUIRED)
-MSG-NB-153: "No proposal slip has been prepared yet" (PS_NOT_PREPARED)
-MSG-NB-154: "&lt;insurer name&gt; has not quoted terms" (PS_TERMS_MISSING)
-MSG-NB-155: "The chosen terms are gone" (PS_TERMS_MISSING)
-MSG-NB-156: "Insurers are selected before the quotation slip is submitted" (QS_CLOSED)
-MSG-NB-157: "The quotation slip is approved by another TSU officer" (QS_FOUR_EYES)
-MSG-NB-158: "No quotation slip has been prepared yet" (QS_NOT_PREPARED)
-MSG-NB-159: "Select at least one insurer of the panel for the quotation slip" (QS_NO_INSURER)
-MSG-NB-160: "Insurer terms are keyed in after the quotation slip is sent" (RESPONSES_CLOSED)
-MSG-NB-161: "Only received terms can be recommended" (RESPONSE_NOT_RECEIVED)
-MSG-NB-162: "Enter the premium quoted by &lt;insurer name&gt;" (RESPONSE_PREMIUM_REQUIRED)
-MSG-NB-163: "No insurer terms have been received" (TERMS_NONE)
-MSG-NB-164: "&lt;pending&gt; insurer(s) have not answered: close the request to proceed" (TERMS_PENDING)</t>
+MSG-NB-146: "Attach the client's acceptance e-mail first" (ACCEPTANCE_EMAIL_REQUIRED)
+MSG-NB-147: "The proposal covers risk groups &lt;offered&gt; only" (ACCEPTANCE_GROUP_UNKNOWN)
+MSG-NB-148: "&lt;name&gt; has no placement e-mail address" (INSURER_NO_EMAIL)
+MSG-NB-149: "Insurer response not found: &lt;response id&gt;" (NOT_FOUND)
+MSG-NB-150: "Record the client's acceptance of the proposal first" (PROPOSAL_NOT_ACCEPTED)
+MSG-NB-151: "No terms of &lt;chosen insurer&gt; are recorded" (PROPOSAL_TERMS_MISSING)
+MSG-NB-152: "The proposal slip is approved by another TSU officer" (PS_FOUR_EYES)
+MSG-NB-153: "Choose the insurer (or flag the recommended one) for the proposal slip" (PS_INSURER_REQUIRED)
+MSG-NB-154: "No proposal slip has been prepared yet" (PS_NOT_PREPARED)
+MSG-NB-155: "&lt;insurer name&gt; has not quoted terms" (PS_TERMS_MISSING)
+MSG-NB-156: "The chosen terms are gone" (PS_TERMS_MISSING)
+MSG-NB-157: "Insurers are selected before the quotation slip is submitted" (QS_CLOSED)
+MSG-NB-158: "The quotation slip is approved by another TSU officer" (QS_FOUR_EYES)
+MSG-NB-159: "No quotation slip has been prepared yet" (QS_NOT_PREPARED)
+MSG-NB-160: "Select at least one insurer of the panel for the quotation slip" (QS_NO_INSURER)
+MSG-NB-161: "Insurer terms are keyed in after the quotation slip is sent" (RESPONSES_CLOSED)
+MSG-NB-162: "Only received terms can be recommended" (RESPONSE_NOT_RECEIVED)
+MSG-NB-163: "Enter the premium quoted by &lt;insurer name&gt;" (RESPONSE_PREMIUM_REQUIRED)
+MSG-NB-164: "No insurer terms have been received" (TERMS_NONE)
+MSG-NB-165: "&lt;pending&gt; insurer(s) have not answered: close the request to proceed" (TERMS_PENDING)</t>
         </is>
       </c>
       <c r="M447" s="12" t="inlineStr">
@@ -51461,12 +51462,12 @@
       <c r="L448" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-167: "Account &lt;arn&gt; is &lt;status&gt;" (ACCOUNT_NOT_ACTIVE)
-MSG-NB-168: "Product &lt;product code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
-MSG-NB-169: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
-MSG-NB-170: "Account &lt;arn&gt; is not tagged Free First Year" (FFY_NOT_TAGGED)
-MSG-NB-171: "Enter the Free First Year start" (FFY_START_REQUIRED)
-MSG-NB-172: "The payment gate of &lt;arn&gt; is passed" (PAYMENT_ARRANGEMENT_LOCKED)</t>
+MSG-NB-168: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_ACTIVE)
+MSG-NB-169: "Product &lt;product code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
+MSG-NB-170: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
+MSG-NB-171: "Account &lt;arn&gt; is not tagged Free First Year" (FFY_NOT_TAGGED)
+MSG-NB-172: "Enter the Free First Year start" (FFY_START_REQUIRED)
+MSG-NB-173: "The payment gate of &lt;arn&gt; is passed" (PAYMENT_ARRANGEMENT_LOCKED)</t>
         </is>
       </c>
       <c r="M448" s="12" t="inlineStr">
@@ -51542,17 +51543,17 @@
       <c r="L449" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-175: "Account &lt;arn&gt; is &lt;status&gt;" (ACCOUNT_NOT_EDITABLE)
-MSG-NB-176: "Account &lt;arn&gt; is &lt;status&gt;, not &lt;status&gt;" (ACCOUNT_STATUS_INVALID)
-MSG-NB-177: "The ARN must read ARN-yyyy-nnnnnn (or ARN-yyyy-nnnnnn-nn)" (ARN_INVALID)
-MSG-NB-178: "An account already has ARN &lt;given&gt;" (ARN_IN_USE)
-MSG-NB-179: "Account not found: &lt;arn&gt;" (NOT_FOUND)
-MSG-NB-180: "Account not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-181: "Account &lt;arn&gt; is set up with insurer &lt;insurer code&gt;" (PLACEMENT_INSURER_MISMATCH)
-MSG-NB-182: "Attach the issued policy (policy copy or e-policy) before direct booking" (POLICY_DOCUMENT_REQUIRED)
-MSG-NB-183: "Account &lt;arn&gt; needs &lt;term years&gt; policy number(s), one per year" (POLICY_NUMBERS_MISMATCH)
-MSG-NB-184: "TSU clearance is given before the account is validated" (TSU_CLEARANCE_CLOSED)
-MSG-NB-185: "TSU must clear the account first: &lt;reason&gt;" (TSU_CLEARANCE_REQUIRED)</t>
+MSG-NB-176: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
+MSG-NB-177: "Account &lt;arn&gt; is &lt;&gt;, not &lt;status&gt;" (ACCOUNT_STATUS_INVALID)
+MSG-NB-178: "The ARN must read ARN-yyyy-nnnnnn (or ARN-yyyy-nnnnnn-nn)" (ARN_INVALID)
+MSG-NB-179: "An account already has ARN &lt;given&gt;" (ARN_IN_USE)
+MSG-NB-180: "Account not found: &lt;arn&gt;" (NOT_FOUND)
+MSG-NB-181: "Account not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-182: "Account &lt;arn&gt; is set up with insurer &lt;insurer code&gt;" (PLACEMENT_INSURER_MISMATCH)
+MSG-NB-183: "Attach the issued policy (policy copy or e-policy) before direct booking" (POLICY_DOCUMENT_REQUIRED)
+MSG-NB-184: "Account &lt;arn&gt; needs &lt;term years&gt; policy number(s), one per year" (POLICY_NUMBERS_MISMATCH)
+MSG-NB-185: "TSU clearance is given before the account is validated" (TSU_CLEARANCE_CLOSED)
+MSG-NB-186: "TSU must clear the account first: &lt;reason&gt;" (TSU_CLEARANCE_REQUIRED)</t>
         </is>
       </c>
       <c r="M449" s="12" t="inlineStr">
@@ -51628,24 +51629,28 @@
       <c r="L450" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-188: "Duplicate risks: &lt;list&gt;"
-MSG-NB-189: "Not ready to submit: &lt;list&gt;"
-MSG-NB-190: "These risks are already on account &lt;list&gt; — open the existing account instead of creating a new one."
-MSG-NB-191: "Select the client" (ACCOUNT_CLIENT_REQUIRED)
-MSG-NB-192: "Complete the mandatory fields of &lt;product code&gt;: &lt;check&gt;" (ACCOUNT_INCOMPLETE)
-MSG-NB-193: "The period end must be after the period start" (ACCOUNT_PERIOD_INVALID)
-MSG-NB-194: "Select the product" (ACCOUNT_PRODUCT_REQUIRED)
-MSG-NB-195: "Only a renewal account names the policy it renews (&lt;renewal of ref&gt;)" (ACCOUNT_RENEWAL_OF_NOT_RENEWAL)
-MSG-NB-196: "A multi-year account needs a term of at least 2 years" (ACCOUNT_TERM_INVALID)
-MSG-NB-197: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
-MSG-NB-198: "Duplicate of existing account &lt;arns&gt;: &lt;details&gt;" (DUPLICATE_ACCOUNT)
-MSG-NB-199: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
-MSG-NB-200: "Upload the mandatory documents: &lt;check&gt;" (MISSING_DOCUMENTS)
-MSG-NB-201: "Product &lt;code&gt; carries no mortgagee" (MORTGAGE_NOT_APPLICABLE)
-MSG-NB-202: "Product &lt;code&gt; allows a term of up to &lt;max term years&gt; year(s)" (MULTI_YEAR_NOT_ALLOWED)
-MSG-NB-203: "Compute the premium (sum insured and rate of every item) first" (PREMIUM_NOT_RATED)
-MSG-NB-204: "Account &lt;arn&gt; is priced on version &lt;priced&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: update the account to re-price it or request a rate exception" (RATE_SCHEME_NOT_CURRENT)
-MSG-NB-205: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-188: "Choose the client and product to save the draft."
+MSG-NB-190: "Duplicate risks: &lt;list&gt;"
+MSG-NB-191: "Not ready to submit: &lt;list&gt;"
+MSG-NB-192: "The draft is not saved yet: click Save Draft to check it before submission."
+MSG-NB-193: "The draft was not saved: correct what the message above describes, then save the draft again."
+MSG-NB-194: "The draft was not saved: its risks are already on the account shown above. Change the risk items, or open the existing account instead."
+MSG-NB-195: "These risks are already on account &lt;list&gt; — open the existing account instead of creating a new one."
+MSG-NB-196: "Select the client" (ACCOUNT_CLIENT_REQUIRED)
+MSG-NB-197: "Complete the mandatory fields of &lt;product code&gt;: &lt;check&gt;" (ACCOUNT_INCOMPLETE)
+MSG-NB-198: "The period end must be after the period start" (ACCOUNT_PERIOD_INVALID)
+MSG-NB-199: "Select the product" (ACCOUNT_PRODUCT_REQUIRED)
+MSG-NB-200: "Only a renewal account names the policy it renews (&lt;renewal of ref&gt;)" (ACCOUNT_RENEWAL_OF_NOT_RENEWAL)
+MSG-NB-201: "A multi-year account needs a term of at least 2 years" (ACCOUNT_TERM_INVALID)
+MSG-NB-202: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
+MSG-NB-203: "Duplicate of existing account &lt;arns&gt;: &lt;details&gt;" (DUPLICATE_ACCOUNT)
+MSG-NB-204: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
+MSG-NB-205: "Upload the mandatory documents: &lt;check&gt;" (MISSING_DOCUMENTS)
+MSG-NB-206: "Product &lt;code&gt; carries no mortgagee" (MORTGAGE_NOT_APPLICABLE)
+MSG-NB-207: "Product &lt;code&gt; allows a term of up to &lt;max term years&gt; year(s)" (MULTI_YEAR_NOT_ALLOWED)
+MSG-NB-208: "Compute the premium (sum insured and rate of every item) first" (PREMIUM_NOT_RATED)
+MSG-NB-209: "Account &lt;arn&gt; is priced on version &lt;priced&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: update the account to re-price it or request a rate exception" (RATE_SCHEME_NOT_CURRENT)
+MSG-NB-210: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M450" s="12" t="inlineStr">
@@ -51721,9 +51726,9 @@
       <c r="L451" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-210: "Account &lt;arn&gt; is &lt;status&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
-MSG-NB-211: "Account &lt;arn&gt; is not paid directly to the insurer" (GATE_NOT_DIRECT_PAYMENT)
-MSG-NB-212: "Account &lt;arn&gt; must be paid: match its payment from a payment report" (GATE_REQUIRES_PAYMENT)</t>
+MSG-NB-215: "Account &lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
+MSG-NB-216: "Account &lt;arn&gt; is not paid directly to the insurer" (GATE_NOT_DIRECT_PAYMENT)
+MSG-NB-217: "Account &lt;arn&gt; must be paid: match its payment from a payment report" (GATE_REQUIRES_PAYMENT)</t>
         </is>
       </c>
       <c r="M451" s="12" t="inlineStr">
@@ -51799,15 +51804,15 @@
       <c r="L452" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-215: "Record Hold Cover Confirmation"
-MSG-NB-216: "Record Hold Cover Decline"
-MSG-NB-217: "The hold cover of &lt;arn&gt; is &lt;status&gt;" (HOLD_COVER_CLOSED)
-MSG-NB-218: "The hold cover cannot expire before it starts (&lt;start date&gt;)" (HOLD_COVER_DATES)
-MSG-NB-219: "Account &lt;arn&gt; has no open hold cover" (HOLD_COVER_NONE)
-MSG-NB-220: "A hold cover is requested while the account is being placed, not &lt;status&gt;" (HOLD_COVER_NOT_ALLOWED)
-MSG-NB-221: "Account &lt;arn&gt; already has a hold cover requested or confirmed" (HOLD_COVER_OPEN)
-MSG-NB-222: "Enter the insurer's reference" (HOLD_COVER_REFERENCE)
-MSG-NB-223: "Choose the insurer on the account first" (INSURER_NOT_SET)</t>
+MSG-NB-220: "Record Hold Cover Confirmation"
+MSG-NB-221: "Record Hold Cover Decline"
+MSG-NB-222: "The hold cover of &lt;arn&gt; is &lt;status&gt;" (HOLD_COVER_CLOSED)
+MSG-NB-223: "The hold cover cannot expire before it starts (&lt;start date&gt;)" (HOLD_COVER_DATES)
+MSG-NB-224: "Account &lt;arn&gt; has no open hold cover" (HOLD_COVER_NONE)
+MSG-NB-225: "A hold cover is requested while the account is being placed, not &lt;&gt;" (HOLD_COVER_NOT_ALLOWED)
+MSG-NB-226: "Account &lt;arn&gt; already has a hold cover requested or confirmed" (HOLD_COVER_OPEN)
+MSG-NB-227: "Enter the insurer's reference" (HOLD_COVER_REFERENCE)
+MSG-NB-228: "Choose the insurer on the account first" (INSURER_NOT_SET)</t>
         </is>
       </c>
       <c r="M452" s="12" t="inlineStr">
@@ -51883,20 +51888,20 @@
       <c r="L453" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-232: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
-MSG-NB-233: "Missing documents: &lt;missing&gt;" (DOCUMENTS_MISSING)
-MSG-NB-234: "Choose the insurer and branch on the account before placement" (INSURER_NOT_SET)
-MSG-NB-235: "Placement slip file not found: &lt;format&gt;" (NOT_FOUND)
-MSG-NB-236: "PlacementSlip not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-237: "The account is &lt;status&gt;; a slip needs Ready for placement" (NOT_READY_FOR_PLACEMENT)
-MSG-NB-238: "The payment or client confirmation is not recorded" (PAYMENT_NOT_CONFIRMED)
-MSG-NB-239: "&lt;name&gt; is set up for &lt;placement channel&gt; placements; only e-mail is available: set the insurer to e-mail placement" (PLACEMENT_CHANNEL_PARKED)
-MSG-NB-240: "Select at least one account" (PLACEMENT_NO_ACCOUNTS)
-MSG-NB-241: "Select the accounts to place" (SLIP_NO_ACCOUNTS)
-MSG-NB-242: "Placement prerequisites not met - &lt;problems&gt;" (SLIP_PREREQUISITES_UNMET)
-MSG-NB-243: "Slip &lt;display no&gt; was already replaced" (SLIP_SUPERSEDED)
-MSG-NB-244: "Slip &lt;slip no&gt; v&lt;version no&gt; was replaced by a new version" (SLIP_SUPERSEDED)
-MSG-NB-245: "TSU clearance is required (&lt;rule&gt;) and not given" (TSU_NOT_CLEARED)</t>
+MSG-NB-237: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
+MSG-NB-238: "Missing documents: &lt;missing&gt;" (DOCUMENTS_MISSING)
+MSG-NB-239: "Choose the insurer and branch on the account before placement" (INSURER_NOT_SET)
+MSG-NB-240: "Placement slip file not found: &lt;format&gt;" (NOT_FOUND)
+MSG-NB-241: "PlacementSlip not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-242: "The account is &lt;&gt;; a slip needs Ready for placement" (NOT_READY_FOR_PLACEMENT)
+MSG-NB-243: "The payment or client confirmation is not recorded" (PAYMENT_NOT_CONFIRMED)
+MSG-NB-244: "&lt;name&gt; is set up for &lt;placement channel&gt; placements; only e-mail is available: set the insurer to e-mail placement" (PLACEMENT_CHANNEL_PARKED)
+MSG-NB-245: "Select at least one account" (PLACEMENT_NO_ACCOUNTS)
+MSG-NB-246: "Select the accounts to place" (SLIP_NO_ACCOUNTS)
+MSG-NB-247: "Placement prerequisites not met - &lt;problems&gt;" (SLIP_PREREQUISITES_UNMET)
+MSG-NB-248: "Slip &lt;display no&gt; was already replaced" (SLIP_SUPERSEDED)
+MSG-NB-249: "Slip &lt;slip no&gt; v&lt;version no&gt; was replaced by a new version" (SLIP_SUPERSEDED)
+MSG-NB-250: "TSU clearance is required (&lt;rule&gt;) and not given" (TSU_NOT_CLEARED)</t>
         </is>
       </c>
       <c r="M453" s="12" t="inlineStr">
@@ -51972,10 +51977,10 @@
       <c r="L454" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-249: "Choose the billing file format XLSX or ODS" (BILLING_FORMAT)
-MSG-NB-250: "No CBG Fire account awaiting payment is left to bill" (BILLING_NOTHING_TO_BILL)
-MSG-NB-251: "Not CBG Fire accounts awaiting payment, or already billed: &lt;wanted&gt;" (BILLING_NOT_CANDIDATE)
-MSG-NB-252: "BillingBatch not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-254: "Choose the billing file format XLSX or ODS" (BILLING_FORMAT)
+MSG-NB-255: "No CBG Fire account awaiting payment is left to bill" (BILLING_NOTHING_TO_BILL)
+MSG-NB-256: "Not CBG Fire accounts awaiting payment, or already billed: &lt;wanted&gt;" (BILLING_NOT_CANDIDATE)
+MSG-NB-257: "BillingBatch not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M454" s="12" t="inlineStr">
@@ -52051,19 +52056,19 @@
       <c r="L455" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-254: "&lt;arn&gt; is &lt;status&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
-MSG-NB-255: "Billing batch &lt;batch no&gt; is closed" (BILLING_BATCH_CLOSED)
-MSG-NB-256: "BillingBatch not found: &lt;batch id&gt;" (NOT_FOUND)
-MSG-NB-257: "Payment report line not found: &lt;line id&gt;" (NOT_FOUND)
-MSG-NB-258: "PaymentReport not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-259: "Row &lt;row no&gt; is already matched to &lt;arn&gt;" (PAYMENT_LINE_MATCHED)
-MSG-NB-260: "Choose the CLPC billing batch the report answers" (PAYMENT_REPORT_BATCH_REQUIRED)
-MSG-NB-261: "Payment report &lt;report no&gt; is &lt;status&gt;" (PAYMENT_REPORT_CLOSED)
-MSG-NB-262: "The payment report has no rows" (PAYMENT_REPORT_EMPTY)
-MSG-NB-263: "The CLPC report needs a 'PN No.' or 'Loan Application No.' column" (PAYMENT_REPORT_LAYOUT)
-MSG-NB-264: "The payment report needs an 'ARN' or 'Reference' column" (PAYMENT_REPORT_LAYOUT)
-MSG-NB-265: "Row &lt;row no&gt;: '&lt;value&gt;' is not a date (yyyy-mm-dd)" (PAYMENT_REPORT_VALUE)
-MSG-NB-266: "Row &lt;row no&gt;: '&lt;value&gt;' is not an amount" (PAYMENT_REPORT_VALUE)</t>
+MSG-NB-259: "&lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
+MSG-NB-260: "Billing batch &lt;batch no&gt; is closed" (BILLING_BATCH_CLOSED)
+MSG-NB-261: "BillingBatch not found: &lt;batch id&gt;" (NOT_FOUND)
+MSG-NB-262: "Payment report line not found: &lt;line id&gt;" (NOT_FOUND)
+MSG-NB-263: "PaymentReport not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-264: "Row &lt;row no&gt; is already matched to &lt;arn&gt;" (PAYMENT_LINE_MATCHED)
+MSG-NB-265: "Choose the CLPC billing batch the report answers" (PAYMENT_REPORT_BATCH_REQUIRED)
+MSG-NB-266: "Payment report &lt;report no&gt; is &lt;status&gt;" (PAYMENT_REPORT_CLOSED)
+MSG-NB-267: "The payment report has no rows" (PAYMENT_REPORT_EMPTY)
+MSG-NB-268: "The CLPC report needs a 'PN No.' or 'Loan Application No.' column" (PAYMENT_REPORT_LAYOUT)
+MSG-NB-269: "The payment report needs an 'ARN' or 'Reference' column" (PAYMENT_REPORT_LAYOUT)
+MSG-NB-270: "Row &lt;row no&gt;: '&lt;value&gt;' is not a date (yyyy-mm-dd)" (PAYMENT_REPORT_VALUE)
+MSG-NB-271: "Row &lt;row no&gt;: '&lt;value&gt;' is not an amount" (PAYMENT_REPORT_VALUE)</t>
         </is>
       </c>
       <c r="M455" s="12" t="inlineStr">
@@ -52139,14 +52144,14 @@
       <c r="L456" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-269: "No account found for &lt;file name&gt;: choose the account (ARN)" (EPOLICY_ACCOUNT_NOT_FOUND)
-MSG-NB-270: "Account &lt;arn&gt; is &lt;status&gt;; an e-policy is received once placed" (EPOLICY_ACCOUNT_STATUS)
-MSG-NB-271: "Upload between 1 and 50 e-policies at a time" (EPOLICY_FILE_COUNT)
-MSG-NB-272: "The e-policy &lt;file name&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)
-MSG-NB-273: "This upload is &lt;status&gt;" (EPOLICY_UPLOAD_CLOSED)
-MSG-NB-274: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-275: "E-policy upload file not found: &lt;item id&gt;" (NOT_FOUND)
-MSG-NB-276: "Epolicy not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-274: "No account found for &lt;file name&gt;: choose the account (ARN)" (EPOLICY_ACCOUNT_NOT_FOUND)
+MSG-NB-275: "Account &lt;arn&gt; is &lt;&gt;; an e-policy is received once placed" (EPOLICY_ACCOUNT_STATUS)
+MSG-NB-276: "Upload between 1 and 50 e-policies at a time" (EPOLICY_FILE_COUNT)
+MSG-NB-277: "The e-policy &lt;file name&gt; is already &lt;&gt;" (EPOLICY_REVIEWED)
+MSG-NB-278: "This upload is &lt;status&gt;" (EPOLICY_UPLOAD_CLOSED)
+MSG-NB-279: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-280: "E-policy upload file not found: &lt;item id&gt;" (NOT_FOUND)
+MSG-NB-281: "Epolicy not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M456" s="12" t="inlineStr">
@@ -52222,12 +52227,12 @@
       <c r="L457" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-277: "Check before confirming &lt;list&gt;"
-MSG-NB-279: "Enter one policy number per policy year."
-MSG-NB-283: "Rejected by &lt;user&gt;: &lt;reject reason&gt;"
-MSG-NB-284: "The policy numbers must be different."
-MSG-NB-285: "Confirm the policy data of &lt;arn&gt; before sending the e-policy" (EPOLICY_NOT_CONFIRMED)
-MSG-NB-286: "The e-policy &lt;file name&gt; of &lt;arn&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)</t>
+MSG-NB-282: "Check before confirming &lt;list&gt;"
+MSG-NB-284: "Enter one policy number per policy year."
+MSG-NB-288: "Rejected by &lt;user&gt;: &lt;reject reason&gt;"
+MSG-NB-289: "The policy numbers must be different."
+MSG-NB-290: "Confirm the policy data of &lt;arn&gt; before sending the e-policy" (EPOLICY_NOT_CONFIRMED)
+MSG-NB-291: "The e-policy &lt;file name&gt; of &lt;arn&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)</t>
         </is>
       </c>
       <c r="M457" s="12" t="inlineStr">
@@ -52303,10 +52308,10 @@
       <c r="L458" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-289: "Account &lt;arn&gt; is &lt;status&gt;; it must be placed first" (IA_ACCOUNT_STATUS)
-MSG-NB-290: "Account &lt;arn&gt; has no mortgagee bank: no Insurance Advice" (IA_NOT_MORTGAGED)
-MSG-NB-291: "Select between 1 and 50 Insurance Advices" (IA_SELECTION)
-MSG-NB-292: "InsuranceAdvice not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-294: "Account &lt;arn&gt; is &lt;status&gt;; it must be placed first" (IA_ACCOUNT_STATUS)
+MSG-NB-295: "Account &lt;arn&gt; has no mortgagee bank: no Insurance Advice" (IA_NOT_MORTGAGED)
+MSG-NB-296: "Select between 1 and 50 Insurance Advices" (IA_SELECTION)
+MSG-NB-297: "InsuranceAdvice not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M458" s="12" t="inlineStr">
@@ -52382,8 +52387,8 @@
       <c r="L459" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-295: "Account &lt;arn&gt; has no contact e-mail: enter the recipient" (EPOLICY_NO_RECIPIENT)
-MSG-NB-296: "Select between 1 and 200 records" (ISSUANCE_SELECTION)</t>
+MSG-NB-300: "Account &lt;arn&gt; has no contact e-mail: enter the recipient" (EPOLICY_NO_RECIPIENT)
+MSG-NB-301: "Select between 1 and 200 records" (ISSUANCE_SELECTION)</t>
         </is>
       </c>
       <c r="M459" s="12" t="inlineStr">
@@ -52459,20 +52464,20 @@
       <c r="L460" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-299: "A negative endorsement reduces the sum insured (enter a minus)"
-MSG-NB-300: "A positive endorsement increases the sum insured"
-MSG-NB-301: "Choose the reason"
-MSG-NB-302: "Describe the cancellation"
-MSG-NB-303: "Describe the change"
-MSG-NB-304: "Enter a rate of zero or more, or leave it blank"
-MSG-NB-305: "Enter the cancellation date"
-MSG-NB-306: "Enter the change of the sum insured"
-MSG-NB-307: "Enter the effective date"
-MSG-NB-309: "No queued account to book" (BATCH_EMPTY)
-MSG-NB-310: "Select at least one account to book" (BATCH_EMPTY)
-MSG-NB-311: "The booking date &lt;booking date&gt; is in the future" (BOOKING_DATE_FUTURE)
-MSG-NB-312: "BookingQueue not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-313: "Account &lt;arn&gt; is no longer queued (&lt;status&gt;)" (QUEUE_ENTRY_CLOSED)</t>
+MSG-NB-304: "A negative endorsement reduces the sum insured (enter a minus)"
+MSG-NB-305: "A positive endorsement increases the sum insured"
+MSG-NB-306: "Choose the reason"
+MSG-NB-307: "Describe the cancellation"
+MSG-NB-308: "Describe the change"
+MSG-NB-309: "Enter a rate of zero or more, or leave it blank"
+MSG-NB-310: "Enter the cancellation date"
+MSG-NB-311: "Enter the change of the sum insured"
+MSG-NB-312: "Enter the effective date"
+MSG-NB-314: "No queued account to book" (BATCH_EMPTY)
+MSG-NB-315: "Select at least one account to book" (BATCH_EMPTY)
+MSG-NB-316: "The booking date &lt;booking date&gt; is in the future" (BOOKING_DATE_FUTURE)
+MSG-NB-317: "BookingQueue not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-318: "Account &lt;arn&gt; is no longer queued (&lt;status&gt;)" (QUEUE_ENTRY_CLOSED)</t>
         </is>
       </c>
       <c r="M460" s="12" t="inlineStr">
@@ -52548,24 +52553,24 @@
       <c r="L461" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-315: "Account &lt;arn&gt; has no insurer" (ACCOUNT_INSURER_MISSING)
-MSG-NB-316: "Account &lt;arn&gt; is &lt;status&gt;: only issued policies are booked" (ACCOUNT_NOT_BOOKABLE)
-MSG-NB-317: "Account &lt;arn&gt; has no period of cover" (ACCOUNT_PERIOD_MISSING)
-MSG-NB-318: "Billing number &lt;billing no&gt; of &lt;insurer code&gt; is already on invoice &lt;invoice no&gt;" (BILLING_NO_DUPLICATE)
-MSG-NB-319: "Enter the insurer billing number" (BILLING_NO_REQUIRED)
-MSG-NB-320: "The insurer billing number has at most 60 characters" (BILLING_NO_TOO_LONG)
-MSG-NB-321: "The company has no branch to book invoices" (BOOKING_BRANCH_MISSING)
-MSG-NB-322: "The booking date &lt;date&gt; is in the future" (BOOKING_DATE_FUTURE)
-MSG-NB-323: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (CLIENT_PARTY_MISSING)
-MSG-NB-324: "Enter the cost center of account &lt;arn&gt;" (COST_CENTER_REQUIRED)
-MSG-NB-325: "Account &lt;arn&gt; is already booked" (DUPLICATE_BOOKING)
-MSG-NB-326: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (INSURER_PARTY_MISSING)
-MSG-NB-327: "Each insurer appears once with a positive share" (INSURER_SHARES_INVALID)
-MSG-NB-328: "Insurer shares must add up to 100% and include the lead insurer &lt;insurer code&gt;" (INSURER_SHARES_INVALID)
-MSG-NB-329: "Invoice &lt;arn&gt;/&lt;transaction no&gt; is &lt;status&gt;" (INVOICE_ALREADY_BOOKED)
-MSG-NB-330: "No invoice" (INVOICE_NOT_FOUND)
-MSG-NB-331: "Policy year &lt;policy year&gt; of &lt;arn&gt; is not due for booking" (POLICY_YEAR_NOT_DUE)
-MSG-NB-332: "Account &lt;arn&gt; has no rated premium" (PREMIUM_NOT_RATED)</t>
+MSG-NB-320: "Account &lt;arn&gt; has no insurer" (ACCOUNT_INSURER_MISSING)
+MSG-NB-321: "Account &lt;arn&gt; is &lt;&gt;: only issued policies are booked" (ACCOUNT_NOT_BOOKABLE)
+MSG-NB-322: "Account &lt;arn&gt; has no period of cover" (ACCOUNT_PERIOD_MISSING)
+MSG-NB-323: "Billing number &lt;billing no&gt; of &lt;insurer code&gt; is already on invoice &lt;invoice no&gt;" (BILLING_NO_DUPLICATE)
+MSG-NB-324: "Enter the insurer billing number" (BILLING_NO_REQUIRED)
+MSG-NB-325: "The insurer billing number has at most 60 characters" (BILLING_NO_TOO_LONG)
+MSG-NB-326: "The company has no branch to book invoices" (BOOKING_BRANCH_MISSING)
+MSG-NB-327: "The booking date &lt;date&gt; is in the future" (BOOKING_DATE_FUTURE)
+MSG-NB-328: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (CLIENT_PARTY_MISSING)
+MSG-NB-329: "Enter the cost center of account &lt;arn&gt;" (COST_CENTER_REQUIRED)
+MSG-NB-330: "Account &lt;arn&gt; is already booked" (DUPLICATE_BOOKING)
+MSG-NB-331: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (INSURER_PARTY_MISSING)
+MSG-NB-332: "Each insurer appears once with a positive share" (INSURER_SHARES_INVALID)
+MSG-NB-333: "Insurer shares must add up to 100% and include the lead insurer &lt;insurer code&gt;" (INSURER_SHARES_INVALID)
+MSG-NB-334: "Invoice &lt;arn&gt;/&lt;transaction no&gt; is &lt;status&gt;" (INVOICE_ALREADY_BOOKED)
+MSG-NB-335: "No invoice" (INVOICE_NOT_FOUND)
+MSG-NB-336: "Policy year &lt;policy year&gt; of &lt;arn&gt; is not due for booking" (POLICY_YEAR_NOT_DUE)
+MSG-NB-337: "Account &lt;arn&gt; has no rated premium" (PREMIUM_NOT_RATED)</t>
         </is>
       </c>
       <c r="M461" s="12" t="inlineStr">
@@ -52641,15 +52646,15 @@
       <c r="L462" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-339: "Account &lt;arn&gt; is &lt;status&gt;: only booked accounts are endorsed" (ACCOUNT_NOT_BOOKED)
-MSG-NB-340: "A cancellation, and only a cancellation, has a kind" (CANCELLATION_KIND_REQUIRED)
-MSG-NB-341: "Enter the change of the sum insured or the premium" (ENDORSEMENT_CHANGE_REQUIRED)
-MSG-NB-342: "The effective date &lt;effective&gt; is not within a booked policy year of &lt;arn&gt;" (ENDORSEMENT_DATE_OUTSIDE_TERM)
-MSG-NB-343: "Enter the account, type, effective date and description" (ENDORSEMENT_INCOMPLETE)
-MSG-NB-344: "A negative endorsement or cancellation must return premium" (ENDORSEMENT_SIGN_MISMATCH)
-MSG-NB-345: "A positive endorsement must add premium" (ENDORSEMENT_SIGN_MISMATCH)
-MSG-NB-346: "The return premium exceeds the premium in force of policy year &lt;year&gt;" (RETURN_EXCEEDS_PREMIUM)
-MSG-NB-347: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
+MSG-NB-344: "Account &lt;arn&gt; is &lt;&gt;: only booked accounts are endorsed" (ACCOUNT_NOT_BOOKED)
+MSG-NB-345: "A cancellation, and only a cancellation, has a kind" (CANCELLATION_KIND_REQUIRED)
+MSG-NB-346: "Enter the change of the sum insured or the premium" (ENDORSEMENT_CHANGE_REQUIRED)
+MSG-NB-347: "The effective date &lt;effective&gt; is not within a booked policy year of &lt;arn&gt;" (ENDORSEMENT_DATE_OUTSIDE_TERM)
+MSG-NB-348: "Enter the account, type, effective date and description" (ENDORSEMENT_INCOMPLETE)
+MSG-NB-349: "A negative endorsement or cancellation must return premium" (ENDORSEMENT_SIGN_MISMATCH)
+MSG-NB-350: "A positive endorsement must add premium" (ENDORSEMENT_SIGN_MISMATCH)
+MSG-NB-351: "The return premium exceeds the premium in force of policy year &lt;year&gt;" (RETURN_EXCEEDS_PREMIUM)
+MSG-NB-352: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
         </is>
       </c>
       <c r="M462" s="12" t="inlineStr">
@@ -52725,14 +52730,14 @@
       <c r="L463" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-349: "E-mail: &lt;dispatch error&gt;"
-MSG-NB-351: "Service invoice &lt;si no&gt; has &lt;commission&gt; commission and &lt;vat&gt; VAT left to credit" (CREDIT_EXCEEDS_INVOICE)
-MSG-NB-352: "&lt;si no&gt; is itself a credit" (CREDIT_OF_CREDIT)
-MSG-NB-353: "Service invoice type not found: &lt;code&gt;" (NOT_FOUND)
-MSG-NB-354: "ServiceInvoice not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-355: "ServiceInvoice not found: &lt;si no&gt;" (NOT_FOUND)
-MSG-NB-356: "Service invoices of type &lt;type code&gt; are issued automatically with the early remittance incentive" (SERVICE_INVOICE_AUTOMATIC_ONLY)
-MSG-NB-357: "Service invoice type &lt;code&gt; is inactive" (SERVICE_INVOICE_TYPE_INACTIVE)</t>
+MSG-NB-354: "E-mail: &lt;dispatch error&gt;"
+MSG-NB-356: "Service invoice &lt;si no&gt; has &lt;commission&gt; commission and &lt;vat&gt; VAT left to credit" (CREDIT_EXCEEDS_INVOICE)
+MSG-NB-357: "&lt;si no&gt; is itself a credit" (CREDIT_OF_CREDIT)
+MSG-NB-358: "Service invoice type not found: &lt;code&gt;" (NOT_FOUND)
+MSG-NB-359: "ServiceInvoice not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-360: "ServiceInvoice not found: &lt;si no&gt;" (NOT_FOUND)
+MSG-NB-361: "Service invoices of type &lt;type code&gt; are issued automatically with the early remittance incentive" (SERVICE_INVOICE_AUTOMATIC_ONLY)
+MSG-NB-362: "Service invoice type &lt;code&gt; is inactive" (SERVICE_INVOICE_TYPE_INACTIVE)</t>
         </is>
       </c>
       <c r="M463" s="12" t="inlineStr">
@@ -52808,12 +52813,12 @@
       <c r="L464" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-360: "Service invoice type already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-361: "The period end must not be before the period start" (INCENTIVE_PERIOD_INVALID)
-MSG-NB-362: "Incentive rules are maintained in Product Maintenance &gt; Incentive Criteria" (INCENTIVE_RULES_FROZEN)
-MSG-NB-363: "AutoBookRule not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-364: "IncentiveRule not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-365: "ServiceInvoiceType not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-365: "Service invoice type already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-366: "The period end must not be before the period start" (INCENTIVE_PERIOD_INVALID)
+MSG-NB-367: "Incentive rules are maintained in Product Maintenance &gt; Incentive Criteria" (INCENTIVE_RULES_FROZEN)
+MSG-NB-368: "AutoBookRule not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-369: "IncentiveRule not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-370: "ServiceInvoiceType not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M464" s="12" t="inlineStr">
@@ -52889,31 +52894,31 @@
       <c r="L465" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-370: "Risk groups are numbers separated by ';'" (ACCEPTANCE_GROUP_INVALID)
-MSG-NB-371: "Account &lt;arn&gt; is &lt;status&gt;" (ACCOUNT_NOT_EDITABLE)
-MSG-NB-372: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
-MSG-NB-373: "Business Type must be NEW_BUSINESS or RENEWAL" (BULK_BUSINESS_TYPE_INVALID)
-MSG-NB-374: "Enter an individual's name as 'Last, First'" (BULK_CLIENT_NAME_FORMAT)
-MSG-NB-375: "Give the Client Code or the Client Name" (BULK_CLIENT_REQUIRED)
-MSG-NB-376: "This file was already uploaded as &lt;job no&gt; (&lt;file name&gt;)" (BULK_DUPLICATE_FILE)
-MSG-NB-377: "The file has no data rows" (BULK_FILE_EMPTY)
-MSG-NB-378: "The file has no header row" (BULK_FILE_EMPTY)
-MSG-NB-379: "The file has &lt;size&gt; rows; the maximum is &lt;max&gt;" (BULK_FILE_TOO_LARGE)
-MSG-NB-380: "Upload an Excel (.xlsx), OpenDocument (.ods), CSV (.csv) or text (.txt) file" (BULK_FILE_TYPE)
-MSG-NB-381: "The file cannot be read: &lt;message&gt;" (BULK_FILE_UNREADABLE)
-MSG-NB-382: "The file is not an OpenDocument spreadsheet" (BULK_FILE_UNREADABLE)
-MSG-NB-383: "Upload &lt;job no&gt; is already &lt;status&gt;" (BULK_JOB_CLOSED)
-MSG-NB-384: "Upload &lt;job no&gt; has not been committed yet" (BULK_JOB_NOT_COMPLETED)
-MSG-NB-385: "You are not allowed to use '&lt;title&gt;'" (BULK_NOT_PERMITTED)
-MSG-NB-386: "Choose the product of the upload" (BULK_PRODUCT_REQUIRED)
-MSG-NB-387: "The file does not follow the current template; missing column(s): &lt;missing&gt;" (BULK_TEMPLATE_MISMATCH)
-MSG-NB-388: "The fixed-width layout of this upload type has no fields" (BULK_TEXT_LAYOUT)
-MSG-NB-389: "The text file has no tab, pipe, semicolon or comma separated header line" (BULK_TEXT_LAYOUT)
-MSG-NB-390: "Action must be TAG or CANCEL" (FFY_ACTION_INVALID)
-MSG-NB-391: "No live account insures vehicle &lt;identifier&gt;" (FFY_VEHICLE_NOT_UNIQUE)
-MSG-NB-392: "Several accounts insure vehicle &lt;identifier&gt;: &lt;details&gt;" (FFY_VEHICLE_NOT_UNIQUE)
-MSG-NB-393: "Bulk upload type not found: &lt;code&gt;" (NOT_FOUND)
-MSG-NB-394: "BulkJob not found: &lt;job id&gt;" (NOT_FOUND)</t>
+MSG-NB-375: "Risk groups are numbers separated by ';'" (ACCEPTANCE_GROUP_INVALID)
+MSG-NB-376: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
+MSG-NB-377: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
+MSG-NB-378: "Business Type must be NEW_BUSINESS or RENEWAL" (BULK_BUSINESS_TYPE_INVALID)
+MSG-NB-379: "Enter an individual's name as 'Last, First'" (BULK_CLIENT_NAME_FORMAT)
+MSG-NB-380: "Give the Client Code or the Client Name" (BULK_CLIENT_REQUIRED)
+MSG-NB-381: "This file was already uploaded as &lt;job no&gt; (&lt;file name&gt;)" (BULK_DUPLICATE_FILE)
+MSG-NB-382: "The file has no data rows" (BULK_FILE_EMPTY)
+MSG-NB-383: "The file has no header row" (BULK_FILE_EMPTY)
+MSG-NB-384: "The file has &lt;size&gt; rows; the maximum is &lt;max&gt;" (BULK_FILE_TOO_LARGE)
+MSG-NB-385: "Upload an Excel (.xlsx), OpenDocument (.ods), CSV (.csv) or text (.txt) file" (BULK_FILE_TYPE)
+MSG-NB-386: "The file cannot be read: &lt;message&gt;" (BULK_FILE_UNREADABLE)
+MSG-NB-387: "The file is not an OpenDocument spreadsheet" (BULK_FILE_UNREADABLE)
+MSG-NB-388: "Upload &lt;job no&gt; is already &lt;status&gt;" (BULK_JOB_CLOSED)
+MSG-NB-389: "Upload &lt;job no&gt; has not been committed yet" (BULK_JOB_NOT_COMPLETED)
+MSG-NB-390: "You are not allowed to use '&lt;title&gt;'" (BULK_NOT_PERMITTED)
+MSG-NB-391: "Choose the product of the upload" (BULK_PRODUCT_REQUIRED)
+MSG-NB-392: "The file does not follow the current template; missing column(s): &lt;missing&gt;" (BULK_TEMPLATE_MISMATCH)
+MSG-NB-393: "The fixed-width layout of this upload type has no fields" (BULK_TEXT_LAYOUT)
+MSG-NB-394: "The text file has no tab, pipe, semicolon or comma separated header line" (BULK_TEXT_LAYOUT)
+MSG-NB-395: "Action must be TAG or CANCEL" (FFY_ACTION_INVALID)
+MSG-NB-396: "No live account insures vehicle &lt;identifier&gt;" (FFY_VEHICLE_NOT_UNIQUE)
+MSG-NB-397: "Several accounts insure vehicle &lt;identifier&gt;: &lt;details&gt;" (FFY_VEHICLE_NOT_UNIQUE)
+MSG-NB-398: "Bulk upload type not found: &lt;code&gt;" (NOT_FOUND)
+MSG-NB-399: "BulkJob not found: &lt;job id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M465" s="12" t="inlineStr">
@@ -52977,18 +52982,18 @@
       <c r="L466" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-396: "The file content does not match its .&lt;type&gt; type" (ATTACHMENT_CONTENT_MISMATCH)
-MSG-NB-397: "The file is empty" (ATTACHMENT_EMPTY)
-MSG-NB-398: "The file was rejected by the malware scan: &lt;detail&gt;" (ATTACHMENT_INFECTED)
-MSG-NB-399: "Stored file failed its checksum verification" (ATTACHMENT_INTEGRITY_FAILURE)
-MSG-NB-400: "The file exceeds the maximum size of &lt;to megabytes&gt; MB" (ATTACHMENT_TOO_LARGE)
-MSG-NB-401: "Only these file types are allowed: &lt;allowed extensions&gt;" (ATTACHMENT_TYPE_NOT_ALLOWED)
-MSG-NB-402: "Select between 1 and 50 documents" (DOCUMENT_FILE_COUNT)
-MSG-NB-403: "Upload between 1 and 50 files at a time" (DOCUMENT_FILE_COUNT)
-MSG-NB-404: "A reference is needed to nominate the file names" (DOCUMENT_REFERENCE_REQUIRED)
-MSG-NB-405: "Invalid entity type or id" (INVALID_ATTACHMENT_TARGET)
-MSG-NB-406: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-407: "Attachment content not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-401: "The file content does not match its .&lt;type&gt; type" (ATTACHMENT_CONTENT_MISMATCH)
+MSG-NB-402: "The file is empty" (ATTACHMENT_EMPTY)
+MSG-NB-403: "The file was rejected by the malware scan: &lt;detail&gt;" (ATTACHMENT_INFECTED)
+MSG-NB-404: "Stored file failed its checksum verification" (ATTACHMENT_INTEGRITY_FAILURE)
+MSG-NB-405: "The file exceeds the maximum size of &lt;to megabytes&gt; MB" (ATTACHMENT_TOO_LARGE)
+MSG-NB-406: "Only these file types are allowed: &lt;allowed extensions&gt;" (ATTACHMENT_TYPE_NOT_ALLOWED)
+MSG-NB-407: "Select between 1 and 50 documents" (DOCUMENT_FILE_COUNT)
+MSG-NB-408: "Upload between 1 and 50 files at a time" (DOCUMENT_FILE_COUNT)
+MSG-NB-409: "A reference is needed to nominate the file names" (DOCUMENT_REFERENCE_REQUIRED)
+MSG-NB-410: "Invalid entity type or id" (INVALID_ATTACHMENT_TARGET)
+MSG-NB-411: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-412: "Attachment content not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M466" s="12" t="inlineStr">
@@ -53052,16 +53057,16 @@
       <c r="L467" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-409: "&lt;entity type&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-410: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
-MSG-NB-411: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)
-MSG-NB-412: "Workflow not found: &lt;workflow code&gt;" (NOT_FOUND)
-MSG-NB-413: "Workflow stage not found: &lt;stage code&gt;" (NOT_FOUND)
-MSG-NB-414: "'&lt;label&gt;' must be done from the record screen" (WORKFLOW_ACTION_NOT_GENERIC)
-MSG-NB-415: "You are not allowed to '&lt;label&gt;'" (WORKFLOW_ACTION_NOT_PERMITTED)
-MSG-NB-416: "Select a reason for '&lt;label&gt;'" (WORKFLOW_REASON_REQUIRED)
-MSG-NB-417: "'&lt;action&gt;' is not allowed while &lt;reference&gt; is in stage &lt;name&gt;" (WORKFLOW_TRANSITION_NOT_ALLOWED)
-MSG-NB-418: "The item is closed" (WORK_CASE_CLOSED)</t>
+MSG-NB-414: "&lt;entity type&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-415: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
+MSG-NB-416: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)
+MSG-NB-417: "Workflow not found: &lt;workflow code&gt;" (NOT_FOUND)
+MSG-NB-418: "Workflow stage not found: &lt;stage code&gt;" (NOT_FOUND)
+MSG-NB-419: "'&lt;label&gt;' must be done from the record screen" (WORKFLOW_ACTION_NOT_GENERIC)
+MSG-NB-420: "You are not allowed to '&lt;label&gt;'" (WORKFLOW_ACTION_NOT_PERMITTED)
+MSG-NB-421: "Select a reason for '&lt;label&gt;'" (WORKFLOW_REASON_REQUIRED)
+MSG-NB-422: "'&lt;action&gt;' is not allowed while &lt;reference&gt; is in stage &lt;name&gt;" (WORKFLOW_TRANSITION_NOT_ALLOWED)
+MSG-NB-423: "The item is closed" (WORK_CASE_CLOSED)</t>
         </is>
       </c>
       <c r="M467" s="12" t="inlineStr">
@@ -53137,10 +53142,10 @@
       <c r="L468" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-421: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)
-MSG-NB-422: "&lt;assignee&gt; does not work this queue" (WORK_ASSIGNEE_NOT_ELIGIBLE)
-MSG-NB-423: "The item is closed" (WORK_CASE_CLOSED)
-MSG-NB-424: "This item is not in your queue" (WORK_CLAIM_NOT_ALLOWED)</t>
+MSG-NB-426: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)
+MSG-NB-427: "&lt;assignee&gt; does not work this queue" (WORK_ASSIGNEE_NOT_ELIGIBLE)
+MSG-NB-428: "The item is closed" (WORK_CASE_CLOSED)
+MSG-NB-429: "This item is not in your queue" (WORK_CLAIM_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M468" s="12" t="inlineStr">
@@ -53216,14 +53221,14 @@
       <c r="L469" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-427: "&lt;file name&gt; cannot be password protected. Send it as PDF, Excel or Word" (DOCUMENT_NOT_PROTECTABLE)
-MSG-NB-428: "Could not protect &lt;file name&gt;: &lt;message&gt;" (DOCUMENT_PROTECTION_FAILED)
-MSG-NB-429: "Invalid e-mail address: &lt;a&gt;" (EMAIL_ADDRESS_INVALID)
-MSG-NB-430: "Enter the &lt;field&gt;" (EMAIL_CONTENT_REQUIRED)
-MSG-NB-431: "Enter at least one recipient" (EMAIL_RECIPIENT_REQUIRED)
-MSG-NB-432: "Too many recipients" (EMAIL_TOO_MANY_RECIPIENTS)
-MSG-NB-433: "Only a failed message can be resent" (MESSAGE_NOT_FAILED)
-MSG-NB-434: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-432: "&lt;file name&gt; cannot be password protected. Send it as PDF, Excel or Word" (DOCUMENT_NOT_PROTECTABLE)
+MSG-NB-433: "Could not protect &lt;file name&gt;: &lt;message&gt;" (DOCUMENT_PROTECTION_FAILED)
+MSG-NB-434: "Invalid e-mail address: &lt;a&gt;" (EMAIL_ADDRESS_INVALID)
+MSG-NB-435: "Enter the &lt;field&gt;" (EMAIL_CONTENT_REQUIRED)
+MSG-NB-436: "Enter at least one recipient" (EMAIL_RECIPIENT_REQUIRED)
+MSG-NB-437: "Too many recipients" (EMAIL_TOO_MANY_RECIPIENTS)
+MSG-NB-438: "Only a failed message can be resent" (MESSAGE_NOT_FAILED)
+MSG-NB-439: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M469" s="12" t="inlineStr">
@@ -53299,12 +53304,12 @@
       <c r="L470" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-435: "&lt;type code&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-436: "The effective-to date is before the effective-from date" (LOV_EFFECTIVITY_INVALID)
-MSG-NB-437: "The list &lt;type code&gt; is maintained by the system" (LOV_NOT_MAINTAINABLE)
-MSG-NB-438: "'&lt;code&gt;' is not a valid value of &lt;type code&gt; on &lt;date&gt;" (LOV_VALUE_INVALID)
-MSG-NB-439: "LovType not found: &lt;type code&gt;" (NOT_FOUND)
-MSG-NB-440: "LovValue not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-440: "&lt;type code&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-441: "The effective-to date is before the effective-from date" (LOV_EFFECTIVITY_INVALID)
+MSG-NB-442: "The list &lt;type code&gt; is maintained by the system" (LOV_NOT_MAINTAINABLE)
+MSG-NB-443: "'&lt;code&gt;' is not a valid value of &lt;type code&gt; on &lt;date&gt;" (LOV_VALUE_INVALID)
+MSG-NB-444: "LovType not found: &lt;type code&gt;" (NOT_FOUND)
+MSG-NB-445: "LovValue not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M470" s="12" t="inlineStr">
@@ -53380,13 +53385,13 @@
       <c r="L471" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-441: "Enter a whole number of bookings (0 or more)"
-MSG-NB-442: "Enter an amount of 0 or more"
-MSG-NB-443: "Enter the period"
-MSG-NB-444: "Enter the unit code or the officer username"
-MSG-NB-447: "The period end must not be before the start"
-MSG-NB-448: "Targets cannot be negative" (TARGET_NEGATIVE)
-MSG-NB-449: "The period end must not be before the period start" (TARGET_PERIOD_INVALID)</t>
+MSG-NB-446: "Enter a whole number of bookings (0 or more)"
+MSG-NB-447: "Enter an amount of 0 or more"
+MSG-NB-448: "Enter the period"
+MSG-NB-449: "Enter the unit code or the officer username"
+MSG-NB-452: "The period end must not be before the start"
+MSG-NB-453: "Targets cannot be negative" (TARGET_NEGATIVE)
+MSG-NB-454: "The period end must not be before the period start" (TARGET_PERIOD_INVALID)</t>
         </is>
       </c>
       <c r="M471" s="12" t="inlineStr">
@@ -53462,9 +53467,9 @@
       <c r="L472" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-450: "ReportVariant not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-451: "Report &lt;report code&gt; is not available to you" (REPORT_NOT_AVAILABLE)
-MSG-NB-452: "Only the user who saved a report variant may delete it" (VARIANT_NOT_OWNER)</t>
+MSG-NB-455: "ReportVariant not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-456: "Report &lt;report code&gt; is not available to you" (REPORT_NOT_AVAILABLE)
+MSG-NB-457: "Only the user who saved a report variant may delete it" (VARIANT_NOT_OWNER)</t>
         </is>
       </c>
       <c r="M472" s="12" t="inlineStr">
@@ -53540,13 +53545,13 @@
       <c r="L473" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-457: "This document cannot be produced in Word" (DOCUMENT_WORD_UNAVAILABLE)
-MSG-NB-458: "Document template not found: &lt;code&gt;" (NOT_FOUND)
-MSG-NB-459: "Document template not found: &lt;version no&gt;" (NOT_FOUND)
-MSG-NB-460: "Word copy of document not found: &lt;D&gt;" (NOT_FOUND)
-MSG-NB-461: "Enter the template text" (TEMPLATE_BODY_REQUIRED)
-MSG-NB-462: "The Word file needs the title in its first paragraph and the text below it" (TEMPLATE_WORD_INVALID)
-MSG-NB-463: "The file is not a Word (.docx) document" (TEMPLATE_WORD_INVALID)</t>
+MSG-NB-462: "This document cannot be produced in Word" (DOCUMENT_WORD_UNAVAILABLE)
+MSG-NB-463: "Document template not found: &lt;code&gt;" (NOT_FOUND)
+MSG-NB-464: "Document template not found: &lt;version no&gt;" (NOT_FOUND)
+MSG-NB-465: "Word copy of document not found: &lt;D&gt;" (NOT_FOUND)
+MSG-NB-466: "Enter the template text" (TEMPLATE_BODY_REQUIRED)
+MSG-NB-467: "The Word file needs the title in its first paragraph and the text below it" (TEMPLATE_WORD_INVALID)
+MSG-NB-468: "The file is not a Word (.docx) document" (TEMPLATE_WORD_INVALID)</t>
         </is>
       </c>
       <c r="M473" s="12" t="inlineStr">
@@ -53610,15 +53615,15 @@
       <c r="L474" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-466: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-NB-467: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-NB-468: "An unexpected error occurred. Quote reference &lt;reference&gt; to support." (INTERNAL_ERROR)
-MSG-NB-469: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-NB-470: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
-MSG-NB-471: "The request body is not valid JSON or has fields of the wrong type" (MALFORMED_REQUEST)
-MSG-NB-472: "No such endpoint: &lt;resource path&gt;" (NOT_FOUND)
-MSG-NB-473: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
-MSG-NB-474: "Invalid request" (VALIDATION_FAILED)</t>
+MSG-NB-471: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-NB-472: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-NB-473: "An unexpected error occurred. Quote reference &lt;reference&gt; to support." (INTERNAL_ERROR)
+MSG-NB-474: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-NB-475: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-NB-476: "The request body is not valid JSON or has fields of the wrong type" (MALFORMED_REQUEST)
+MSG-NB-477: "No such endpoint: &lt;resource path&gt;" (NOT_FOUND)
+MSG-NB-478: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
+MSG-NB-479: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
       </c>
       <c r="M474" s="12" t="inlineStr">
@@ -53694,8 +53699,8 @@
       <c r="L475" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-479: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
-MSG-NB-480: "&lt;Column&gt; is mandatory"</t>
+MSG-NB-484: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
+MSG-NB-485: "&lt;Column&gt; is mandatory"</t>
         </is>
       </c>
       <c r="M475" s="12" t="inlineStr">
@@ -53771,7 +53776,7 @@
       <c r="L476" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-481: "&lt;quotation no&gt; is &lt;status&gt;, not sent to the client"</t>
+MSG-NB-486: "&lt;quotation no&gt; is &lt;&gt;, not sent to the client"</t>
         </is>
       </c>
       <c r="M476" s="12" t="inlineStr">
@@ -53847,8 +53852,8 @@
       <c r="L477" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-482: "Account &lt;arn&gt; belongs to another company"
-MSG-NB-485: "The booking date &lt;date&gt; is in the future"</t>
+MSG-NB-487: "Account &lt;arn&gt; belongs to another company"
+MSG-NB-490: "The booking date &lt;date&gt; is in the future"</t>
         </is>
       </c>
       <c r="M477" s="12" t="inlineStr">
@@ -53924,9 +53929,9 @@
       <c r="L478" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-483: "Client Type must be INDIVIDUAL or CORPORATE"
-MSG-NB-484: "Client code &lt;code&gt; does not exist"
-MSG-NB-486: "The row matches several clients: &lt;details&gt;"</t>
+MSG-NB-488: "Client Type must be INDIVIDUAL or CORPORATE"
+MSG-NB-489: "Client code &lt;code&gt; does not exist"
+MSG-NB-491: "The row matches several clients: &lt;details&gt;"</t>
         </is>
       </c>
       <c r="M478" s="12" t="inlineStr">
@@ -53990,18 +53995,18 @@
       <c r="L479" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-487: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
-MSG-NB-488: "Account not found: &lt;arn&gt;" (NOT_FOUND)
-MSG-NB-489: "Account not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-490: "Batch run not found: &lt;run no&gt;" (NOT_FOUND)
-MSG-NB-491: "Booked invoice not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-492: "Booked invoice not found: &lt;invoice no&gt;" (NOT_FOUND)
-MSG-NB-493: "Notification not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-494: "ProposalRequest not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-495: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-496: "Quotation not found: &lt;key&gt;" (NOT_FOUND)
-MSG-NB-497: "Quotation version not found: &lt;version no&gt;" (NOT_FOUND)
-MSG-NB-498: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)</t>
+MSG-NB-492: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
+MSG-NB-493: "Account not found: &lt;arn&gt;" (NOT_FOUND)
+MSG-NB-494: "Account not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-495: "Batch run not found: &lt;run no&gt;" (NOT_FOUND)
+MSG-NB-496: "Booked invoice not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-497: "Booked invoice not found: &lt;invoice no&gt;" (NOT_FOUND)
+MSG-NB-498: "Notification not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-499: "ProposalRequest not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-500: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-501: "Quotation not found: &lt;key&gt;" (NOT_FOUND)
+MSG-NB-502: "Quotation version not found: &lt;version no&gt;" (NOT_FOUND)
+MSG-NB-503: "WorkCase not found: &lt;case id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M479" s="12" t="inlineStr">

</xml_diff>

<commit_message>
BRD-01: a locked account is refused with the sign-in message of a wrong password; FRS, sign-off workbook and test plan rebuilt
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-01_New_Business/04_BIBS_TestPlan_BRD-01_New_Business_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-01_New_Business/04_BIBS_TestPlan_BRD-01_New_Business_v2.0.xlsx
@@ -42603,8 +42603,8 @@
       </c>
       <c r="L366" s="12" t="inlineStr">
         <is>
-          <t>The account locks at the third failure and the correct password is refused.
-Message "Account is locked. Contact your administrator." (AUTHENTICATION_FAILED).</t>
+          <t>The account locks at the third failure and the correct password is refused with the same message as a wrong password.
+Message "Invalid user name or password" (AUTHENTICATION_FAILED).</t>
         </is>
       </c>
       <c r="M366" s="12" t="inlineStr">
@@ -49099,22 +49099,22 @@
       <c r="L449" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-174: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
-MSG-NB-175: "Account &lt;arn&gt; is not a renewal account" (ACCOUNT_NOT_RENEWAL)
-MSG-NB-176: "Account &lt;arn&gt; is &lt;&gt;, not &lt;status&gt;" (ACCOUNT_STATUS_INVALID)
-MSG-NB-177: "Account &lt;arn&gt; is &lt;status&gt;, not DRAFT" (ACCOUNT_STATUS_INVALID)
-MSG-NB-178: "The ARN must read ARN-yyyy-nnnnnn (or ARN-yyyy-nnnnnn-nn)" (ARN_INVALID)
-MSG-NB-179: "An account already has ARN &lt;given&gt;" (ARN_IN_USE)
-MSG-NB-180: "The insurer of account &lt;arn&gt; cannot be changed when it is &lt;&gt;" (INSURER_CHANGE_NOT_ALLOWED)
-MSG-NB-181: "Select the new insurer" (INSURER_REQUIRED)
-MSG-NB-182: "Select an insurer other than the current one" (INSURER_UNCHANGED)
-MSG-NB-183: "Account not found: &lt;arn&gt;" (NOT_FOUND)
-MSG-NB-184: "Account not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-185: "Account &lt;arn&gt; is set up with insurer &lt;insurer code&gt;" (PLACEMENT_INSURER_MISMATCH)
-MSG-NB-186: "Attach the issued policy (policy copy or e-policy) before direct booking" (POLICY_DOCUMENT_REQUIRED)
-MSG-NB-187: "Account &lt;arn&gt; needs &lt;term years&gt; policy number(s), one per year" (POLICY_NUMBERS_MISMATCH)
-MSG-NB-188: "TSU clearance is given before the account is validated" (TSU_CLEARANCE_CLOSED)
-MSG-NB-189: "TSU must clear the account first: &lt;reason&gt;" (TSU_CLEARANCE_REQUIRED)</t>
+MSG-NB-173: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
+MSG-NB-174: "Account &lt;arn&gt; is not a renewal account" (ACCOUNT_NOT_RENEWAL)
+MSG-NB-175: "Account &lt;arn&gt; is &lt;&gt;, not &lt;status&gt;" (ACCOUNT_STATUS_INVALID)
+MSG-NB-176: "Account &lt;arn&gt; is &lt;status&gt;, not DRAFT" (ACCOUNT_STATUS_INVALID)
+MSG-NB-177: "The ARN must read ARN-yyyy-nnnnnn (or ARN-yyyy-nnnnnn-nn)" (ARN_INVALID)
+MSG-NB-178: "An account already has ARN &lt;given&gt;" (ARN_IN_USE)
+MSG-NB-179: "The insurer of account &lt;arn&gt; cannot be changed when it is &lt;&gt;" (INSURER_CHANGE_NOT_ALLOWED)
+MSG-NB-180: "Select the new insurer" (INSURER_REQUIRED)
+MSG-NB-181: "Select an insurer other than the current one" (INSURER_UNCHANGED)
+MSG-NB-182: "Account not found: &lt;arn&gt;" (NOT_FOUND)
+MSG-NB-183: "Account not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-184: "Account &lt;arn&gt; is set up with insurer &lt;insurer code&gt;" (PLACEMENT_INSURER_MISMATCH)
+MSG-NB-185: "Attach the issued policy (policy copy or e-policy) before direct booking" (POLICY_DOCUMENT_REQUIRED)
+MSG-NB-186: "Account &lt;arn&gt; needs &lt;term years&gt; policy number(s), one per year" (POLICY_NUMBERS_MISMATCH)
+MSG-NB-187: "TSU clearance is given before the account is validated" (TSU_CLEARANCE_CLOSED)
+MSG-NB-188: "TSU must clear the account first: &lt;reason&gt;" (TSU_CLEARANCE_REQUIRED)</t>
         </is>
       </c>
       <c r="M449" s="12" t="inlineStr">
@@ -49189,25 +49189,25 @@
       <c r="L450" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-191: "Choose the client and product to save the draft."
-MSG-NB-192: "The draft is not saved yet: click Save Draft to check it before submission."
-MSG-NB-193: "The draft was not saved: correct what the message above describes, then save the draft again."
-MSG-NB-194: "The draft was not saved: its risks are already on the account shown above. Change the risk items, or open the existing account instead."
-MSG-NB-195: "Select the client" (ACCOUNT_CLIENT_REQUIRED)
-MSG-NB-196: "Complete the mandatory fields of &lt;product code&gt;: &lt;check&gt;" (ACCOUNT_INCOMPLETE)
-MSG-NB-197: "The period end must be after the period start" (ACCOUNT_PERIOD_INVALID)
-MSG-NB-198: "Select the product" (ACCOUNT_PRODUCT_REQUIRED)
-MSG-NB-199: "Only a renewal account names the policy it renews (&lt;renewal of ref&gt;)" (ACCOUNT_RENEWAL_OF_NOT_RENEWAL)
-MSG-NB-200: "A multi-year account needs a term of at least 2 years" (ACCOUNT_TERM_INVALID)
-MSG-NB-201: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
-MSG-NB-202: "Duplicate of existing account &lt;arns&gt;: &lt;details&gt;" (DUPLICATE_ACCOUNT)
-MSG-NB-203: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
-MSG-NB-204: "Upload the mandatory documents: &lt;check&gt;" (MISSING_DOCUMENTS)
-MSG-NB-205: "Product &lt;code&gt; carries no mortgagee" (MORTGAGE_NOT_APPLICABLE)
-MSG-NB-206: "Product &lt;code&gt; allows a term of up to &lt;max term years&gt; year(s)" (MULTI_YEAR_NOT_ALLOWED)
-MSG-NB-207: "Compute the premium (sum insured and rate of every item) first" (PREMIUM_NOT_RATED)
-MSG-NB-208: "Account &lt;arn&gt; is priced on version &lt;priced&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: update the account to re-price it or request a rate exception" (RATE_SCHEME_NOT_CURRENT)
-MSG-NB-209: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-190: "Choose the client and product to save the draft."
+MSG-NB-191: "The draft is not saved yet: click Save Draft to check it before submission."
+MSG-NB-192: "The draft was not saved: correct what the message above describes, then save the draft again."
+MSG-NB-193: "The draft was not saved: its risks are already on the account shown above. Change the risk items, or open the existing account instead."
+MSG-NB-194: "Select the client" (ACCOUNT_CLIENT_REQUIRED)
+MSG-NB-195: "Complete the mandatory fields of &lt;product code&gt;: &lt;check&gt;" (ACCOUNT_INCOMPLETE)
+MSG-NB-196: "The period end must be after the period start" (ACCOUNT_PERIOD_INVALID)
+MSG-NB-197: "Select the product" (ACCOUNT_PRODUCT_REQUIRED)
+MSG-NB-198: "Only a renewal account names the policy it renews (&lt;renewal of ref&gt;)" (ACCOUNT_RENEWAL_OF_NOT_RENEWAL)
+MSG-NB-199: "A multi-year account needs a term of at least 2 years" (ACCOUNT_TERM_INVALID)
+MSG-NB-200: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
+MSG-NB-201: "Duplicate of existing account &lt;arns&gt;: &lt;details&gt;" (DUPLICATE_ACCOUNT)
+MSG-NB-202: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
+MSG-NB-203: "Upload the mandatory documents: &lt;check&gt;" (MISSING_DOCUMENTS)
+MSG-NB-204: "Product &lt;code&gt; carries no mortgagee" (MORTGAGE_NOT_APPLICABLE)
+MSG-NB-205: "Product &lt;code&gt; allows a term of up to &lt;max term years&gt; year(s)" (MULTI_YEAR_NOT_ALLOWED)
+MSG-NB-206: "Compute the premium (sum insured and rate of every item) first" (PREMIUM_NOT_RATED)
+MSG-NB-207: "Account &lt;arn&gt; is priced on version &lt;priced&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: update the account to re-price it or request a rate exception" (RATE_SCHEME_NOT_CURRENT)
+MSG-NB-208: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M450" s="12" t="inlineStr">
@@ -49282,9 +49282,9 @@
       <c r="L451" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-214: "Account &lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
-MSG-NB-215: "Account &lt;arn&gt; is not paid directly to the insurer" (GATE_NOT_DIRECT_PAYMENT)
-MSG-NB-216: "Account &lt;arn&gt; must be paid: match its payment from a payment report" (GATE_REQUIRES_PAYMENT)</t>
+MSG-NB-213: "Account &lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
+MSG-NB-214: "Account &lt;arn&gt; is not paid directly to the insurer" (GATE_NOT_DIRECT_PAYMENT)
+MSG-NB-215: "Account &lt;arn&gt; must be paid: match its payment from a payment report" (GATE_REQUIRES_PAYMENT)</t>
         </is>
       </c>
       <c r="M451" s="12" t="inlineStr">
@@ -49359,17 +49359,17 @@
       <c r="L452" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-219: "Record Hold Cover Confirmation"
-MSG-NB-220: "Record Hold Cover Decline"
-MSG-NB-221: "The hold cover of &lt;arn&gt; is &lt;status&gt;" (HOLD_COVER_CLOSED)
-MSG-NB-222: "The hold cover cannot expire before it starts (&lt;start date&gt;)" (HOLD_COVER_DATES)
-MSG-NB-223: "Account &lt;arn&gt; has no open hold cover" (HOLD_COVER_NONE)
-MSG-NB-224: "Account &lt;arn&gt; has no open hold cover request" (HOLD_COVER_NONE)
-MSG-NB-225: "A hold cover is requested while the account is being placed, not &lt;&gt;" (HOLD_COVER_NOT_ALLOWED)
-MSG-NB-226: "Account &lt;arn&gt; already has a hold cover requested or confirmed" (HOLD_COVER_OPEN)
-MSG-NB-227: "Enter the insurer's reference" (HOLD_COVER_REFERENCE)
-MSG-NB-228: "Choose the insurer on the account first" (INSURER_NOT_SET)
-MSG-NB-229: "Select the reason" (REASSIGN_REASON_REQUIRED)</t>
+MSG-NB-218: "Record Hold Cover Confirmation"
+MSG-NB-219: "Record Hold Cover Decline"
+MSG-NB-220: "The hold cover of &lt;arn&gt; is &lt;status&gt;" (HOLD_COVER_CLOSED)
+MSG-NB-221: "The hold cover cannot expire before it starts (&lt;start date&gt;)" (HOLD_COVER_DATES)
+MSG-NB-222: "Account &lt;arn&gt; has no open hold cover" (HOLD_COVER_NONE)
+MSG-NB-223: "Account &lt;arn&gt; has no open hold cover request" (HOLD_COVER_NONE)
+MSG-NB-224: "A hold cover is requested while the account is being placed, not &lt;&gt;" (HOLD_COVER_NOT_ALLOWED)
+MSG-NB-225: "Account &lt;arn&gt; already has a hold cover requested or confirmed" (HOLD_COVER_OPEN)
+MSG-NB-226: "Enter the insurer's reference" (HOLD_COVER_REFERENCE)
+MSG-NB-227: "Choose the insurer on the account first" (INSURER_NOT_SET)
+MSG-NB-228: "Select the reason" (REASSIGN_REASON_REQUIRED)</t>
         </is>
       </c>
       <c r="M452" s="12" t="inlineStr">
@@ -49444,20 +49444,20 @@
       <c r="L453" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-238: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
-MSG-NB-239: "Missing documents: &lt;missing&gt;" (DOCUMENTS_MISSING)
-MSG-NB-240: "Choose the insurer and branch on the account before placement" (INSURER_NOT_SET)
-MSG-NB-241: "Placement slip file not found: &lt;format&gt;" (NOT_FOUND)
-MSG-NB-242: "Placement slip not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-243: "The account is &lt;&gt;; a slip needs Ready for placement" (NOT_READY_FOR_PLACEMENT)
-MSG-NB-244: "The payment or client confirmation is not recorded" (PAYMENT_NOT_CONFIRMED)
-MSG-NB-245: "&lt;name&gt; is set up for &lt;placement channel&gt; placements; only e-mail is available: set the insurer to e-mail placement" (PLACEMENT_CHANNEL_PARKED)
-MSG-NB-246: "Select at least one account" (PLACEMENT_NO_ACCOUNTS)
-MSG-NB-247: "Select the accounts to place" (SLIP_NO_ACCOUNTS)
-MSG-NB-248: "Placement prerequisites not met - &lt;problems&gt;" (SLIP_PREREQUISITES_UNMET)
-MSG-NB-249: "Slip &lt;display no&gt; was already replaced" (SLIP_SUPERSEDED)
-MSG-NB-250: "Slip &lt;slip no&gt; v&lt;version no&gt; was replaced by a new version" (SLIP_SUPERSEDED)
-MSG-NB-251: "TSU clearance is required (&lt;rule&gt;) and not given" (TSU_NOT_CLEARED)</t>
+MSG-NB-237: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
+MSG-NB-238: "Missing documents: &lt;missing&gt;" (DOCUMENTS_MISSING)
+MSG-NB-239: "Choose the insurer and branch on the account before placement" (INSURER_NOT_SET)
+MSG-NB-240: "Placement slip file not found: &lt;format&gt;" (NOT_FOUND)
+MSG-NB-241: "Placement slip not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-242: "The account is &lt;&gt;; a slip needs Ready for placement" (NOT_READY_FOR_PLACEMENT)
+MSG-NB-243: "The payment or client confirmation is not recorded" (PAYMENT_NOT_CONFIRMED)
+MSG-NB-244: "&lt;name&gt; is set up for &lt;placement channel&gt; placements; only e-mail is available: set the insurer to e-mail placement" (PLACEMENT_CHANNEL_PARKED)
+MSG-NB-245: "Select at least one account" (PLACEMENT_NO_ACCOUNTS)
+MSG-NB-246: "Select the accounts to place" (SLIP_NO_ACCOUNTS)
+MSG-NB-247: "Placement prerequisites not met - &lt;problems&gt;" (SLIP_PREREQUISITES_UNMET)
+MSG-NB-248: "Slip &lt;display no&gt; was already replaced" (SLIP_SUPERSEDED)
+MSG-NB-249: "Slip &lt;slip no&gt; v&lt;version no&gt; was replaced by a new version" (SLIP_SUPERSEDED)
+MSG-NB-250: "TSU clearance is required (&lt;rule&gt;) and not given" (TSU_NOT_CLEARED)</t>
         </is>
       </c>
       <c r="M453" s="12" t="inlineStr">
@@ -49532,10 +49532,10 @@
       <c r="L454" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-255: "Choose the billing file format XLSX or ODS" (BILLING_FORMAT)
-MSG-NB-256: "No CBG Fire account awaiting payment is left to bill" (BILLING_NOTHING_TO_BILL)
-MSG-NB-257: "Not CBG Fire accounts awaiting payment, or already billed: &lt;wanted&gt;" (BILLING_NOT_CANDIDATE)
-MSG-NB-258: "Billing batch not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-254: "Choose the billing file format XLSX or ODS" (BILLING_FORMAT)
+MSG-NB-255: "No CBG Fire account awaiting payment is left to bill" (BILLING_NOTHING_TO_BILL)
+MSG-NB-256: "Not CBG Fire accounts awaiting payment, or already billed: &lt;wanted&gt;" (BILLING_NOT_CANDIDATE)
+MSG-NB-257: "Billing batch not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M454" s="12" t="inlineStr">
@@ -49610,19 +49610,19 @@
       <c r="L455" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-260: "&lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
-MSG-NB-261: "Billing batch &lt;batch no&gt; is closed" (BILLING_BATCH_CLOSED)
-MSG-NB-262: "Billing batch not found: &lt;batch id&gt;" (NOT_FOUND)
-MSG-NB-263: "Payment report line not found: &lt;line id&gt;" (NOT_FOUND)
-MSG-NB-264: "Payment report not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-265: "Row &lt;row no&gt; is already matched to &lt;arn&gt;" (PAYMENT_LINE_MATCHED)
-MSG-NB-266: "Choose the CLPC billing batch the report answers" (PAYMENT_REPORT_BATCH_REQUIRED)
-MSG-NB-267: "Payment report &lt;report no&gt; is &lt;status&gt;" (PAYMENT_REPORT_CLOSED)
-MSG-NB-268: "The payment report has no rows" (PAYMENT_REPORT_EMPTY)
-MSG-NB-269: "The CLPC report needs a 'PN No.' or 'Loan Application No.' column" (PAYMENT_REPORT_LAYOUT)
-MSG-NB-270: "The payment report needs an 'ARN' or 'Reference' column" (PAYMENT_REPORT_LAYOUT)
-MSG-NB-271: "Row &lt;row no&gt;: '&lt;value&gt;' is not a date (yyyy-mm-dd)" (PAYMENT_REPORT_VALUE)
-MSG-NB-272: "Row &lt;row no&gt;: '&lt;value&gt;' is not an amount" (PAYMENT_REPORT_VALUE)</t>
+MSG-NB-259: "&lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
+MSG-NB-260: "Billing batch &lt;batch no&gt; is closed" (BILLING_BATCH_CLOSED)
+MSG-NB-261: "Billing batch not found: &lt;batch id&gt;" (NOT_FOUND)
+MSG-NB-262: "Payment report line not found: &lt;line id&gt;" (NOT_FOUND)
+MSG-NB-263: "Payment report not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-264: "Row &lt;row no&gt; is already matched to &lt;arn&gt;" (PAYMENT_LINE_MATCHED)
+MSG-NB-265: "Choose the CLPC billing batch the report answers" (PAYMENT_REPORT_BATCH_REQUIRED)
+MSG-NB-266: "Payment report &lt;report no&gt; is &lt;status&gt;" (PAYMENT_REPORT_CLOSED)
+MSG-NB-267: "The payment report has no rows" (PAYMENT_REPORT_EMPTY)
+MSG-NB-268: "The CLPC report needs a 'PN No.' or 'Loan Application No.' column" (PAYMENT_REPORT_LAYOUT)
+MSG-NB-269: "The payment report needs an 'ARN' or 'Reference' column" (PAYMENT_REPORT_LAYOUT)
+MSG-NB-270: "Row &lt;row no&gt;: '&lt;value&gt;' is not a date (yyyy-mm-dd)" (PAYMENT_REPORT_VALUE)
+MSG-NB-271: "Row &lt;row no&gt;: '&lt;value&gt;' is not an amount" (PAYMENT_REPORT_VALUE)</t>
         </is>
       </c>
       <c r="M455" s="12" t="inlineStr">
@@ -49697,14 +49697,14 @@
       <c r="L456" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-275: "No account found for &lt;file name&gt;: choose the account (ARN)" (EPOLICY_ACCOUNT_NOT_FOUND)
-MSG-NB-276: "Account &lt;arn&gt; is &lt;&gt;; an e-policy is received once placed" (EPOLICY_ACCOUNT_STATUS)
-MSG-NB-277: "Upload between 1 and 50 e-policies at a time" (EPOLICY_FILE_COUNT)
-MSG-NB-278: "The e-policy &lt;file name&gt; is already &lt;&gt;" (EPOLICY_REVIEWED)
-MSG-NB-279: "This upload is &lt;status&gt;" (EPOLICY_UPLOAD_CLOSED)
-MSG-NB-280: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-281: "E-policy upload file not found: &lt;item id&gt;" (NOT_FOUND)
-MSG-NB-282: "Epolicy not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-274: "No account found for &lt;file name&gt;: choose the account (ARN)" (EPOLICY_ACCOUNT_NOT_FOUND)
+MSG-NB-275: "Account &lt;arn&gt; is &lt;&gt;; an e-policy is received once placed" (EPOLICY_ACCOUNT_STATUS)
+MSG-NB-276: "Upload between 1 and 50 e-policies at a time" (EPOLICY_FILE_COUNT)
+MSG-NB-277: "The e-policy &lt;file name&gt; is already &lt;&gt;" (EPOLICY_REVIEWED)
+MSG-NB-278: "This upload is &lt;status&gt;" (EPOLICY_UPLOAD_CLOSED)
+MSG-NB-279: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-280: "E-policy upload file not found: &lt;item id&gt;" (NOT_FOUND)
+MSG-NB-281: "Epolicy not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M456" s="12" t="inlineStr">
@@ -49779,10 +49779,10 @@
       <c r="L457" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-284: "Enter one policy number per policy year."
-MSG-NB-287: "The policy numbers must be different."
-MSG-NB-288: "Confirm the policy data of &lt;arn&gt; before sending the e-policy" (EPOLICY_NOT_CONFIRMED)
-MSG-NB-289: "The e-policy &lt;file name&gt; of &lt;arn&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)</t>
+MSG-NB-283: "Enter one policy number per policy year."
+MSG-NB-286: "The policy numbers must be different."
+MSG-NB-287: "Confirm the policy data of &lt;arn&gt; before sending the e-policy" (EPOLICY_NOT_CONFIRMED)
+MSG-NB-288: "The e-policy &lt;file name&gt; of &lt;arn&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)</t>
         </is>
       </c>
       <c r="M457" s="12" t="inlineStr">
@@ -49857,10 +49857,10 @@
       <c r="L458" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-292: "Account &lt;arn&gt; is &lt;status&gt;; it must be placed first" (IA_ACCOUNT_STATUS)
-MSG-NB-293: "Account &lt;arn&gt; has no mortgagee bank: no Insurance Advice" (IA_NOT_MORTGAGED)
-MSG-NB-294: "Select between 1 and 50 Insurance Advices" (IA_SELECTION)
-MSG-NB-295: "Insurance advice not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-291: "Account &lt;arn&gt; is &lt;status&gt;; it must be placed first" (IA_ACCOUNT_STATUS)
+MSG-NB-292: "Account &lt;arn&gt; has no mortgagee bank: no Insurance Advice" (IA_NOT_MORTGAGED)
+MSG-NB-293: "Select between 1 and 50 Insurance Advices" (IA_SELECTION)
+MSG-NB-294: "Insurance advice not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M458" s="12" t="inlineStr">
@@ -49935,8 +49935,8 @@
       <c r="L459" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-298: "Account &lt;arn&gt; has no contact e-mail: enter the recipient" (EPOLICY_NO_RECIPIENT)
-MSG-NB-299: "Select between 1 and 200 records" (ISSUANCE_SELECTION)</t>
+MSG-NB-297: "Account &lt;arn&gt; has no contact e-mail: enter the recipient" (EPOLICY_NO_RECIPIENT)
+MSG-NB-298: "Select between 1 and 200 records" (ISSUANCE_SELECTION)</t>
         </is>
       </c>
       <c r="M459" s="12" t="inlineStr">
@@ -50011,22 +50011,22 @@
       <c r="L460" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-302: "A negative endorsement reduces the sum insured (enter a minus)"
-MSG-NB-303: "A positive endorsement increases the sum insured"
-MSG-NB-304: "Choose the reason"
-MSG-NB-305: "Describe the cancellation"
-MSG-NB-306: "Describe the change"
-MSG-NB-307: "Enter a booking date that is not in the future"
-MSG-NB-308: "Enter a rate of zero or more, or leave it blank"
-MSG-NB-309: "Enter the cancellation date"
-MSG-NB-310: "Enter the change of the sum insured"
-MSG-NB-311: "Enter the effective date"
-MSG-NB-313: "The booking date cannot be in the future"
-MSG-NB-314: "No queued account to book" (BATCH_EMPTY)
-MSG-NB-315: "Select at least one account to book" (BATCH_EMPTY)
-MSG-NB-316: "The booking date &lt;booking date&gt; is in the future" (BOOKING_DATE_FUTURE)
-MSG-NB-317: "Booking queue not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-318: "Account &lt;arn&gt; is no longer queued (&lt;status&gt;)" (QUEUE_ENTRY_CLOSED)</t>
+MSG-NB-301: "A negative endorsement reduces the sum insured (enter a minus)"
+MSG-NB-302: "A positive endorsement increases the sum insured"
+MSG-NB-303: "Choose the reason"
+MSG-NB-304: "Describe the cancellation"
+MSG-NB-305: "Describe the change"
+MSG-NB-306: "Enter a booking date that is not in the future"
+MSG-NB-307: "Enter a rate of zero or more, or leave it blank"
+MSG-NB-308: "Enter the cancellation date"
+MSG-NB-309: "Enter the change of the sum insured"
+MSG-NB-310: "Enter the effective date"
+MSG-NB-312: "The booking date cannot be in the future"
+MSG-NB-313: "No queued account to book" (BATCH_EMPTY)
+MSG-NB-314: "Select at least one account to book" (BATCH_EMPTY)
+MSG-NB-315: "The booking date &lt;booking date&gt; is in the future" (BOOKING_DATE_FUTURE)
+MSG-NB-316: "Booking queue not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-317: "Account &lt;arn&gt; is no longer queued (&lt;status&gt;)" (QUEUE_ENTRY_CLOSED)</t>
         </is>
       </c>
       <c r="M460" s="12" t="inlineStr">
@@ -50101,25 +50101,25 @@
       <c r="L461" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-320: "Enter a booking date that is not in the future"
-MSG-NB-321: "Account &lt;arn&gt; has no insurer" (ACCOUNT_INSURER_MISSING)
-MSG-NB-322: "Account &lt;arn&gt; is &lt;&gt;: only issued policies are booked" (ACCOUNT_NOT_BOOKABLE)
-MSG-NB-323: "Account &lt;arn&gt; has no period of cover" (ACCOUNT_PERIOD_MISSING)
-MSG-NB-324: "Billing number &lt;billing no&gt; of &lt;insurer code&gt; is already on invoice &lt;invoice no&gt;" (BILLING_NO_DUPLICATE)
-MSG-NB-325: "Enter the insurer billing number" (BILLING_NO_REQUIRED)
-MSG-NB-326: "The insurer billing number has at most 60 characters" (BILLING_NO_TOO_LONG)
-MSG-NB-327: "The company has no branch to book invoices" (BOOKING_BRANCH_MISSING)
-MSG-NB-328: "The booking date &lt;date&gt; is in the future" (BOOKING_DATE_FUTURE)
-MSG-NB-329: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (CLIENT_PARTY_MISSING)
-MSG-NB-330: "Enter the cost center of account &lt;arn&gt;" (COST_CENTER_REQUIRED)
-MSG-NB-331: "Account &lt;arn&gt; is already booked" (DUPLICATE_BOOKING)
-MSG-NB-332: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (INSURER_PARTY_MISSING)
-MSG-NB-333: "Each insurer appears once with a positive share" (INSURER_SHARES_INVALID)
-MSG-NB-334: "Insurer shares must add up to 100% and include the lead insurer &lt;insurer code&gt;" (INSURER_SHARES_INVALID)
-MSG-NB-335: "Invoice &lt;arn&gt;/&lt;transaction no&gt; is &lt;status&gt;" (INVOICE_ALREADY_BOOKED)
-MSG-NB-336: "No invoice" (INVOICE_NOT_FOUND)
-MSG-NB-337: "Policy year &lt;policy year&gt; of &lt;arn&gt; is not due for booking" (POLICY_YEAR_NOT_DUE)
-MSG-NB-338: "Account &lt;arn&gt; has no rated premium" (PREMIUM_NOT_RATED)</t>
+MSG-NB-319: "Enter a booking date that is not in the future"
+MSG-NB-320: "Account &lt;arn&gt; has no insurer" (ACCOUNT_INSURER_MISSING)
+MSG-NB-321: "Account &lt;arn&gt; is &lt;&gt;: only issued policies are booked" (ACCOUNT_NOT_BOOKABLE)
+MSG-NB-322: "Account &lt;arn&gt; has no period of cover" (ACCOUNT_PERIOD_MISSING)
+MSG-NB-323: "Billing number &lt;billing no&gt; of &lt;insurer code&gt; is already on invoice &lt;invoice no&gt;" (BILLING_NO_DUPLICATE)
+MSG-NB-324: "Enter the insurer billing number" (BILLING_NO_REQUIRED)
+MSG-NB-325: "The insurer billing number has at most 60 characters" (BILLING_NO_TOO_LONG)
+MSG-NB-326: "The company has no branch to book invoices" (BOOKING_BRANCH_MISSING)
+MSG-NB-327: "The booking date &lt;date&gt; is in the future" (BOOKING_DATE_FUTURE)
+MSG-NB-328: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (CLIENT_PARTY_MISSING)
+MSG-NB-329: "Enter the cost center of account &lt;arn&gt;" (COST_CENTER_REQUIRED)
+MSG-NB-330: "Account &lt;arn&gt; is already booked" (DUPLICATE_BOOKING)
+MSG-NB-331: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (INSURER_PARTY_MISSING)
+MSG-NB-332: "Each insurer appears once with a positive share" (INSURER_SHARES_INVALID)
+MSG-NB-333: "Insurer shares must add up to 100% and include the lead insurer &lt;insurer code&gt;" (INSURER_SHARES_INVALID)
+MSG-NB-334: "Invoice &lt;arn&gt;/&lt;transaction no&gt; is &lt;status&gt;" (INVOICE_ALREADY_BOOKED)
+MSG-NB-335: "No invoice" (INVOICE_NOT_FOUND)
+MSG-NB-336: "Policy year &lt;policy year&gt; of &lt;arn&gt; is not due for booking" (POLICY_YEAR_NOT_DUE)
+MSG-NB-337: "Account &lt;arn&gt; has no rated premium" (PREMIUM_NOT_RATED)</t>
         </is>
       </c>
       <c r="M461" s="12" t="inlineStr">
@@ -50194,15 +50194,15 @@
       <c r="L462" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-344: "Account &lt;arn&gt; is &lt;&gt;: only booked accounts are endorsed" (ACCOUNT_NOT_BOOKED)
-MSG-NB-345: "A cancellation, and only a cancellation, has a kind" (CANCELLATION_KIND_REQUIRED)
-MSG-NB-346: "Enter the change of the sum insured or the premium" (ENDORSEMENT_CHANGE_REQUIRED)
-MSG-NB-347: "The effective date &lt;effective&gt; is not within a booked policy year of &lt;arn&gt;" (ENDORSEMENT_DATE_OUTSIDE_TERM)
-MSG-NB-348: "Enter the account, type, effective date and description" (ENDORSEMENT_INCOMPLETE)
-MSG-NB-349: "A negative endorsement or cancellation must return premium" (ENDORSEMENT_SIGN_MISMATCH)
-MSG-NB-350: "A positive endorsement must add premium" (ENDORSEMENT_SIGN_MISMATCH)
-MSG-NB-351: "The return premium exceeds the premium in force of policy year &lt;year&gt;" (RETURN_EXCEEDS_PREMIUM)
-MSG-NB-352: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
+MSG-NB-343: "Account &lt;arn&gt; is &lt;&gt;: only booked accounts are endorsed" (ACCOUNT_NOT_BOOKED)
+MSG-NB-344: "A cancellation, and only a cancellation, has a kind" (CANCELLATION_KIND_REQUIRED)
+MSG-NB-345: "Enter the change of the sum insured or the premium" (ENDORSEMENT_CHANGE_REQUIRED)
+MSG-NB-346: "The effective date &lt;effective&gt; is not within a booked policy year of &lt;arn&gt;" (ENDORSEMENT_DATE_OUTSIDE_TERM)
+MSG-NB-347: "Enter the account, type, effective date and description" (ENDORSEMENT_INCOMPLETE)
+MSG-NB-348: "A negative endorsement or cancellation must return premium" (ENDORSEMENT_SIGN_MISMATCH)
+MSG-NB-349: "A positive endorsement must add premium" (ENDORSEMENT_SIGN_MISMATCH)
+MSG-NB-350: "The return premium exceeds the premium in force of policy year &lt;year&gt;" (RETURN_EXCEEDS_PREMIUM)
+MSG-NB-351: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
         </is>
       </c>
       <c r="M462" s="12" t="inlineStr">
@@ -50277,14 +50277,14 @@
       <c r="L463" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-354: "Give the reason of the credit"
-MSG-NB-356: "Service invoice &lt;si no&gt; has &lt;commission&gt; commission and &lt;vat&gt; VAT left to credit" (CREDIT_EXCEEDS_INVOICE)
-MSG-NB-357: "&lt;si no&gt; is itself a credit" (CREDIT_OF_CREDIT)
-MSG-NB-358: "Service invoice not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-359: "Service invoice not found: &lt;si no&gt;" (NOT_FOUND)
-MSG-NB-360: "Service invoice type not found: &lt;code&gt;" (NOT_FOUND)
-MSG-NB-361: "Service invoices of type &lt;type code&gt; are issued automatically with the early remittance incentive" (SERVICE_INVOICE_AUTOMATIC_ONLY)
-MSG-NB-362: "Service invoice type &lt;code&gt; is inactive" (SERVICE_INVOICE_TYPE_INACTIVE)</t>
+MSG-NB-353: "Give the reason of the credit"
+MSG-NB-355: "Service invoice &lt;si no&gt; has &lt;commission&gt; commission and &lt;vat&gt; VAT left to credit" (CREDIT_EXCEEDS_INVOICE)
+MSG-NB-356: "&lt;si no&gt; is itself a credit" (CREDIT_OF_CREDIT)
+MSG-NB-357: "Service invoice not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-358: "Service invoice not found: &lt;si no&gt;" (NOT_FOUND)
+MSG-NB-359: "Service invoice type not found: &lt;code&gt;" (NOT_FOUND)
+MSG-NB-360: "Service invoices of type &lt;type code&gt; are issued automatically with the early remittance incentive" (SERVICE_INVOICE_AUTOMATIC_ONLY)
+MSG-NB-361: "Service invoice type &lt;code&gt; is inactive" (SERVICE_INVOICE_TYPE_INACTIVE)</t>
         </is>
       </c>
       <c r="M463" s="12" t="inlineStr">
@@ -50359,12 +50359,12 @@
       <c r="L464" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-365: "Service invoice type already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-366: "The period end must not be before the period start" (INCENTIVE_PERIOD_INVALID)
-MSG-NB-367: "Incentive rules are maintained in Product Maintenance &gt; Incentive Criteria" (INCENTIVE_RULES_FROZEN)
-MSG-NB-368: "Auto-booking rule not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-369: "Incentive rule not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-370: "Service invoice type not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-364: "Service invoice type already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-365: "The period end must not be before the period start" (INCENTIVE_PERIOD_INVALID)
+MSG-NB-366: "Incentive rules are maintained in Product Maintenance &gt; Incentive Criteria" (INCENTIVE_RULES_FROZEN)
+MSG-NB-367: "Auto-booking rule not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-368: "Incentive rule not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-369: "Service invoice type not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M464" s="12" t="inlineStr">
@@ -50439,16 +50439,17 @@
       <c r="L465" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-375: "Risk groups are numbers separated by ';'" (ACCEPTANCE_GROUP_INVALID)
-MSG-NB-376: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
-MSG-NB-377: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
-MSG-NB-378: "Business Type must be NEW_BUSINESS or RENEWAL" (BULK_BUSINESS_TYPE_INVALID)
-MSG-NB-379: "Enter an individual's name as 'Last, First'" (BULK_CLIENT_NAME_FORMAT)
-MSG-NB-380: "Give the Client Code or the Client Name" (BULK_CLIENT_REQUIRED)
-MSG-NB-381: "This file was already uploaded as &lt;job no&gt; (&lt;file name&gt;)" (BULK_DUPLICATE_FILE)
-MSG-NB-382: "The file has no data rows" (BULK_FILE_EMPTY)
-MSG-NB-383: "The file has no header row" (BULK_FILE_EMPTY)
-MSG-NB-384: "The file has &lt;size&gt; rows; the maximum is &lt;max&gt;" (BULK_FILE_TOO_LARGE)
+MSG-NB-374: "Risk groups are numbers separated by ';'" (ACCEPTANCE_GROUP_INVALID)
+MSG-NB-375: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
+MSG-NB-376: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
+MSG-NB-377: "Business Type must be NEW_BUSINESS or RENEWAL" (BULK_BUSINESS_TYPE_INVALID)
+MSG-NB-378: "Enter an individual's name as 'Last, First'" (BULK_CLIENT_NAME_FORMAT)
+MSG-NB-379: "Give the Client Code or the Client Name" (BULK_CLIENT_REQUIRED)
+MSG-NB-380: "This file was already uploaded as &lt;job no&gt; (&lt;file name&gt;)" (BULK_DUPLICATE_FILE)
+MSG-NB-381: "The file has no data rows" (BULK_FILE_EMPTY)
+MSG-NB-382: "The file has no header row" (BULK_FILE_EMPTY)
+MSG-NB-383: "The file has &lt;size&gt; rows; the maximum is &lt;max&gt;" (BULK_FILE_TOO_LARGE)
+MSG-NB-384: "The spreadsheet has more than 100000 rows" (BULK_FILE_TOO_LARGE)
 MSG-NB-385: "Upload an Excel (.xlsx), OpenDocument (.ods), CSV (.csv) or text (.txt) file" (BULK_FILE_TYPE)
 MSG-NB-386: "The file cannot be read: &lt;message&gt;" (BULK_FILE_UNREADABLE)
 MSG-NB-387: "The file is not an OpenDocument spreadsheet" (BULK_FILE_UNREADABLE)
@@ -51621,13 +51622,14 @@
 MSG-NB-518: "Booked invoice not found: &lt;id&gt;" (NOT_FOUND)
 MSG-NB-519: "Booked invoice not found: &lt;invoice no&gt;" (NOT_FOUND)
 MSG-NB-520: "Client not found: &lt;client id&gt;" (NOT_FOUND)
-MSG-NB-521: "Legacy account header not found: &lt;account id&gt;" (NOT_FOUND)
-MSG-NB-522: "Notification not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-523: "Proposal request not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-524: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-525: "Quotation not found: &lt;key&gt;" (NOT_FOUND)
-MSG-NB-526: "Quotation version not found: &lt;version no&gt;" (NOT_FOUND)
-MSG-NB-527: "Work item not found: &lt;case id&gt;" (NOT_FOUND)</t>
+MSG-NB-521: "Company not found: &lt;company id&gt;" (NOT_FOUND)
+MSG-NB-522: "Legacy account header not found: &lt;account id&gt;" (NOT_FOUND)
+MSG-NB-523: "Notification not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-524: "Proposal request not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-525: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-526: "Quotation not found: &lt;key&gt;" (NOT_FOUND)
+MSG-NB-527: "Quotation version not found: &lt;version no&gt;" (NOT_FOUND)
+MSG-NB-528: "Work item not found: &lt;case id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M480" s="12" t="inlineStr">

</xml_diff>

<commit_message>
BRD-01 New Business set v2.0 built with the UX documents 07 to 09 (interim, before the final screenshots)
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-1_Transactional/BRD-01_New_Business/04_BIBS_TestPlan_BRD-01_New_Business_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-1_Transactional/BRD-01_New_Business/04_BIBS_TestPlan_BRD-01_New_Business_v2.0.xlsx
@@ -44785,7 +44785,7 @@
       <c r="L395" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-05 Quotations of the FRS.
-Fields in this order: 1 My Drafts / For Review / Sent / Accepted / Expiring (Toggle buttons, mandatory -); 2 Drafts / For Review / Sent to Client / Accepted / Not Proceeded (Tab, mandatory -); 3 Search Quotation No., ARN or client (Text, mandatory N); 4 Only My Drafts / Expiring within 7 days (Check box, mandatory N); 5 Select (Check box, mandatory N); 6 Quotation No. (Column, mandatory -); 7 ARN (Column, mandatory -); 8 Client (Column, mandatory -); 9 Product (Column, mandatory -); 10 Insurer (Column, mandatory -); 11 Gross Premium (Column, mandatory -); 12 Valid Until (Column, mandatory -); 13 Status (Column, mandatory -).
+Fields in this order: 1 My Drafts / For Review / Sent / Accepted / Expiring (Toggle buttons, mandatory -); 2 Drafts / For Review / Sent to Client / Accepted / Not Proceeded (Tab, mandatory -); 3 Search Quotation No., ARN or client (Text, mandatory N); 4 Only My Drafts / Expiring within 7 days (Check box, mandatory N); 5 Select (Check box, mandatory N); 6 Quotation No. (Column, mandatory -); 7 ARN (Column, mandatory -); 8 Client (Column, mandatory -); 9 Product / Insurer (Column, mandatory -); 10 Gross Premium (Column, mandatory -); 11 Valid Until (Column, mandatory -); 12 Status (Column, mandatory -).
 Actions: Request Inbox; Bulk Upload; New Quotation; Send via Email (n); Open a row.</t>
         </is>
       </c>
@@ -45021,7 +45021,7 @@
       <c r="L398" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-08 Quotation Requests of the FRS.
-Fields in this order: 1 To Quote / Quoted / Closed (Tab, mandatory -); 2 Search Request No. (Text, mandatory N); 3 Request No. (Column, mandatory -); 4 Channel (Column, mandatory -); 5 Client / Prospect (Column, mandatory -); 6 Product (Column, mandatory -); 7 Requested Cover (Column, mandatory -); 8 Status (Column, mandatory -); 9 Channel (Drop-down, mandatory Y); 10 Source reference (Text, mandatory N); 11 Existing client (Look-up, mandatory Cond.: the client or the prospect name); 12 Prospect name (Text, mandatory Cond.: when no client is chosen); 13 Prospect e-mail (Text, mandatory N); 14 Prospect mobile (Text, mandatory N); 15 Requested product (Drop-down, mandatory N); 16 Market segment (Drop-down, mandatory N); 17 Requested cover (Text area, mandatory Y); 18 Request e-mail (File, mandatory N); 19 Reason for Closing (Text area, mandatory Y).
+Fields in this order: 1 To Quote / Quoted / Closed (Tab, mandatory -); 2 Search Request No. (Text, mandatory N); 3 Request No. (Column, mandatory -); 4 Channel (Column, mandatory -); 5 Client / Prospect (Column, mandatory -); 6 Product (Column, mandatory -); 7 Requested Cover (Column, mandatory -); 8 Status (Column, mandatory -); 9 Actions (Row action menu, mandatory -); 10 Channel (Drop-down, mandatory Y); 11 Source reference (Text, mandatory N); 12 Existing client (Look-up, mandatory Cond.: the client or the prospect name); 13 Prospect name (Text, mandatory Cond.: when no client is chosen); 14 Prospect e-mail (Text, mandatory N); 15 Prospect mobile (Text, mandatory N); 16 Requested product (Drop-down, mandatory N); 17 Market segment (Drop-down, mandatory N); 18 Requested cover (Text area, mandatory Y); 19 Request e-mail (File, mandatory N); 20 Reason for Closing (Text area, mandatory Y).
 Actions: Capture Request; Create Prospect; Create Quotation; Close; Open Quotation.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -45099,7 +45099,7 @@
       <c r="L399" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-09 Proposal Requests of the FRS.
-Fields in this order: 1 Drafts / For Approval / With TSU / With Client / Accepted / Not Proceeded (Tab, mandatory -); 2 Search PRF No., ARN or client (Text, mandatory N); 3 Only My PRFs (Check box, mandatory N); 4 PRF No. (Column, mandatory -); 5 ARN (Column, mandatory -); 6 Client (Column, mandatory -); 7 Product (Column, mandatory -); 8 Sum Insured (Column, mandatory -); 9 Slips (Column, mandatory -); 10 Chosen Insurer (Column, mandatory -); 11 Stage (Column, mandatory -).
+Fields in this order: 1 Drafts / For Approval / With TSU / With Client / Accepted / Not Proceeded (Tab, mandatory -); 2 Search PRF No., ARN or client (Text, mandatory N); 3 Only My PRFs (Check box, mandatory N); 4 PRF No. (Column, mandatory -); 5 ARN (Column, mandatory -); 6 Client (Column, mandatory -); 7 Product (Column, mandatory -); 8 Sum Insured (Column, mandatory -); 9 Slips / Chosen Insurer (Column, mandatory -); 10 Stage (Column, mandatory -).
 Actions: TSU Workbench; New PRF; Open a row.</t>
         </is>
       </c>
@@ -45334,7 +45334,7 @@
       <c r="L402" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-12 TSU Workbench of the FRS.
-Fields in this order: 1 Received by TSU, Quotation slip in preparation, Quotation slip for approval, Awaiting insurer terms, Insurer terms received, Proposal slip for approval (Tile, mandatory -); 2 Reference, Description, Stage, From, In Stage, Due, Assignee (Column, mandatory -).
+Fields in this order: 1 Received by TSU, Quotation slip in preparation, Quotation slip for approval, Awaiting insurer terms, Insurer terms received, Proposal slip for approval (Tile, mandatory -); 2 Reference, Description, Stage, From, In Stage, Due, Assignee, Actions (Column, mandatory -).
 Actions: Claim; Assign; Open a row.</t>
         </is>
       </c>
@@ -45411,7 +45411,7 @@
       <c r="L403" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-13 Accounts of the FRS.
-Fields in this order: 1 All / My Drafts / Returned to Me / Awaiting Payment / FFY / Direct Payment (Tab, mandatory -); 2 Search ARN, client code or name (Text, mandatory N); 3 PN Number (Text, mandatory N); 4 Plate, Conduction, Engine or Chassis (Text, mandatory N); 5 Location of Risk (Text, mandatory N); 6 Product (Text, mandatory N); 7 Insurer (Text, mandatory N); 8 Status (Drop-down, mandatory N); 9 Business Type (Drop-down, mandatory N); 10 Starts On or After / Starts On or Before (Date, mandatory N); 11 Include Voided (Check box, mandatory N); 12 ARN (Column, mandatory -); 13 Client (Column, mandatory -); 14 Product / Insurer / Period / Gross Premium (Column, mandatory -); 15 Status (Column, mandatory -); 16 Flags (Column, mandatory -); 17 Officer (Column, mandatory -).
+Fields in this order: 1 All / My Drafts / Returned to Me / Awaiting Payment / FFY / Direct Payment (Tab, mandatory -); 2 Search ARN, client code or name (Text, mandatory N); 3 PN Number (Text, mandatory N); 4 Plate, Conduction, Engine or Chassis (Text, mandatory N); 5 Location of Risk (Text, mandatory N); 6 Product (Text, mandatory N); 7 Insurer (Text, mandatory N); 8 Status (Drop-down, mandatory N); 9 Business Type (Drop-down, mandatory N); 10 Starts On or After / Starts On or Before (Date, mandatory N); 11 Include Voided (Check box, mandatory N); 12 ARN (Column, mandatory -); 13 Client (Column, mandatory -); 14 Product / Insurer (Column, mandatory -); 15 Period / Gross Premium (Column, mandatory -); 16 Status / Flags (Column, mandatory -); 17 Officer (Column, mandatory -).
 Actions: Bulk Upload; New Account; Filters / Apply Filters / Clear Filters; Open a row.</t>
         </is>
       </c>
@@ -45881,7 +45881,7 @@
         <is>
           <t>The screen matches SCR-NB-19 Account Placement of the FRS.
 Fields in this order: 1 Product, Insurer, Gross premium, Payment gate, Placement slip, Hold cover (Display, mandatory -); 2 Rule, Gate, Segment / line (Display, mandatory -); 3 Evidence (Table, mandatory -); 4 Confirmation channel (Drop-down, mandatory Y); 5 Remarks (Text area, mandatory N); 6 Placement slips (Table, mandatory -); 7 Hold covers (Table, mandatory -); 8 Hold cover starts on / Confirmed on (Date, mandatory N); 9 Insurer reference (Text, mandatory Y to record a confirmation); 10 Expires on (Date, mandatory N); 11 Insurer returns (Table, mandatory -).
-Actions: Open Account; Record Client Confirmation / Release Direct Payment; Generate Placement Slip; Send / Resend, Regenerate, PDF, Excel (slip); Request Hold Cover; Record Confirmation; Record Decline; Record Insurer Return; Resubmit for Placement; Return To Marketing; Cancel Placement / Reactivate.
+Actions: Open Account; Record Client Confirmation / Release Direct Payment; Generate Placement Slip; Send / Resend, Regenerate, Download PDF, Download Excel (slip); Request Hold Cover; Record Confirmation; Record Decline; Record Insurer Return; Resubmit for Placement; Return To Marketing; Cancel Placement / Reactivate.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -45959,8 +45959,8 @@
       <c r="L410" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-20 Placement Slips of the FRS.
-Fields in this order: 1 All Slips / To Send / Sent / Superseded (Tab, mandatory -); 2 Slip (Column, mandatory -); 3 Status (Column, mandatory -); 4 Insurer / Branch (Column, mandatory -); 5 Accounts (Column, mandatory -); 6 Sent (Column, mandatory -); 7 To, Cc, Subject, Message (Text, mandatory To, Subject and Message Y); 8 Password-protect the attachments (Check box, mandatory N).
-Actions: PDF / Excel; Send / Resend; Regenerate.
+Fields in this order: 1 All Slips / To Send / Sent / Superseded (Tab, mandatory -); 2 Slip (Column, mandatory -); 3 Status (Column, mandatory -); 4 Insurer / Branch (Column, mandatory -); 5 Accounts (Column, mandatory -); 6 Sent (Column, mandatory -); 7 Actions (Row action menu, mandatory -); 8 To, Cc, Subject, Message (Text, mandatory To, Subject and Message Y); 9 Password-protect the attachments (Check box, mandatory N).
+Actions: Download PDF / Download Excel; Send / Resend; Regenerate.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -46038,8 +46038,8 @@
       <c r="L411" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-21 CLPC Billing of the FRS.
-Fields in this order: 1 Billing Batches / Payment Reports (Tab, mandatory -); 2 Reference, Borrower, PN No., Loan Application No., Premium (Column, mandatory -); 3 Select (Check box, mandatory N); 4 Batch, Billing Date, Status, Accounts, Total Premium (Column, mandatory -); 5 Report, Kind, File, Status, Matched / Unpaid / Unmatched / Ambiguous, Uploaded (Column, mandatory -); 6 Report (Drop-down, mandatory Y); 7 Billing batch (Drop-down, mandatory Y for a CLPC report); 8 File (File, mandatory Y).
-Actions: Bill Selected (n) / Bill All; Excel / ODS; Upload Payment Report / Upload Report.
+Fields in this order: 1 Billing Batches / Payment Reports (Tab, mandatory -); 2 Reference, Borrower, PN No., Loan Application No., Premium (Column, mandatory -); 3 Select (Check box, mandatory N); 4 Batch, Billing Date, Status, Accounts, Total Premium, Actions (Column, mandatory -); 5 Report, Kind, File, Status, Matched / Unpaid / Unmatched / Ambiguous, Uploaded (Column, mandatory -); 6 Report (Drop-down, mandatory Y); 7 Billing batch (Drop-down, mandatory Y for a CLPC report); 8 File (File, mandatory Y).
+Actions: Bill Selected (n) / Bill All; Download Excel / Download ODS; Upload Payment Report / Upload Report.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -46117,7 +46117,7 @@
       <c r="L412" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-22 Payment Report of the FRS.
-Fields in this order: 1 Matched / Unpaid / Unmatched / Ambiguous (Tile, mandatory -); 2 Row, Reported Reference, Paid, Amount, Payment Date, Account, Detail (Column, mandatory -); 3 Account (ARN) (Drop-down or Text, mandatory Y).
+Fields in this order: 1 Matched / Unpaid / Unmatched / Ambiguous (Tile, mandatory -); 2 Row, Reported Reference, Paid, Amount, Payment Date, Account, Detail, Actions (Column, mandatory -); 3 Account (ARN) (Drop-down or Text, mandatory Y).
 Actions: Match; Confirm Matches; Discard.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -46195,8 +46195,8 @@
       <c r="L413" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-23 Issuance Workbench of the FRS.
-Fields in this order: 1 Placed – Awaiting Policy / Policy Received – Review Extraction / Ready to Dispatch / IA to Generate (Tile and tab, mandatory -); 2 Search Reference No. (Text, mandatory N); 3 Select (Check box, mandatory N); 4 Name / Client Code (Column, mandatory -); 5 ARN (Column, mandatory -); 6 Status (Column, mandatory -); 7 Product Line (Column, mandatory -); 8 Policy No. (Column, mandatory -); 9 E-policy / Mortgagee / Upload E-policy (Column, mandatory -).
-Actions: Upload E-policies; Upload E-policy (row); Generate Insurance Advice; Send E-policies.</t>
+Fields in this order: 1 Placed – Awaiting Policy / Policy Received – Review Extraction / Ready to Dispatch / IA to Generate (Tile and tab, mandatory -); 2 Search Reference No. (Text, mandatory N); 3 Select (Check box, mandatory N); 4 Name / Client Code (Column, mandatory -); 5 ARN (Column, mandatory -); 6 Status (Column, mandatory -); 7 Product Line (Column, mandatory -); 8 Policy No. (Column, mandatory -); 9 E-policy / Mortgagee / Actions (Column, mandatory -).
+Actions: Upload E-policies; Upload E-policy (row action menu); Generate Insurance Advice; Send E-policies.</t>
         </is>
       </c>
       <c r="M413" s="12" t="inlineStr">
@@ -46431,8 +46431,8 @@
       <c r="L416" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-26 Insurance Advice of the FRS.
-Fields in this order: 1 Search IA No., ARN or client (Text, mandatory N); 2 Select (Check box, mandatory N); 3 IA No. (Column, mandatory -); 4 Insured / ARN (Column, mandatory -); 5 Mortgagee (Column, mandatory -); 6 Policy No. (Column, mandatory -); 7 Generated (Column, mandatory -); 8 Status / Last Sent (Column, mandatory -); 9 Accounts (ARN) (Text area, mandatory Y); 10 To (Text, mandatory Y); 11 Cc, Password hint (Text, mandatory N).
-Actions: Generate Insurance Advice; Send Selected; PDF.
+Fields in this order: 1 Search IA No., ARN or client (Text, mandatory N); 2 Select (Check box, mandatory N); 3 IA No. (Column, mandatory -); 4 Insured / ARN (Column, mandatory -); 5 Mortgagee (Column, mandatory -); 6 Policy No. (Column, mandatory -); 7 Generated (Column, mandatory -); 8 Status / Last Sent (Column, mandatory -); 9 Actions (Row action menu, mandatory -); 10 Accounts (ARN) (Text area, mandatory Y); 11 To (Text, mandatory Y); 12 Cc, Password hint (Text, mandatory N).
+Actions: Generate Insurance Advice; Send Selected; Download PDF.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -46510,8 +46510,8 @@
       <c r="L417" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-27 E-policy Dispatch of the FRS.
-Fields in this order: 1 Ready to Dispatch / Dispatch Report (Tab, mandatory -); 2 Name / Client Code, ARN, Policy No., E-policy (Column, mandatory -); 3 To, Cc, Subject, Message (Text, mandatory To, Subject and Message Y); 4 Password hint (Text, mandatory N); 5 Queued, Reference No., To, Subject, Outcome, Delivered (Column, mandatory -).
-Actions: Send (row); Send Selected.
+Fields in this order: 1 Ready to Dispatch / Dispatch Report (Tab, mandatory -); 2 Name / Client Code, ARN, Policy No., E-policy, Actions (Column, mandatory -); 3 To, Cc, Subject, Message (Text, mandatory To, Subject and Message Y); 4 Password hint (Text, mandatory N); 5 Queued, Reference No., To, Subject, Outcome, Delivered (Column, mandatory -).
+Actions: Send (row action menu); Send Selected.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -46590,7 +46590,7 @@
         <is>
           <t>The screen matches SCR-NB-28 Booking Workbench of the FRS.
 Fields in this order: 1 Ready to Book / Queued for Batch / Booked Today / Failed (Tile, mandatory -); 2 Ready to Book / Queued for Batch / Booked Account / Failed (Tab, mandatory -); 3 Accounts sent from placement (Banner, mandatory -); 4 Search Reference No. (Text, mandatory N); 5 Product line (Drop-down, mandatory N); 6 Select (Check box, mandatory N); 7 Name / Client Code, ARN, Invoice No., Status, Product Line, Department, Booking Date (Column, mandatory -); 8 Booking date (Date, mandatory Y); 9 Booking date (Date, mandatory N); 10 Cost center (Text, mandatory N).
-Actions: Batch Runs; Upload Bookings; Add All to Batch; Add to Batch; Book Now; Confirm Batch; Cancel Batch; Edit / Remove (row); Open a row.
+Actions: Batch Runs; Upload Bookings; Add All to Batch; Add to Batch; Book Now; Confirm Batch; Cancel Batch; Edit / Remove (row action menu); Open a row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -46905,7 +46905,7 @@
       <c r="L422" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-32 Service Invoices of the FRS.
-Fields in this order: 1 All / Service Invoices / Credits (Tab, mandatory -); 2 Search Service Invoice No., invoice, ARN or recipient (Text, mandatory N); 3 Service Invoice No., Issue Date, Kind, Type, Booked Invoice, ARN, Recipient, Net, Dispatch (Column, mandatory -); 4 Service invoice, Invoice, ARN (Reference, mandatory -); 5 Recipient, Billing e-mail, Issue date, Template, Owner, Credit of (Display, mandatory -); 6 Lines (Display, mandatory -); 7 E-mail dispatch problem (Banner, mandatory -); 8 Commission to credit / VAT to credit (Amount, mandatory N); 9 Reason (Text, mandatory Y).
+Fields in this order: 1 All / Service Invoices / Credits (Tab, mandatory -); 2 Search Service Invoice No., invoice, ARN or recipient (Text, mandatory N); 3 Service Invoice No., Kind / Type, Recipient, Invoice No., Issue Date, Net, E-mail (Column, mandatory -); 4 Service invoice, Invoice, ARN (Reference, mandatory -); 5 Recipient, Billing e-mail, Issue date, Template, Owner, Credit of (Display, mandatory -); 6 Lines (Display, mandatory -); 7 E-mail dispatch problem (Banner, mandatory -); 8 Commission to credit / VAT to credit (Amount, mandatory N); 9 Reason (Text, mandatory Y).
 Actions: Open a row; Download PDF; Send via Email; Credit.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -47377,7 +47377,7 @@
       <c r="L428" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-38 My Work of the FRS.
-Fields in this order: 1 Assigned to me / Open in my queues / Overdue / Queues I work (Figure, mandatory -); 2 One tile per stage of each workflow the user works (Tile, mandatory -); 3 Assigned to me / Team queue / All my queues (Tab, mandatory -); 4 Overdue only (Check box, mandatory N); 5 Reference or name (Text, mandatory N); 6 Reference, Description, Stage, From, In Stage, Due, Assignee (Column, mandatory -); 7 Assignee (Drop-down, mandatory N).
+Fields in this order: 1 Assigned to me / Open in my queues / Overdue / Queues I work (Figure, mandatory -); 2 One tile per stage of each workflow the user works (Tile, mandatory -); 3 Assigned to me / Team queue / All my queues (Tab, mandatory -); 4 Overdue only (Check box, mandatory N); 5 Reference or name (Text, mandatory N); 6 Reference, Description, Stage, From, In Stage, Due, Assignee, Actions (Column, mandatory -); 7 Assignee (Drop-down, mandatory N).
 Actions: Claim; Assign; Clear Stage Filter; Open a row.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -47691,7 +47691,7 @@
       <c r="L432" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-42 Lists of Values of the FRS.
-Fields in this order: 1 List names (List, mandatory -); 2 Code, Label, Order, Parent, Effective, Status, Maker / Checker (Column, mandatory -); 3 Code (Text, mandatory Y); 4 Label (Text, mandatory Y); 5 Sort order (Number, mandatory Y); 6 Parent value (Text, mandatory N); 7 Effective from (Date, mandatory Y); 8 Effective to (Date, mandatory N).
+Fields in this order: 1 List names (List, mandatory -); 2 Code, Label, Order, Parent, Effective, Status, Maker / Checker, Actions (Column, mandatory -); 3 Code (Text, mandatory Y); 4 Label (Text, mandatory Y); 5 Sort order (Number, mandatory Y); 6 Parent value (Text, mandatory N); 7 Effective from (Date, mandatory Y); 8 Effective to (Date, mandatory N).
 Actions: New Value; Edit / Deactivate; Authorize.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -47770,8 +47770,8 @@
       <c r="L433" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-43 Data Retention of the FRS.
-Fields in this order: 1 Record Type, Statuses, Years Online, Years Archive, Action, Rule, Last Review, Eligible Records (Column, mandatory -); 2 Statuses (Text, mandatory Y); 3 Years online (Number, mandatory Y); 4 Years in archive (Number, mandatory Y); 5 Action (Drop-down, mandatory N); 6 Active (Check box, mandatory N); 7 Description (Text, mandatory Y); 8 Reference, Description, Status, Last Activity (Column, mandatory -).
-Actions: Run Review Now; Records (row); Edit (row).
+Fields in this order: 1 Record Type, Statuses, Years Online, Years Archive, Action, Rule, Last Review, Eligible Records, Actions (Column, mandatory -); 2 Statuses (Text, mandatory Y); 3 Years online (Number, mandatory Y); 4 Years in archive (Number, mandatory Y); 5 Action (Drop-down, mandatory N); 6 Active (Check box, mandatory N); 7 Description (Text, mandatory Y); 8 Reference, Description, Status, Last Activity (Column, mandatory -).
+Actions: Run Review Now; Records (row action menu); Edit (row action menu).
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -47849,8 +47849,8 @@
       <c r="L434" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-NB-44 Document Templates of the FRS.
-Fields in this order: 1 Template list (List, mandatory -); 2 Current version (Display, mandatory -); 3 Version, Title, Effective from, Status, Created (Column, mandatory -); 4 Load from Word (File, mandatory N); 5 Title (Text, mandatory Y); 6 Effective from (Date, mandatory Y); 7 Text (Text area, mandatory Y).
-Actions: New Version; Download icon of a version (as Word).
+Fields in this order: 1 Template list (List, mandatory -); 2 Current version (Display, mandatory -); 3 Version, Title, Effective from, Status, Created, Actions (Column, mandatory -); 4 Load from Word (File, mandatory N); 5 Title (Text, mandatory Y); 6 Effective from (Date, mandatory Y); 7 Text (Text area, mandatory Y).
+Actions: New Version; Download Word (row action menu of a version).
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -48183,11 +48183,11 @@
       <c r="L438" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-035: "The client is inactive" (CLIENT_INACTIVE)
-MSG-NB-036: "Complete the client information before you &lt;step&gt;: &lt;missing&gt;" (CLIENT_INFO_INCOMPLETE)
-MSG-NB-037: "Upload the mandatory KYC documents before you &lt;step&gt;: &lt;missing&gt;" (KYC_DOCUMENTS_MISSING)
-MSG-NB-038: "The KYC must be verified by a user other than its maker" (KYC_FOUR_EYES)
-MSG-NB-039: "Client &lt;code&gt; has no verified KYC" (KYC_NOT_VERIFIED)</t>
+MSG-NB-034: "The client is inactive" (CLIENT_INACTIVE)
+MSG-NB-035: "Complete the client information before you &lt;step&gt;: &lt;missing&gt;" (CLIENT_INFO_INCOMPLETE)
+MSG-NB-036: "Upload the mandatory KYC documents before you &lt;step&gt;: &lt;missing&gt;" (KYC_DOCUMENTS_MISSING)
+MSG-NB-037: "The KYC must be verified by a user other than its maker" (KYC_FOUR_EYES)
+MSG-NB-038: "Client &lt;code&gt; has no verified KYC" (KYC_NOT_VERIFIED)</t>
         </is>
       </c>
       <c r="M438" s="12" t="inlineStr">
@@ -48262,16 +48262,16 @@
       <c r="L439" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-040: "Enter the first day"
-MSG-NB-041: "Enter the instruction"
-MSG-NB-044: "Select the instruction type"
-MSG-NB-047: "The end date must not be before the start date"
-MSG-NB-048: "The client is already tagged &lt;tag code&gt;" (CLIENT_TAG_EXISTS)
-MSG-NB-049: "The end date must not be before the start date" (INSTRUCTION_DATES)
-MSG-NB-050: "An ended instruction cannot be changed" (INSTRUCTION_ENDED)
-MSG-NB-051: "Enter the instruction" (INSTRUCTION_TEXT_REQUIRED)
-MSG-NB-052: "Client instruction not found: &lt;instruction id&gt;" (NOT_FOUND)
-MSG-NB-053: "Client tag not found: &lt;tag code&gt;" (NOT_FOUND)</t>
+MSG-NB-039: "Enter the first day"
+MSG-NB-040: "Enter the instruction"
+MSG-NB-043: "Select the instruction type"
+MSG-NB-046: "The end date must not be before the start date"
+MSG-NB-047: "The client is already tagged &lt;tag code&gt;" (CLIENT_TAG_EXISTS)
+MSG-NB-048: "The end date must not be before the start date" (INSTRUCTION_DATES)
+MSG-NB-049: "An ended instruction cannot be changed" (INSTRUCTION_ENDED)
+MSG-NB-050: "Enter the instruction" (INSTRUCTION_TEXT_REQUIRED)
+MSG-NB-051: "Client instruction not found: &lt;instruction id&gt;" (NOT_FOUND)
+MSG-NB-052: "Client tag not found: &lt;tag code&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M439" s="12" t="inlineStr">
@@ -48346,11 +48346,11 @@
       <c r="L440" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-056: "Client information incomplete: &lt;missing&gt;" (INFO_INCOMPLETE)
-MSG-NB-057: "The periodic KYC review was due on &lt;kyc review due&gt;" (KYC_EXPIRED)
-MSG-NB-058: "Confirmed client without a sub-ledger party code" (MISSING_PARTY)
-MSG-NB-059: "Party &lt;party code&gt; is not active" (PARTY_INACTIVE)
-MSG-NB-060: "Party &lt;party code&gt; does not exist" (PARTY_NOT_FOUND)</t>
+MSG-NB-055: "Client information incomplete: &lt;missing&gt;" (INFO_INCOMPLETE)
+MSG-NB-056: "The periodic KYC review was due on &lt;kyc review due&gt;" (KYC_EXPIRED)
+MSG-NB-057: "Confirmed client without a sub-ledger party code" (MISSING_PARTY)
+MSG-NB-058: "Party &lt;party code&gt; is not active" (PARTY_INACTIVE)
+MSG-NB-059: "Party &lt;party code&gt; does not exist" (PARTY_NOT_FOUND)</t>
         </is>
       </c>
       <c r="M440" s="12" t="inlineStr">
@@ -48425,15 +48425,15 @@
       <c r="L441" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-067: "Choose the client or give the prospect name"
-MSG-NB-068: "Describe the requested cover"
-MSG-NB-069: "Enter a valid e-mail address"
-MSG-NB-071: "Quotation request not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-072: "Give the client code or the prospect's name" (QUOTATION_REQUEST_CLIENT)
-MSG-NB-073: "Request &lt;request no&gt; is already &lt;status&gt;" (QUOTATION_REQUEST_CLOSED)
-MSG-NB-074: "Request &lt;external ref&gt; of &lt;channel&gt; was already received" (QUOTATION_REQUEST_DUPLICATE)
-MSG-NB-075: "Request &lt;request no&gt; has a client" (QUOTATION_REQUEST_HAS_CLIENT)
-MSG-NB-076: "Give the reason for closing" (QUOTATION_REQUEST_REASON)</t>
+MSG-NB-066: "Choose the client or give the prospect name"
+MSG-NB-067: "Describe the requested cover"
+MSG-NB-068: "Enter a valid e-mail address"
+MSG-NB-070: "Quotation request not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-071: "Give the client code or the prospect's name" (QUOTATION_REQUEST_CLIENT)
+MSG-NB-072: "Request &lt;request no&gt; is already &lt;status&gt;" (QUOTATION_REQUEST_CLOSED)
+MSG-NB-073: "Request &lt;external ref&gt; of &lt;channel&gt; was already received" (QUOTATION_REQUEST_DUPLICATE)
+MSG-NB-074: "Request &lt;request no&gt; has a client" (QUOTATION_REQUEST_HAS_CLIENT)
+MSG-NB-075: "Give the reason for closing" (QUOTATION_REQUEST_REASON)</t>
         </is>
       </c>
       <c r="M441" s="12" t="inlineStr">
@@ -48508,9 +48508,9 @@
       <c r="L442" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-079: "Select the quotations to send" (QUOTATION_BATCH_EMPTY)
-MSG-NB-080: "Cannot send: &lt;problems&gt;" (QUOTATION_BATCH_INVALID)
-MSG-NB-081: "Quotation &lt;quotation no&gt; must be approved before it is sent" (QUOTATION_NOT_APPROVED)</t>
+MSG-NB-078: "Select the quotations to send" (QUOTATION_BATCH_EMPTY)
+MSG-NB-079: "Cannot send: &lt;problems&gt;" (QUOTATION_BATCH_INVALID)
+MSG-NB-080: "Quotation &lt;quotation no&gt; must be approved before it is sent" (QUOTATION_NOT_APPROVED)</t>
         </is>
       </c>
       <c r="M442" s="12" t="inlineStr">
@@ -48585,9 +48585,9 @@
       <c r="L443" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-082: "Attach the client's acceptance e-mail (document type Client acceptance e-mail) first" (ACCEPTANCE_EMAIL_REQUIRED)
-MSG-NB-083: "The quotation offers risk groups &lt;offered&gt; only" (ACCEPTANCE_GROUP_UNKNOWN)
-MSG-NB-084: "Record the client's acceptance first" (QUOTATION_NOT_ACCEPTED)</t>
+MSG-NB-081: "Attach the client's acceptance e-mail (document type Client acceptance e-mail) first" (ACCEPTANCE_EMAIL_REQUIRED)
+MSG-NB-082: "The quotation offers risk groups &lt;offered&gt; only" (ACCEPTANCE_GROUP_UNKNOWN)
+MSG-NB-083: "Record the client's acceptance first" (QUOTATION_NOT_ACCEPTED)</t>
         </is>
       </c>
       <c r="M443" s="12" t="inlineStr">
@@ -48662,30 +48662,30 @@
       <c r="L444" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-087: "Add at least one risk item"
-MSG-NB-088: "Enter the sum insured of every item"
-MSG-NB-089: "Select the client or prospect"
-MSG-NB-090: "Select the product"
-MSG-NB-091: "The period end must be after the period start"
-MSG-NB-092: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
-MSG-NB-093: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-094: "Give the client code or the prospect's name" (QUOTATION_CLIENT_REQUIRED)
-MSG-NB-095: "The validity date has passed: change it before submitting" (QUOTATION_EXPIRED)
-MSG-NB-096: "A quotation is approved by someone other than its maker" (QUOTATION_FOUR_EYES)
-MSG-NB-097: "Select the client and the product" (QUOTATION_INCOMPLETE)
-MSG-NB-098: "Select the product" (QUOTATION_INCOMPLETE)
-MSG-NB-099: "Quotation &lt;quotation no&gt; is &lt;&gt;" (QUOTATION_NOT_EDITABLE)
-MSG-NB-100: "The premium cannot be computed: give each item a sum insured (and a rate when the product has no default rate)" (QUOTATION_NOT_RATED)
-MSG-NB-101: "Add at least one risk item" (QUOTATION_NO_ITEMS)
-MSG-NB-102: "The period end must be after the period start" (QUOTATION_PERIOD_INVALID)
-MSG-NB-103: "The product of a quotation cannot change" (QUOTATION_PRODUCT_FIXED)
-MSG-NB-104: "Renewal &lt;renewal ref&gt; already has quotation &lt;quotation no&gt;" (QUOTATION_RENEWAL_EXISTS)
-MSG-NB-105: "Choose the market segment on the Client step before you submit the quotation" (QUOTATION_SEGMENT_REQUIRED)
-MSG-NB-106: "The validity date cannot be in the past" (QUOTATION_VALIDITY_PAST)
-MSG-NB-107: "Version &lt;version no&gt; was submitted and is read-only" (QUOTATION_VERSION_FROZEN)
-MSG-NB-108: "The quotation is priced on version &lt;scheme version&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: save the quotation again to re-price it" (RATE_SCHEME_NOT_CURRENT)
-MSG-NB-109: "Unknown rating basis &lt;value&gt;" (RATING_BASIS_INVALID)
-MSG-NB-110: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-086: "Add at least one risk item"
+MSG-NB-087: "Enter the sum insured of every item"
+MSG-NB-088: "Select the client or prospect"
+MSG-NB-089: "Select the product"
+MSG-NB-090: "The period end must be after the period start"
+MSG-NB-091: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
+MSG-NB-092: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-093: "Give the client code or the prospect's name" (QUOTATION_CLIENT_REQUIRED)
+MSG-NB-094: "The validity date has passed: change it before submitting" (QUOTATION_EXPIRED)
+MSG-NB-095: "A quotation is approved by someone other than its maker" (QUOTATION_FOUR_EYES)
+MSG-NB-096: "Select the client and the product" (QUOTATION_INCOMPLETE)
+MSG-NB-097: "Select the product" (QUOTATION_INCOMPLETE)
+MSG-NB-098: "Quotation &lt;quotation no&gt; is &lt;&gt;" (QUOTATION_NOT_EDITABLE)
+MSG-NB-099: "The premium cannot be computed: give each item a sum insured (and a rate when the product has no default rate)" (QUOTATION_NOT_RATED)
+MSG-NB-100: "Add at least one risk item" (QUOTATION_NO_ITEMS)
+MSG-NB-101: "The period end must be after the period start" (QUOTATION_PERIOD_INVALID)
+MSG-NB-102: "The product of a quotation cannot change" (QUOTATION_PRODUCT_FIXED)
+MSG-NB-103: "Renewal &lt;renewal ref&gt; already has quotation &lt;quotation no&gt;" (QUOTATION_RENEWAL_EXISTS)
+MSG-NB-104: "Choose the market segment on the Client step before you submit the quotation" (QUOTATION_SEGMENT_REQUIRED)
+MSG-NB-105: "The validity date cannot be in the past" (QUOTATION_VALIDITY_PAST)
+MSG-NB-106: "Version &lt;version no&gt; was submitted and is read-only" (QUOTATION_VERSION_FROZEN)
+MSG-NB-107: "The quotation is priced on version &lt;scheme version&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: save the quotation again to re-price it" (RATE_SCHEME_NOT_CURRENT)
+MSG-NB-108: "Unknown rating basis &lt;value&gt;" (RATING_BASIS_INVALID)
+MSG-NB-109: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M444" s="12" t="inlineStr">
@@ -48760,8 +48760,8 @@
       <c r="L445" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-112: "Enter the item rate between 0 and 100"
-MSG-NB-113: "Explain why the scheme rate cannot be used"</t>
+MSG-NB-111: "Enter the item rate between 0 and 100"
+MSG-NB-112: "Explain why the scheme rate cannot be used"</t>
         </is>
       </c>
       <c r="M445" s="12" t="inlineStr">
@@ -48836,20 +48836,20 @@
       <c r="L446" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-120: "Select the client or prospect"
-MSG-NB-121: "Select the product"
-MSG-NB-122: "The period end must be after the period start"
-MSG-NB-123: "Attach the mandatory documents: &lt;missing&gt;" (MISSING_DOCUMENTS)
-MSG-NB-124: "Proposal request not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-125: "A PRF is approved by someone other than its maker" (PRF_FOUR_EYES)
-MSG-NB-126: "Complete the PRF header" (PRF_INCOMPLETE)
-MSG-NB-127: "Describe the risk (sections or risk items) before submitting" (PRF_INCOMPLETE)
-MSG-NB-128: "PRF &lt;prf no&gt; cannot be changed while &lt;&gt;" (PRF_NOT_EDITABLE)
-MSG-NB-129: "No TSU rule applies to this package risk: quote it directly as a package quotation" (PRF_NOT_NEEDED)
-MSG-NB-130: "The period end must be after the period start" (PRF_PERIOD_INVALID)
-MSG-NB-131: "The product of a PRF cannot change" (PRF_PRODUCT_FIXED)
-MSG-NB-132: "Renewal &lt;renewal ref&gt; already has proposal request &lt;prf no&gt;" (PROPOSAL_RENEWAL_EXISTS)
-MSG-NB-133: "Product &lt;code&gt; is not offered to segment &lt;market segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-119: "Select the client or prospect"
+MSG-NB-120: "Select the product"
+MSG-NB-121: "The period end must be after the period start"
+MSG-NB-122: "Attach the mandatory documents: &lt;missing&gt;" (MISSING_DOCUMENTS)
+MSG-NB-123: "Proposal request not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-124: "A PRF is approved by someone other than its maker" (PRF_FOUR_EYES)
+MSG-NB-125: "Complete the PRF header" (PRF_INCOMPLETE)
+MSG-NB-126: "Describe the risk (sections or risk items) before submitting" (PRF_INCOMPLETE)
+MSG-NB-127: "PRF &lt;prf no&gt; cannot be changed while &lt;&gt;" (PRF_NOT_EDITABLE)
+MSG-NB-128: "No TSU rule applies to this package risk: quote it directly as a package quotation" (PRF_NOT_NEEDED)
+MSG-NB-129: "The period end must be after the period start" (PRF_PERIOD_INVALID)
+MSG-NB-130: "The product of a PRF cannot change" (PRF_PRODUCT_FIXED)
+MSG-NB-131: "Renewal &lt;renewal ref&gt; already has proposal request &lt;prf no&gt;" (PROPOSAL_RENEWAL_EXISTS)
+MSG-NB-132: "Product &lt;code&gt; is not offered to segment &lt;market segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M446" s="12" t="inlineStr">
@@ -48924,27 +48924,27 @@
       <c r="L447" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-137: "Enter the premium quoted"
-MSG-NB-144: "Attach the client's acceptance e-mail first" (ACCEPTANCE_EMAIL_REQUIRED)
-MSG-NB-145: "The proposal covers risk groups &lt;offered&gt; only" (ACCEPTANCE_GROUP_UNKNOWN)
-MSG-NB-146: "&lt;name&gt; has no placement e-mail address" (INSURER_NO_EMAIL)
-MSG-NB-147: "Insurer response not found: &lt;response id&gt;" (NOT_FOUND)
-MSG-NB-148: "Record the client's acceptance of the proposal first" (PROPOSAL_NOT_ACCEPTED)
-MSG-NB-149: "No terms of &lt;chosen insurer&gt; are recorded" (PROPOSAL_TERMS_MISSING)
-MSG-NB-150: "The proposal slip is approved by another TSU officer" (PS_FOUR_EYES)
-MSG-NB-151: "Choose the insurer (or flag the recommended one) for the proposal slip" (PS_INSURER_REQUIRED)
-MSG-NB-152: "No proposal slip has been prepared yet" (PS_NOT_PREPARED)
-MSG-NB-153: "&lt;insurer name&gt; has not quoted terms" (PS_TERMS_MISSING)
-MSG-NB-154: "The chosen terms are gone" (PS_TERMS_MISSING)
-MSG-NB-155: "Insurers are selected before the quotation slip is submitted" (QS_CLOSED)
-MSG-NB-156: "The quotation slip is approved by another TSU officer" (QS_FOUR_EYES)
-MSG-NB-157: "No quotation slip has been prepared yet" (QS_NOT_PREPARED)
-MSG-NB-158: "Select at least one insurer of the panel for the quotation slip" (QS_NO_INSURER)
-MSG-NB-159: "Insurer terms are keyed in after the quotation slip is sent" (RESPONSES_CLOSED)
-MSG-NB-160: "Only received terms can be recommended" (RESPONSE_NOT_RECEIVED)
-MSG-NB-161: "Enter the premium quoted by &lt;insurer name&gt;" (RESPONSE_PREMIUM_REQUIRED)
-MSG-NB-162: "No insurer terms have been received" (TERMS_NONE)
-MSG-NB-163: "&lt;pending&gt; insurer(s) have not answered: close the request to proceed" (TERMS_PENDING)</t>
+MSG-NB-136: "Enter the premium quoted"
+MSG-NB-143: "Attach the client's acceptance e-mail first" (ACCEPTANCE_EMAIL_REQUIRED)
+MSG-NB-144: "The proposal covers risk groups &lt;offered&gt; only" (ACCEPTANCE_GROUP_UNKNOWN)
+MSG-NB-145: "&lt;name&gt; has no placement e-mail address" (INSURER_NO_EMAIL)
+MSG-NB-146: "Insurer response not found: &lt;response id&gt;" (NOT_FOUND)
+MSG-NB-147: "Record the client's acceptance of the proposal first" (PROPOSAL_NOT_ACCEPTED)
+MSG-NB-148: "No terms of &lt;chosen insurer&gt; are recorded" (PROPOSAL_TERMS_MISSING)
+MSG-NB-149: "The proposal slip is approved by another TSU officer" (PS_FOUR_EYES)
+MSG-NB-150: "Choose the insurer (or flag the recommended one) for the proposal slip" (PS_INSURER_REQUIRED)
+MSG-NB-151: "No proposal slip has been prepared yet" (PS_NOT_PREPARED)
+MSG-NB-152: "&lt;insurer name&gt; has not quoted terms" (PS_TERMS_MISSING)
+MSG-NB-153: "The chosen terms are gone" (PS_TERMS_MISSING)
+MSG-NB-154: "Insurers are selected before the quotation slip is submitted" (QS_CLOSED)
+MSG-NB-155: "The quotation slip is approved by another TSU officer" (QS_FOUR_EYES)
+MSG-NB-156: "No quotation slip has been prepared yet" (QS_NOT_PREPARED)
+MSG-NB-157: "Select at least one insurer of the panel for the quotation slip" (QS_NO_INSURER)
+MSG-NB-158: "Insurer terms are keyed in after the quotation slip is sent" (RESPONSES_CLOSED)
+MSG-NB-159: "Only received terms can be recommended" (RESPONSE_NOT_RECEIVED)
+MSG-NB-160: "Enter the premium quoted by &lt;insurer name&gt;" (RESPONSE_PREMIUM_REQUIRED)
+MSG-NB-161: "No insurer terms have been received" (TERMS_NONE)
+MSG-NB-162: "&lt;pending&gt; insurer(s) have not answered: close the request to proceed" (TERMS_PENDING)</t>
         </is>
       </c>
       <c r="M447" s="12" t="inlineStr">
@@ -49019,12 +49019,12 @@
       <c r="L448" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-166: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_ACTIVE)
-MSG-NB-167: "Product &lt;product code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
-MSG-NB-168: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
-MSG-NB-169: "Account &lt;arn&gt; is not tagged Free First Year" (FFY_NOT_TAGGED)
-MSG-NB-170: "Enter the Free First Year start" (FFY_START_REQUIRED)
-MSG-NB-171: "The payment gate of &lt;arn&gt; is passed" (PAYMENT_ARRANGEMENT_LOCKED)</t>
+MSG-NB-165: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_ACTIVE)
+MSG-NB-166: "Product &lt;product code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
+MSG-NB-167: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
+MSG-NB-168: "Account &lt;arn&gt; is not tagged Free First Year" (FFY_NOT_TAGGED)
+MSG-NB-169: "Enter the Free First Year start" (FFY_START_REQUIRED)
+MSG-NB-170: "The payment gate of &lt;arn&gt; is passed" (PAYMENT_ARRANGEMENT_LOCKED)</t>
         </is>
       </c>
       <c r="M448" s="12" t="inlineStr">
@@ -49099,22 +49099,22 @@
       <c r="L449" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-173: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
-MSG-NB-174: "Account &lt;arn&gt; is not a renewal account" (ACCOUNT_NOT_RENEWAL)
-MSG-NB-175: "Account &lt;arn&gt; is &lt;&gt;, not &lt;status&gt;" (ACCOUNT_STATUS_INVALID)
-MSG-NB-176: "Account &lt;arn&gt; is &lt;status&gt;, not DRAFT" (ACCOUNT_STATUS_INVALID)
-MSG-NB-177: "The ARN must read ARN-yyyy-nnnnnn (or ARN-yyyy-nnnnnn-nn)" (ARN_INVALID)
-MSG-NB-178: "An account already has ARN &lt;given&gt;" (ARN_IN_USE)
-MSG-NB-179: "The insurer of account &lt;arn&gt; cannot be changed when it is &lt;&gt;" (INSURER_CHANGE_NOT_ALLOWED)
-MSG-NB-180: "Select the new insurer" (INSURER_REQUIRED)
-MSG-NB-181: "Select an insurer other than the current one" (INSURER_UNCHANGED)
-MSG-NB-182: "Account not found: &lt;arn&gt;" (NOT_FOUND)
-MSG-NB-183: "Account not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-184: "Account &lt;arn&gt; is set up with insurer &lt;insurer code&gt;" (PLACEMENT_INSURER_MISMATCH)
-MSG-NB-185: "Attach the issued policy (policy copy or e-policy) before direct booking" (POLICY_DOCUMENT_REQUIRED)
-MSG-NB-186: "Account &lt;arn&gt; needs &lt;term years&gt; policy number(s), one per year" (POLICY_NUMBERS_MISMATCH)
-MSG-NB-187: "TSU clearance is given before the account is validated" (TSU_CLEARANCE_CLOSED)
-MSG-NB-188: "TSU must clear the account first: &lt;reason&gt;" (TSU_CLEARANCE_REQUIRED)</t>
+MSG-NB-172: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
+MSG-NB-173: "Account &lt;arn&gt; is not a renewal account" (ACCOUNT_NOT_RENEWAL)
+MSG-NB-174: "Account &lt;arn&gt; is &lt;&gt;, not &lt;status&gt;" (ACCOUNT_STATUS_INVALID)
+MSG-NB-175: "Account &lt;arn&gt; is &lt;status&gt;, not DRAFT" (ACCOUNT_STATUS_INVALID)
+MSG-NB-176: "The ARN must read ARN-yyyy-nnnnnn (or ARN-yyyy-nnnnnn-nn)" (ARN_INVALID)
+MSG-NB-177: "An account already has ARN &lt;given&gt;" (ARN_IN_USE)
+MSG-NB-178: "The insurer of account &lt;arn&gt; cannot be changed when it is &lt;&gt;" (INSURER_CHANGE_NOT_ALLOWED)
+MSG-NB-179: "Select the new insurer" (INSURER_REQUIRED)
+MSG-NB-180: "Select an insurer other than the current one" (INSURER_UNCHANGED)
+MSG-NB-181: "Account not found: &lt;arn&gt;" (NOT_FOUND)
+MSG-NB-182: "Account not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-183: "Account &lt;arn&gt; is set up with insurer &lt;insurer code&gt;" (PLACEMENT_INSURER_MISMATCH)
+MSG-NB-184: "Attach the issued policy (policy copy or e-policy) before direct booking" (POLICY_DOCUMENT_REQUIRED)
+MSG-NB-185: "Account &lt;arn&gt; needs &lt;term years&gt; policy number(s), one per year" (POLICY_NUMBERS_MISMATCH)
+MSG-NB-186: "TSU clearance is given before the account is validated" (TSU_CLEARANCE_CLOSED)
+MSG-NB-187: "TSU must clear the account first: &lt;reason&gt;" (TSU_CLEARANCE_REQUIRED)</t>
         </is>
       </c>
       <c r="M449" s="12" t="inlineStr">
@@ -49189,25 +49189,25 @@
       <c r="L450" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-190: "Choose the client and product to save the draft."
-MSG-NB-191: "The draft is not saved yet: click Save Draft to check it before submission."
-MSG-NB-192: "The draft was not saved: correct what the message above describes, then save the draft again."
-MSG-NB-193: "The draft was not saved: its risks are already on the account shown above. Change the risk items, or open the existing account instead."
-MSG-NB-194: "Select the client" (ACCOUNT_CLIENT_REQUIRED)
-MSG-NB-195: "Complete the mandatory fields of &lt;product code&gt;: &lt;check&gt;" (ACCOUNT_INCOMPLETE)
-MSG-NB-196: "The period end must be after the period start" (ACCOUNT_PERIOD_INVALID)
-MSG-NB-197: "Select the product" (ACCOUNT_PRODUCT_REQUIRED)
-MSG-NB-198: "Only a renewal account names the policy it renews (&lt;renewal of ref&gt;)" (ACCOUNT_RENEWAL_OF_NOT_RENEWAL)
-MSG-NB-199: "A multi-year account needs a term of at least 2 years" (ACCOUNT_TERM_INVALID)
-MSG-NB-200: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
-MSG-NB-201: "Duplicate of existing account &lt;arns&gt;: &lt;details&gt;" (DUPLICATE_ACCOUNT)
-MSG-NB-202: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
-MSG-NB-203: "Upload the mandatory documents: &lt;check&gt;" (MISSING_DOCUMENTS)
-MSG-NB-204: "Product &lt;code&gt; carries no mortgagee" (MORTGAGE_NOT_APPLICABLE)
-MSG-NB-205: "Product &lt;code&gt; allows a term of up to &lt;max term years&gt; year(s)" (MULTI_YEAR_NOT_ALLOWED)
-MSG-NB-206: "Compute the premium (sum insured and rate of every item) first" (PREMIUM_NOT_RATED)
-MSG-NB-207: "Account &lt;arn&gt; is priced on version &lt;priced&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: update the account to re-price it or request a rate exception" (RATE_SCHEME_NOT_CURRENT)
-MSG-NB-208: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
+MSG-NB-189: "Choose the client and product to save the draft."
+MSG-NB-190: "The draft is not saved yet: click Save Draft to check it before submission."
+MSG-NB-191: "The draft was not saved: correct what the message above describes, then save the draft again."
+MSG-NB-192: "The draft was not saved: its risks are already on the account shown above. Change the risk items, or open the existing account instead."
+MSG-NB-193: "Select the client" (ACCOUNT_CLIENT_REQUIRED)
+MSG-NB-194: "Complete the mandatory fields of &lt;product code&gt;: &lt;check&gt;" (ACCOUNT_INCOMPLETE)
+MSG-NB-195: "The period end must be after the period start" (ACCOUNT_PERIOD_INVALID)
+MSG-NB-196: "Select the product" (ACCOUNT_PRODUCT_REQUIRED)
+MSG-NB-197: "Only a renewal account names the policy it renews (&lt;renewal of ref&gt;)" (ACCOUNT_RENEWAL_OF_NOT_RENEWAL)
+MSG-NB-198: "A multi-year account needs a term of at least 2 years" (ACCOUNT_TERM_INVALID)
+MSG-NB-199: "Product &lt;code&gt; cannot be paid directly to the insurer" (DIRECT_PAYMENT_NOT_ELIGIBLE)
+MSG-NB-200: "Duplicate of existing account &lt;arns&gt;: &lt;details&gt;" (DUPLICATE_ACCOUNT)
+MSG-NB-201: "Product &lt;code&gt; is not Free First Year eligible" (FFY_NOT_ELIGIBLE)
+MSG-NB-202: "Upload the mandatory documents: &lt;check&gt;" (MISSING_DOCUMENTS)
+MSG-NB-203: "Product &lt;code&gt; carries no mortgagee" (MORTGAGE_NOT_APPLICABLE)
+MSG-NB-204: "Product &lt;code&gt; allows a term of up to &lt;max term years&gt; year(s)" (MULTI_YEAR_NOT_ALLOWED)
+MSG-NB-205: "Compute the premium (sum insured and rate of every item) first" (PREMIUM_NOT_RATED)
+MSG-NB-206: "Account &lt;arn&gt; is priced on version &lt;priced&gt; of &lt;code&gt;; version &lt;scheme version&gt; is current: update the account to re-price it or request a rate exception" (RATE_SCHEME_NOT_CURRENT)
+MSG-NB-207: "Product &lt;code&gt; is not offered to segment &lt;segment&gt;" (SEGMENT_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M450" s="12" t="inlineStr">
@@ -49282,9 +49282,9 @@
       <c r="L451" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-213: "Account &lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
-MSG-NB-214: "Account &lt;arn&gt; is not paid directly to the insurer" (GATE_NOT_DIRECT_PAYMENT)
-MSG-NB-215: "Account &lt;arn&gt; must be paid: match its payment from a payment report" (GATE_REQUIRES_PAYMENT)</t>
+MSG-NB-212: "Account &lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
+MSG-NB-213: "Account &lt;arn&gt; is not paid directly to the insurer" (GATE_NOT_DIRECT_PAYMENT)
+MSG-NB-214: "Account &lt;arn&gt; must be paid: match its payment from a payment report" (GATE_REQUIRES_PAYMENT)</t>
         </is>
       </c>
       <c r="M451" s="12" t="inlineStr">
@@ -49359,17 +49359,17 @@
       <c r="L452" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-218: "Record Hold Cover Confirmation"
-MSG-NB-219: "Record Hold Cover Decline"
-MSG-NB-220: "The hold cover of &lt;arn&gt; is &lt;status&gt;" (HOLD_COVER_CLOSED)
-MSG-NB-221: "The hold cover cannot expire before it starts (&lt;start date&gt;)" (HOLD_COVER_DATES)
-MSG-NB-222: "Account &lt;arn&gt; has no open hold cover" (HOLD_COVER_NONE)
-MSG-NB-223: "Account &lt;arn&gt; has no open hold cover request" (HOLD_COVER_NONE)
-MSG-NB-224: "A hold cover is requested while the account is being placed, not &lt;&gt;" (HOLD_COVER_NOT_ALLOWED)
-MSG-NB-225: "Account &lt;arn&gt; already has a hold cover requested or confirmed" (HOLD_COVER_OPEN)
-MSG-NB-226: "Enter the insurer's reference" (HOLD_COVER_REFERENCE)
-MSG-NB-227: "Choose the insurer on the account first" (INSURER_NOT_SET)
-MSG-NB-228: "Select the reason" (REASSIGN_REASON_REQUIRED)</t>
+MSG-NB-217: "Record Hold Cover Confirmation"
+MSG-NB-218: "Record Hold Cover Decline"
+MSG-NB-219: "The hold cover of &lt;arn&gt; is &lt;status&gt;" (HOLD_COVER_CLOSED)
+MSG-NB-220: "The hold cover cannot expire before it starts (&lt;start date&gt;)" (HOLD_COVER_DATES)
+MSG-NB-221: "Account &lt;arn&gt; has no open hold cover" (HOLD_COVER_NONE)
+MSG-NB-222: "Account &lt;arn&gt; has no open hold cover request" (HOLD_COVER_NONE)
+MSG-NB-223: "A hold cover is requested while the account is being placed, not &lt;&gt;" (HOLD_COVER_NOT_ALLOWED)
+MSG-NB-224: "Account &lt;arn&gt; already has a hold cover requested or confirmed" (HOLD_COVER_OPEN)
+MSG-NB-225: "Enter the insurer's reference" (HOLD_COVER_REFERENCE)
+MSG-NB-226: "Choose the insurer on the account first" (INSURER_NOT_SET)
+MSG-NB-227: "Select the reason" (REASSIGN_REASON_REQUIRED)</t>
         </is>
       </c>
       <c r="M452" s="12" t="inlineStr">
@@ -49444,20 +49444,20 @@
       <c r="L453" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-237: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
-MSG-NB-238: "Missing documents: &lt;missing&gt;" (DOCUMENTS_MISSING)
-MSG-NB-239: "Choose the insurer and branch on the account before placement" (INSURER_NOT_SET)
-MSG-NB-240: "Placement slip file not found: &lt;format&gt;" (NOT_FOUND)
-MSG-NB-241: "Placement slip not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-242: "The account is &lt;&gt;; a slip needs Ready for placement" (NOT_READY_FOR_PLACEMENT)
-MSG-NB-243: "The payment or client confirmation is not recorded" (PAYMENT_NOT_CONFIRMED)
-MSG-NB-244: "&lt;name&gt; is set up for &lt;placement channel&gt; placements; only e-mail is available: set the insurer to e-mail placement" (PLACEMENT_CHANNEL_PARKED)
-MSG-NB-245: "Select at least one account" (PLACEMENT_NO_ACCOUNTS)
-MSG-NB-246: "Select the accounts to place" (SLIP_NO_ACCOUNTS)
-MSG-NB-247: "Placement prerequisites not met - &lt;problems&gt;" (SLIP_PREREQUISITES_UNMET)
-MSG-NB-248: "Slip &lt;display no&gt; was already replaced" (SLIP_SUPERSEDED)
-MSG-NB-249: "Slip &lt;slip no&gt; v&lt;version no&gt; was replaced by a new version" (SLIP_SUPERSEDED)
-MSG-NB-250: "TSU clearance is required (&lt;rule&gt;) and not given" (TSU_NOT_CLEARED)</t>
+MSG-NB-235: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
+MSG-NB-236: "Missing documents: &lt;names&gt;" (DOCUMENTS_MISSING)
+MSG-NB-237: "Choose the insurer and branch on the account before placement" (INSURER_NOT_SET)
+MSG-NB-238: "Placement slip file not found: &lt;format&gt;" (NOT_FOUND)
+MSG-NB-239: "Placement slip not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-240: "The account is &lt;&gt;; a slip needs Ready for placement" (NOT_READY_FOR_PLACEMENT)
+MSG-NB-241: "The payment or client confirmation is not recorded" (PAYMENT_NOT_CONFIRMED)
+MSG-NB-242: "&lt;name&gt; is set up for &lt;placement channel&gt; placements; only e-mail is available: set the insurer to e-mail placement" (PLACEMENT_CHANNEL_PARKED)
+MSG-NB-243: "Select at least one account" (PLACEMENT_NO_ACCOUNTS)
+MSG-NB-244: "Select the accounts to place" (SLIP_NO_ACCOUNTS)
+MSG-NB-245: "Placement prerequisites not met - &lt;problems&gt;" (SLIP_PREREQUISITES_UNMET)
+MSG-NB-246: "Slip &lt;display no&gt; was already replaced" (SLIP_SUPERSEDED)
+MSG-NB-247: "Slip &lt;slip no&gt; v&lt;version no&gt; was replaced by a new version" (SLIP_SUPERSEDED)
+MSG-NB-248: "TSU clearance is required (&lt;rule&gt;) and not given" (TSU_NOT_CLEARED)</t>
         </is>
       </c>
       <c r="M453" s="12" t="inlineStr">
@@ -49532,10 +49532,10 @@
       <c r="L454" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-254: "Choose the billing file format XLSX or ODS" (BILLING_FORMAT)
-MSG-NB-255: "No CBG Fire account awaiting payment is left to bill" (BILLING_NOTHING_TO_BILL)
-MSG-NB-256: "Not CBG Fire accounts awaiting payment, or already billed: &lt;wanted&gt;" (BILLING_NOT_CANDIDATE)
-MSG-NB-257: "Billing batch not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-252: "Choose the billing file format XLSX or ODS" (BILLING_FORMAT)
+MSG-NB-253: "No CBG Fire account awaiting payment is left to bill" (BILLING_NOTHING_TO_BILL)
+MSG-NB-254: "Not CBG Fire accounts awaiting payment, or already billed: &lt;wanted&gt;" (BILLING_NOT_CANDIDATE)
+MSG-NB-255: "Billing batch not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M454" s="12" t="inlineStr">
@@ -49610,19 +49610,19 @@
       <c r="L455" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-259: "&lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
-MSG-NB-260: "Billing batch &lt;batch no&gt; is closed" (BILLING_BATCH_CLOSED)
-MSG-NB-261: "Billing batch not found: &lt;batch id&gt;" (NOT_FOUND)
-MSG-NB-262: "Payment report line not found: &lt;line id&gt;" (NOT_FOUND)
-MSG-NB-263: "Payment report not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-264: "Row &lt;row no&gt; is already matched to &lt;arn&gt;" (PAYMENT_LINE_MATCHED)
-MSG-NB-265: "Choose the CLPC billing batch the report answers" (PAYMENT_REPORT_BATCH_REQUIRED)
-MSG-NB-266: "Payment report &lt;report no&gt; is &lt;status&gt;" (PAYMENT_REPORT_CLOSED)
-MSG-NB-267: "The payment report has no rows" (PAYMENT_REPORT_EMPTY)
-MSG-NB-268: "The CLPC report needs a 'PN No.' or 'Loan Application No.' column" (PAYMENT_REPORT_LAYOUT)
-MSG-NB-269: "The payment report needs an 'ARN' or 'Reference' column" (PAYMENT_REPORT_LAYOUT)
-MSG-NB-270: "Row &lt;row no&gt;: '&lt;value&gt;' is not a date (yyyy-mm-dd)" (PAYMENT_REPORT_VALUE)
-MSG-NB-271: "Row &lt;row no&gt;: '&lt;value&gt;' is not an amount" (PAYMENT_REPORT_VALUE)</t>
+MSG-NB-257: "&lt;arn&gt; is &lt;&gt;, not awaiting payment" (ACCOUNT_NOT_AWAITING_PAYMENT)
+MSG-NB-258: "Billing batch &lt;batch no&gt; is closed" (BILLING_BATCH_CLOSED)
+MSG-NB-259: "Billing batch not found: &lt;batch id&gt;" (NOT_FOUND)
+MSG-NB-260: "Payment report line not found: &lt;line id&gt;" (NOT_FOUND)
+MSG-NB-261: "Payment report not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-262: "Row &lt;row no&gt; is already matched to &lt;arn&gt;" (PAYMENT_LINE_MATCHED)
+MSG-NB-263: "Choose the CLPC billing batch the report answers" (PAYMENT_REPORT_BATCH_REQUIRED)
+MSG-NB-264: "Payment report &lt;report no&gt; is &lt;status&gt;" (PAYMENT_REPORT_CLOSED)
+MSG-NB-265: "The payment report has no rows" (PAYMENT_REPORT_EMPTY)
+MSG-NB-266: "The CLPC report needs a 'PN No.' or 'Loan Application No.' column" (PAYMENT_REPORT_LAYOUT)
+MSG-NB-267: "The payment report needs an 'ARN' or 'Reference' column" (PAYMENT_REPORT_LAYOUT)
+MSG-NB-268: "Row &lt;row no&gt;: '&lt;value&gt;' is not a date (yyyy-mm-dd)" (PAYMENT_REPORT_VALUE)
+MSG-NB-269: "Row &lt;row no&gt;: '&lt;value&gt;' is not an amount" (PAYMENT_REPORT_VALUE)</t>
         </is>
       </c>
       <c r="M455" s="12" t="inlineStr">
@@ -49697,14 +49697,14 @@
       <c r="L456" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-274: "No account found for &lt;file name&gt;: choose the account (ARN)" (EPOLICY_ACCOUNT_NOT_FOUND)
-MSG-NB-275: "Account &lt;arn&gt; is &lt;&gt;; an e-policy is received once placed" (EPOLICY_ACCOUNT_STATUS)
-MSG-NB-276: "Upload between 1 and 50 e-policies at a time" (EPOLICY_FILE_COUNT)
-MSG-NB-277: "The e-policy &lt;file name&gt; is already &lt;&gt;" (EPOLICY_REVIEWED)
-MSG-NB-278: "This upload is &lt;status&gt;" (EPOLICY_UPLOAD_CLOSED)
-MSG-NB-279: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-280: "E-policy upload file not found: &lt;item id&gt;" (NOT_FOUND)
-MSG-NB-281: "Epolicy not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-272: "No account found for &lt;file name&gt;: choose the account (ARN)" (EPOLICY_ACCOUNT_NOT_FOUND)
+MSG-NB-273: "Account &lt;arn&gt; is &lt;&gt;; an e-policy is received once placed" (EPOLICY_ACCOUNT_STATUS)
+MSG-NB-274: "Upload between 1 and 50 e-policies at a time" (EPOLICY_FILE_COUNT)
+MSG-NB-275: "The e-policy &lt;file name&gt; is already &lt;&gt;" (EPOLICY_REVIEWED)
+MSG-NB-276: "This upload is &lt;status&gt;" (EPOLICY_UPLOAD_CLOSED)
+MSG-NB-277: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-278: "E-policy upload file not found: &lt;item id&gt;" (NOT_FOUND)
+MSG-NB-279: "Epolicy not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M456" s="12" t="inlineStr">
@@ -49779,10 +49779,10 @@
       <c r="L457" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-283: "Enter one policy number per policy year."
-MSG-NB-286: "The policy numbers must be different."
-MSG-NB-287: "Confirm the policy data of &lt;arn&gt; before sending the e-policy" (EPOLICY_NOT_CONFIRMED)
-MSG-NB-288: "The e-policy &lt;file name&gt; of &lt;arn&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)</t>
+MSG-NB-281: "Enter one policy number per policy year."
+MSG-NB-284: "The policy numbers must be different."
+MSG-NB-285: "Confirm the policy data of &lt;arn&gt; before sending the e-policy" (EPOLICY_NOT_CONFIRMED)
+MSG-NB-286: "The e-policy &lt;file name&gt; of &lt;arn&gt; is already &lt;status&gt;" (EPOLICY_REVIEWED)</t>
         </is>
       </c>
       <c r="M457" s="12" t="inlineStr">
@@ -49857,10 +49857,10 @@
       <c r="L458" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-291: "Account &lt;arn&gt; is &lt;status&gt;; it must be placed first" (IA_ACCOUNT_STATUS)
-MSG-NB-292: "Account &lt;arn&gt; has no mortgagee bank: no Insurance Advice" (IA_NOT_MORTGAGED)
-MSG-NB-293: "Select between 1 and 50 Insurance Advices" (IA_SELECTION)
-MSG-NB-294: "Insurance advice not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-289: "Account &lt;arn&gt; is &lt;status&gt;; it must be placed first" (IA_ACCOUNT_STATUS)
+MSG-NB-290: "Account &lt;arn&gt; has no mortgagee bank: no Insurance Advice" (IA_NOT_MORTGAGED)
+MSG-NB-291: "Select between 1 and 50 Insurance Advices" (IA_SELECTION)
+MSG-NB-292: "Insurance advice not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M458" s="12" t="inlineStr">
@@ -49935,8 +49935,8 @@
       <c r="L459" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-297: "Account &lt;arn&gt; has no contact e-mail: enter the recipient" (EPOLICY_NO_RECIPIENT)
-MSG-NB-298: "Select between 1 and 200 records" (ISSUANCE_SELECTION)</t>
+MSG-NB-295: "Account &lt;arn&gt; has no contact e-mail: enter the recipient" (EPOLICY_NO_RECIPIENT)
+MSG-NB-296: "Select between 1 and 200 records" (ISSUANCE_SELECTION)</t>
         </is>
       </c>
       <c r="M459" s="12" t="inlineStr">
@@ -50011,22 +50011,22 @@
       <c r="L460" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-301: "A negative endorsement reduces the sum insured (enter a minus)"
-MSG-NB-302: "A positive endorsement increases the sum insured"
-MSG-NB-303: "Choose the reason"
-MSG-NB-304: "Describe the cancellation"
-MSG-NB-305: "Describe the change"
-MSG-NB-306: "Enter a booking date that is not in the future"
-MSG-NB-307: "Enter a rate of zero or more, or leave it blank"
-MSG-NB-308: "Enter the cancellation date"
-MSG-NB-309: "Enter the change of the sum insured"
-MSG-NB-310: "Enter the effective date"
-MSG-NB-312: "The booking date cannot be in the future"
-MSG-NB-313: "No queued account to book" (BATCH_EMPTY)
-MSG-NB-314: "Select at least one account to book" (BATCH_EMPTY)
-MSG-NB-315: "The booking date &lt;booking date&gt; is in the future" (BOOKING_DATE_FUTURE)
-MSG-NB-316: "Booking queue not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-317: "Account &lt;arn&gt; is no longer queued (&lt;status&gt;)" (QUEUE_ENTRY_CLOSED)</t>
+MSG-NB-299: "A negative endorsement reduces the sum insured (enter a minus)"
+MSG-NB-300: "A positive endorsement increases the sum insured"
+MSG-NB-301: "Choose the reason"
+MSG-NB-302: "Describe the cancellation"
+MSG-NB-303: "Describe the change"
+MSG-NB-304: "Enter a booking date that is not in the future"
+MSG-NB-305: "Enter a rate of zero or more, or leave it blank"
+MSG-NB-306: "Enter the cancellation date"
+MSG-NB-307: "Enter the change of the sum insured"
+MSG-NB-308: "Enter the effective date"
+MSG-NB-310: "The booking date cannot be in the future"
+MSG-NB-311: "No queued account to book" (BATCH_EMPTY)
+MSG-NB-312: "Select at least one account to book" (BATCH_EMPTY)
+MSG-NB-313: "The booking date &lt;booking date&gt; is in the future" (BOOKING_DATE_FUTURE)
+MSG-NB-314: "Booking queue not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-315: "Account &lt;arn&gt; is no longer queued (&lt;status&gt;)" (QUEUE_ENTRY_CLOSED)</t>
         </is>
       </c>
       <c r="M460" s="12" t="inlineStr">
@@ -50101,25 +50101,25 @@
       <c r="L461" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-319: "Enter a booking date that is not in the future"
-MSG-NB-320: "Account &lt;arn&gt; has no insurer" (ACCOUNT_INSURER_MISSING)
-MSG-NB-321: "Account &lt;arn&gt; is &lt;&gt;: only issued policies are booked" (ACCOUNT_NOT_BOOKABLE)
-MSG-NB-322: "Account &lt;arn&gt; has no period of cover" (ACCOUNT_PERIOD_MISSING)
-MSG-NB-323: "Billing number &lt;billing no&gt; of &lt;insurer code&gt; is already on invoice &lt;invoice no&gt;" (BILLING_NO_DUPLICATE)
-MSG-NB-324: "Enter the insurer billing number" (BILLING_NO_REQUIRED)
-MSG-NB-325: "The insurer billing number has at most 60 characters" (BILLING_NO_TOO_LONG)
-MSG-NB-326: "The company has no branch to book invoices" (BOOKING_BRANCH_MISSING)
-MSG-NB-327: "The booking date &lt;date&gt; is in the future" (BOOKING_DATE_FUTURE)
-MSG-NB-328: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (CLIENT_PARTY_MISSING)
-MSG-NB-329: "Enter the cost center of account &lt;arn&gt;" (COST_CENTER_REQUIRED)
-MSG-NB-330: "Account &lt;arn&gt; is already booked" (DUPLICATE_BOOKING)
-MSG-NB-331: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (INSURER_PARTY_MISSING)
-MSG-NB-332: "Each insurer appears once with a positive share" (INSURER_SHARES_INVALID)
-MSG-NB-333: "Insurer shares must add up to 100% and include the lead insurer &lt;insurer code&gt;" (INSURER_SHARES_INVALID)
-MSG-NB-334: "Invoice &lt;arn&gt;/&lt;transaction no&gt; is &lt;status&gt;" (INVOICE_ALREADY_BOOKED)
-MSG-NB-335: "No invoice" (INVOICE_NOT_FOUND)
-MSG-NB-336: "Policy year &lt;policy year&gt; of &lt;arn&gt; is not due for booking" (POLICY_YEAR_NOT_DUE)
-MSG-NB-337: "Account &lt;arn&gt; has no rated premium" (PREMIUM_NOT_RATED)</t>
+MSG-NB-317: "Enter a booking date that is not in the future"
+MSG-NB-318: "Account &lt;arn&gt; has no insurer" (ACCOUNT_INSURER_MISSING)
+MSG-NB-319: "Account &lt;arn&gt; is &lt;&gt;: only issued policies are booked" (ACCOUNT_NOT_BOOKABLE)
+MSG-NB-320: "Account &lt;arn&gt; has no period of cover" (ACCOUNT_PERIOD_MISSING)
+MSG-NB-321: "Billing number &lt;billing no&gt; of &lt;insurer code&gt; is already on invoice &lt;invoice no&gt;" (BILLING_NO_DUPLICATE)
+MSG-NB-322: "Enter the insurer billing number" (BILLING_NO_REQUIRED)
+MSG-NB-323: "The insurer billing number has at most 60 characters" (BILLING_NO_TOO_LONG)
+MSG-NB-324: "The company has no branch to book invoices" (BOOKING_BRANCH_MISSING)
+MSG-NB-325: "The booking date &lt;date&gt; is in the future" (BOOKING_DATE_FUTURE)
+MSG-NB-326: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (CLIENT_PARTY_MISSING)
+MSG-NB-327: "Enter the cost center of account &lt;arn&gt;" (COST_CENTER_REQUIRED)
+MSG-NB-328: "Account &lt;arn&gt; is already booked" (DUPLICATE_BOOKING)
+MSG-NB-329: "No sub-ledger party &lt;code&gt; for invoice &lt;invoice no&gt;" (INSURER_PARTY_MISSING)
+MSG-NB-330: "Each insurer appears once with a positive share" (INSURER_SHARES_INVALID)
+MSG-NB-331: "Insurer shares must add up to 100% and include the lead insurer &lt;insurer code&gt;" (INSURER_SHARES_INVALID)
+MSG-NB-332: "Invoice &lt;arn&gt;/&lt;transaction no&gt; is &lt;status&gt;" (INVOICE_ALREADY_BOOKED)
+MSG-NB-333: "No invoice" (INVOICE_NOT_FOUND)
+MSG-NB-334: "Policy year &lt;policy year&gt; of &lt;arn&gt; is not due for booking" (POLICY_YEAR_NOT_DUE)
+MSG-NB-335: "Account &lt;arn&gt; has no rated premium" (PREMIUM_NOT_RATED)</t>
         </is>
       </c>
       <c r="M461" s="12" t="inlineStr">
@@ -50194,15 +50194,15 @@
       <c r="L462" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-343: "Account &lt;arn&gt; is &lt;&gt;: only booked accounts are endorsed" (ACCOUNT_NOT_BOOKED)
-MSG-NB-344: "A cancellation, and only a cancellation, has a kind" (CANCELLATION_KIND_REQUIRED)
-MSG-NB-345: "Enter the change of the sum insured or the premium" (ENDORSEMENT_CHANGE_REQUIRED)
-MSG-NB-346: "The effective date &lt;effective&gt; is not within a booked policy year of &lt;arn&gt;" (ENDORSEMENT_DATE_OUTSIDE_TERM)
-MSG-NB-347: "Enter the account, type, effective date and description" (ENDORSEMENT_INCOMPLETE)
-MSG-NB-348: "A negative endorsement or cancellation must return premium" (ENDORSEMENT_SIGN_MISMATCH)
-MSG-NB-349: "A positive endorsement must add premium" (ENDORSEMENT_SIGN_MISMATCH)
-MSG-NB-350: "The return premium exceeds the premium in force of policy year &lt;year&gt;" (RETURN_EXCEEDS_PREMIUM)
-MSG-NB-351: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
+MSG-NB-341: "Account &lt;arn&gt; is &lt;&gt;: only booked accounts are endorsed" (ACCOUNT_NOT_BOOKED)
+MSG-NB-342: "A cancellation, and only a cancellation, has a kind" (CANCELLATION_KIND_REQUIRED)
+MSG-NB-343: "Enter the change of the sum insured or the premium" (ENDORSEMENT_CHANGE_REQUIRED)
+MSG-NB-344: "The effective date &lt;effective&gt; is not within a booked policy year of &lt;arn&gt;" (ENDORSEMENT_DATE_OUTSIDE_TERM)
+MSG-NB-345: "Enter the account, type, effective date and description" (ENDORSEMENT_INCOMPLETE)
+MSG-NB-346: "A negative endorsement or cancellation must return premium" (ENDORSEMENT_SIGN_MISMATCH)
+MSG-NB-347: "A positive endorsement must add premium" (ENDORSEMENT_SIGN_MISMATCH)
+MSG-NB-348: "The return premium exceeds the premium in force of policy year &lt;year&gt;" (RETURN_EXCEEDS_PREMIUM)
+MSG-NB-349: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
         </is>
       </c>
       <c r="M462" s="12" t="inlineStr">
@@ -50277,14 +50277,14 @@
       <c r="L463" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-353: "Give the reason of the credit"
-MSG-NB-355: "Service invoice &lt;si no&gt; has &lt;commission&gt; commission and &lt;vat&gt; VAT left to credit" (CREDIT_EXCEEDS_INVOICE)
-MSG-NB-356: "&lt;si no&gt; is itself a credit" (CREDIT_OF_CREDIT)
-MSG-NB-357: "Service invoice not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-358: "Service invoice not found: &lt;si no&gt;" (NOT_FOUND)
-MSG-NB-359: "Service invoice type not found: &lt;code&gt;" (NOT_FOUND)
-MSG-NB-360: "Service invoices of type &lt;type code&gt; are issued automatically with the early remittance incentive" (SERVICE_INVOICE_AUTOMATIC_ONLY)
-MSG-NB-361: "Service invoice type &lt;code&gt; is inactive" (SERVICE_INVOICE_TYPE_INACTIVE)</t>
+MSG-NB-351: "Give the reason of the credit"
+MSG-NB-353: "Service invoice &lt;si no&gt; has &lt;commission&gt; commission and &lt;vat&gt; VAT left to credit" (CREDIT_EXCEEDS_INVOICE)
+MSG-NB-354: "&lt;si no&gt; is itself a credit" (CREDIT_OF_CREDIT)
+MSG-NB-355: "Service invoice not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-356: "Service invoice not found: &lt;si no&gt;" (NOT_FOUND)
+MSG-NB-357: "Service invoice type not found: &lt;code&gt;" (NOT_FOUND)
+MSG-NB-358: "Service invoices of type &lt;type code&gt; are issued automatically with the early remittance incentive" (SERVICE_INVOICE_AUTOMATIC_ONLY)
+MSG-NB-359: "Service invoice type &lt;code&gt; is inactive" (SERVICE_INVOICE_TYPE_INACTIVE)</t>
         </is>
       </c>
       <c r="M463" s="12" t="inlineStr">
@@ -50359,12 +50359,12 @@
       <c r="L464" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-364: "Service invoice type already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-365: "The period end must not be before the period start" (INCENTIVE_PERIOD_INVALID)
-MSG-NB-366: "Incentive rules are maintained in Product Maintenance &gt; Incentive Criteria" (INCENTIVE_RULES_FROZEN)
-MSG-NB-367: "Auto-booking rule not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-368: "Incentive rule not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-369: "Service invoice type not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-362: "Service invoice type already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-363: "The period end must not be before the period start" (INCENTIVE_PERIOD_INVALID)
+MSG-NB-364: "Incentive rules are maintained in Product Maintenance &gt; Incentive Criteria" (INCENTIVE_RULES_FROZEN)
+MSG-NB-365: "Auto-booking rule not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-366: "Incentive rule not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-367: "Service invoice type not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M464" s="12" t="inlineStr">
@@ -50439,32 +50439,32 @@
       <c r="L465" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-374: "Risk groups are numbers separated by ';'" (ACCEPTANCE_GROUP_INVALID)
-MSG-NB-375: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
-MSG-NB-376: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
-MSG-NB-377: "Business Type must be NEW_BUSINESS or RENEWAL" (BULK_BUSINESS_TYPE_INVALID)
-MSG-NB-378: "Enter an individual's name as 'Last, First'" (BULK_CLIENT_NAME_FORMAT)
-MSG-NB-379: "Give the Client Code or the Client Name" (BULK_CLIENT_REQUIRED)
-MSG-NB-380: "This file was already uploaded as &lt;job no&gt; (&lt;file name&gt;)" (BULK_DUPLICATE_FILE)
-MSG-NB-381: "The file has no data rows" (BULK_FILE_EMPTY)
-MSG-NB-382: "The file has no header row" (BULK_FILE_EMPTY)
-MSG-NB-383: "The file has &lt;size&gt; rows; the maximum is &lt;max&gt;" (BULK_FILE_TOO_LARGE)
-MSG-NB-384: "The spreadsheet has more than 100000 rows" (BULK_FILE_TOO_LARGE)
-MSG-NB-385: "Upload an Excel (.xlsx), OpenDocument (.ods), CSV (.csv) or text (.txt) file" (BULK_FILE_TYPE)
-MSG-NB-386: "The file cannot be read: &lt;message&gt;" (BULK_FILE_UNREADABLE)
-MSG-NB-387: "The file is not an OpenDocument spreadsheet" (BULK_FILE_UNREADABLE)
-MSG-NB-388: "Upload &lt;job no&gt; is already &lt;status&gt;" (BULK_JOB_CLOSED)
-MSG-NB-389: "Upload &lt;job no&gt; has not been committed yet" (BULK_JOB_NOT_COMPLETED)
-MSG-NB-390: "You are not allowed to use '&lt;title&gt;'" (BULK_NOT_PERMITTED)
-MSG-NB-391: "Choose the product of the upload" (BULK_PRODUCT_REQUIRED)
-MSG-NB-392: "The file does not follow the current template; missing column(s): &lt;missing&gt;" (BULK_TEMPLATE_MISMATCH)
-MSG-NB-393: "The fixed-width layout of this upload type has no fields" (BULK_TEXT_LAYOUT)
-MSG-NB-394: "The text file has no tab, pipe, semicolon or comma separated header line" (BULK_TEXT_LAYOUT)
-MSG-NB-395: "Action must be TAG or CANCEL" (FFY_ACTION_INVALID)
-MSG-NB-396: "No live account insures vehicle &lt;identifier&gt;" (FFY_VEHICLE_NOT_UNIQUE)
-MSG-NB-397: "Several accounts insure vehicle &lt;identifier&gt;: &lt;details&gt;" (FFY_VEHICLE_NOT_UNIQUE)
-MSG-NB-398: "Bulk job not found: &lt;job id&gt;" (NOT_FOUND)
-MSG-NB-399: "Bulk upload type not found: &lt;code&gt;" (NOT_FOUND)</t>
+MSG-NB-372: "Risk groups are numbers separated by ';'" (ACCEPTANCE_GROUP_INVALID)
+MSG-NB-373: "Account &lt;arn&gt; is &lt;&gt;" (ACCOUNT_NOT_EDITABLE)
+MSG-NB-374: "Account &lt;arn&gt; belongs to another company" (ACCOUNT_OTHER_COMPANY)
+MSG-NB-375: "Business Type must be NEW_BUSINESS or RENEWAL" (BULK_BUSINESS_TYPE_INVALID)
+MSG-NB-376: "Enter an individual's name as 'Last, First'" (BULK_CLIENT_NAME_FORMAT)
+MSG-NB-377: "Give the Client Code or the Client Name" (BULK_CLIENT_REQUIRED)
+MSG-NB-378: "This file was already uploaded as &lt;job no&gt; (&lt;file name&gt;)" (BULK_DUPLICATE_FILE)
+MSG-NB-379: "The file has no data rows" (BULK_FILE_EMPTY)
+MSG-NB-380: "The file has no header row" (BULK_FILE_EMPTY)
+MSG-NB-381: "The file has &lt;size&gt; rows; the maximum is &lt;max&gt;" (BULK_FILE_TOO_LARGE)
+MSG-NB-382: "The spreadsheet has more than 100000 rows" (BULK_FILE_TOO_LARGE)
+MSG-NB-383: "Upload an Excel (.xlsx), OpenDocument (.ods), CSV (.csv) or text (.txt) file" (BULK_FILE_TYPE)
+MSG-NB-384: "The file cannot be read: &lt;message&gt;" (BULK_FILE_UNREADABLE)
+MSG-NB-385: "The file is not an OpenDocument spreadsheet" (BULK_FILE_UNREADABLE)
+MSG-NB-386: "Upload &lt;job no&gt; is already &lt;status&gt;" (BULK_JOB_CLOSED)
+MSG-NB-387: "Upload &lt;job no&gt; has not been committed yet" (BULK_JOB_NOT_COMPLETED)
+MSG-NB-388: "You are not allowed to use '&lt;title&gt;'" (BULK_NOT_PERMITTED)
+MSG-NB-389: "Choose the product of the upload" (BULK_PRODUCT_REQUIRED)
+MSG-NB-390: "The file does not follow the current template; missing column(s): &lt;missing&gt;" (BULK_TEMPLATE_MISMATCH)
+MSG-NB-391: "The fixed-width layout of this upload type has no fields" (BULK_TEXT_LAYOUT)
+MSG-NB-392: "The text file has no tab, pipe, semicolon or comma separated header line" (BULK_TEXT_LAYOUT)
+MSG-NB-393: "Action must be TAG or CANCEL" (FFY_ACTION_INVALID)
+MSG-NB-394: "No live account insures vehicle &lt;identifier&gt;" (FFY_VEHICLE_NOT_UNIQUE)
+MSG-NB-395: "Several accounts insure vehicle &lt;identifier&gt;: &lt;details&gt;" (FFY_VEHICLE_NOT_UNIQUE)
+MSG-NB-396: "Bulk job not found: &lt;job id&gt;" (NOT_FOUND)
+MSG-NB-397: "Bulk upload type not found: &lt;code&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M465" s="12" t="inlineStr">
@@ -50527,18 +50527,18 @@
       <c r="L466" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-401: "The file content does not match its .&lt;type&gt; type" (ATTACHMENT_CONTENT_MISMATCH)
-MSG-NB-402: "The file is empty" (ATTACHMENT_EMPTY)
-MSG-NB-403: "The file was rejected by the malware scan: &lt;detail&gt;" (ATTACHMENT_INFECTED)
-MSG-NB-404: "Stored file failed its checksum verification" (ATTACHMENT_INTEGRITY_FAILURE)
-MSG-NB-405: "The file exceeds the maximum size of &lt;to megabytes&gt; MB" (ATTACHMENT_TOO_LARGE)
-MSG-NB-406: "Only these file types are allowed: &lt;allowed extensions&gt;" (ATTACHMENT_TYPE_NOT_ALLOWED)
-MSG-NB-407: "Select between 1 and 50 documents" (DOCUMENT_FILE_COUNT)
-MSG-NB-408: "Upload between 1 and 50 files at a time" (DOCUMENT_FILE_COUNT)
-MSG-NB-409: "A reference is needed to nominate the file names" (DOCUMENT_REFERENCE_REQUIRED)
-MSG-NB-410: "Invalid entity type or id" (INVALID_ATTACHMENT_TARGET)
-MSG-NB-411: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-412: "Attachment content not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-399: "The file content does not match its .&lt;type&gt; type" (ATTACHMENT_CONTENT_MISMATCH)
+MSG-NB-400: "The file is empty" (ATTACHMENT_EMPTY)
+MSG-NB-401: "The file was rejected by the malware scan: &lt;detail&gt;" (ATTACHMENT_INFECTED)
+MSG-NB-402: "Stored file failed its checksum verification" (ATTACHMENT_INTEGRITY_FAILURE)
+MSG-NB-403: "The file exceeds the maximum size of &lt;to megabytes&gt; MB" (ATTACHMENT_TOO_LARGE)
+MSG-NB-404: "Only these file types are allowed: &lt;allowed extensions&gt;" (ATTACHMENT_TYPE_NOT_ALLOWED)
+MSG-NB-405: "Select between 1 and 50 documents" (DOCUMENT_FILE_COUNT)
+MSG-NB-406: "Upload between 1 and 50 files at a time" (DOCUMENT_FILE_COUNT)
+MSG-NB-407: "A reference is needed to nominate the file names" (DOCUMENT_REFERENCE_REQUIRED)
+MSG-NB-408: "Invalid entity type or id" (INVALID_ATTACHMENT_TARGET)
+MSG-NB-409: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-410: "Attachment content not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M466" s="12" t="inlineStr">
@@ -50601,16 +50601,16 @@
       <c r="L467" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-414: "&lt;entity type&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-415: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
-MSG-NB-416: "Work item not found: &lt;case id&gt;" (NOT_FOUND)
-MSG-NB-417: "Workflow not found: &lt;workflow code&gt;" (NOT_FOUND)
-MSG-NB-418: "Workflow stage not found: &lt;stage code&gt;" (NOT_FOUND)
-MSG-NB-419: "'&lt;label&gt;' must be done from the record screen" (WORKFLOW_ACTION_NOT_GENERIC)
-MSG-NB-420: "You are not allowed to '&lt;label&gt;'" (WORKFLOW_ACTION_NOT_PERMITTED)
-MSG-NB-421: "Select a reason for '&lt;label&gt;'" (WORKFLOW_REASON_REQUIRED)
-MSG-NB-422: "'&lt;action&gt;' is not allowed while &lt;reference&gt; is in stage &lt;name&gt;" (WORKFLOW_TRANSITION_NOT_ALLOWED)
-MSG-NB-423: "The item is closed" (WORK_CASE_CLOSED)</t>
+MSG-NB-412: "&lt;entity type&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-413: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
+MSG-NB-414: "Work item not found: &lt;case id&gt;" (NOT_FOUND)
+MSG-NB-415: "Workflow not found: &lt;workflow code&gt;" (NOT_FOUND)
+MSG-NB-416: "Workflow stage not found: &lt;stage code&gt;" (NOT_FOUND)
+MSG-NB-417: "'&lt;label&gt;' must be done from the record screen" (WORKFLOW_ACTION_NOT_GENERIC)
+MSG-NB-418: "You are not allowed to '&lt;label&gt;'" (WORKFLOW_ACTION_NOT_PERMITTED)
+MSG-NB-419: "Select a reason for '&lt;label&gt;'" (WORKFLOW_REASON_REQUIRED)
+MSG-NB-420: "'&lt;action&gt;' is not allowed while &lt;reference&gt; is in stage &lt;name&gt;" (WORKFLOW_TRANSITION_NOT_ALLOWED)
+MSG-NB-421: "The item is closed" (WORK_CASE_CLOSED)</t>
         </is>
       </c>
       <c r="M467" s="12" t="inlineStr">
@@ -50685,10 +50685,10 @@
       <c r="L468" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-426: "Work item not found: &lt;case id&gt;" (NOT_FOUND)
-MSG-NB-427: "&lt;assignee&gt; does not work this queue" (WORK_ASSIGNEE_NOT_ELIGIBLE)
-MSG-NB-428: "The item is closed" (WORK_CASE_CLOSED)
-MSG-NB-429: "This item is not in your queue" (WORK_CLAIM_NOT_ALLOWED)</t>
+MSG-NB-424: "Work item not found: &lt;case id&gt;" (NOT_FOUND)
+MSG-NB-425: "&lt;assignee&gt; does not work this queue" (WORK_ASSIGNEE_NOT_ELIGIBLE)
+MSG-NB-426: "The item is closed" (WORK_CASE_CLOSED)
+MSG-NB-427: "This item is not in your queue" (WORK_CLAIM_NOT_ALLOWED)</t>
         </is>
       </c>
       <c r="M468" s="12" t="inlineStr">
@@ -50763,14 +50763,14 @@
       <c r="L469" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-432: "&lt;file name&gt; cannot be password protected. Send it as PDF, Excel or Word" (DOCUMENT_NOT_PROTECTABLE)
-MSG-NB-433: "Could not protect &lt;file name&gt;: &lt;message&gt;" (DOCUMENT_PROTECTION_FAILED)
-MSG-NB-434: "Invalid e-mail address: &lt;a&gt;" (EMAIL_ADDRESS_INVALID)
-MSG-NB-435: "Enter the &lt;field&gt;" (EMAIL_CONTENT_REQUIRED)
-MSG-NB-436: "Enter at least one recipient" (EMAIL_RECIPIENT_REQUIRED)
-MSG-NB-437: "Too many recipients" (EMAIL_TOO_MANY_RECIPIENTS)
-MSG-NB-438: "Only a failed message can be resent" (MESSAGE_NOT_FAILED)
-MSG-NB-439: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-430: "&lt;file name&gt; cannot be password protected. Send it as PDF, Excel or Word" (DOCUMENT_NOT_PROTECTABLE)
+MSG-NB-431: "Could not protect &lt;file name&gt;: &lt;message&gt;" (DOCUMENT_PROTECTION_FAILED)
+MSG-NB-432: "Invalid e-mail address: &lt;a&gt;" (EMAIL_ADDRESS_INVALID)
+MSG-NB-433: "Enter the &lt;field&gt;" (EMAIL_CONTENT_REQUIRED)
+MSG-NB-434: "Enter at least one recipient" (EMAIL_RECIPIENT_REQUIRED)
+MSG-NB-435: "Too many recipients" (EMAIL_TOO_MANY_RECIPIENTS)
+MSG-NB-436: "Only a failed message can be resent" (MESSAGE_NOT_FAILED)
+MSG-NB-437: "&lt;entity&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M469" s="12" t="inlineStr">
@@ -50845,17 +50845,17 @@
       <c r="L470" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-441: "Enter a whole number"
-MSG-NB-442: "Enter the first valid date"
-MSG-NB-443: "Enter the label"
-MSG-NB-444: "Must not be before the first valid date"
-MSG-NB-445: "Use capital letters, digits and _ (up to 40)"
-MSG-NB-446: "&lt;type code&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-NB-447: "The effective-to date is before the effective-from date" (LOV_EFFECTIVITY_INVALID)
-MSG-NB-448: "The list &lt;type code&gt; is maintained by the system" (LOV_NOT_MAINTAINABLE)
-MSG-NB-449: "'&lt;code&gt;' is not a valid value of &lt;type code&gt; on &lt;date&gt;" (LOV_VALUE_INVALID)
-MSG-NB-450: "List type not found: &lt;type code&gt;" (NOT_FOUND)
-MSG-NB-451: "List value not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-NB-439: "Enter a whole number"
+MSG-NB-440: "Enter the first valid date"
+MSG-NB-441: "Enter the label"
+MSG-NB-442: "Must not be before the first valid date"
+MSG-NB-443: "Use capital letters, digits and _ (up to 40)"
+MSG-NB-444: "&lt;type code&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-NB-445: "The effective-to date is before the effective-from date" (LOV_EFFECTIVITY_INVALID)
+MSG-NB-446: "The list &lt;type code&gt; is maintained by the system" (LOV_NOT_MAINTAINABLE)
+MSG-NB-447: "'&lt;code&gt;' is not a valid value of &lt;type code&gt; on &lt;date&gt;" (LOV_VALUE_INVALID)
+MSG-NB-448: "List type not found: &lt;type code&gt;" (NOT_FOUND)
+MSG-NB-449: "List value not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M470" s="12" t="inlineStr">
@@ -50930,13 +50930,13 @@
       <c r="L471" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-452: "Enter a whole number of bookings (0 or more)"
-MSG-NB-453: "Enter an amount of 0 or more"
-MSG-NB-454: "Enter the period"
-MSG-NB-455: "Enter the unit code or the officer username"
-MSG-NB-458: "The period end must not be before the start"
-MSG-NB-459: "Targets cannot be negative" (TARGET_NEGATIVE)
-MSG-NB-460: "The period end must not be before the period start" (TARGET_PERIOD_INVALID)</t>
+MSG-NB-450: "Enter a whole number of bookings (0 or more)"
+MSG-NB-451: "Enter an amount of 0 or more"
+MSG-NB-452: "Enter the period"
+MSG-NB-453: "Enter the unit code or the officer username"
+MSG-NB-456: "The period end must not be before the start"
+MSG-NB-457: "Targets cannot be negative" (TARGET_NEGATIVE)
+MSG-NB-458: "The period end must not be before the period start" (TARGET_PERIOD_INVALID)</t>
         </is>
       </c>
       <c r="M471" s="12" t="inlineStr">
@@ -51011,11 +51011,11 @@
       <c r="L472" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-461: "Enter a name"
-MSG-NB-462: "The saved parameter variant is deleted."
-MSG-NB-465: "Report variant not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-466: "Report &lt;report code&gt; is not available to you" (REPORT_NOT_AVAILABLE)
-MSG-NB-467: "Only the user who saved a report variant may delete it" (VARIANT_NOT_OWNER)</t>
+MSG-NB-459: "Enter a name"
+MSG-NB-460: "The saved parameter variant is deleted."
+MSG-NB-463: "Report variant not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-464: "Report &lt;report code&gt; is not available to you" (REPORT_NOT_AVAILABLE)
+MSG-NB-465: "Only the user who saved a report variant may delete it" (VARIANT_NOT_OWNER)</t>
         </is>
       </c>
       <c r="M472" s="12" t="inlineStr">
@@ -51090,13 +51090,13 @@
       <c r="L473" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-471: "This document cannot be produced in Word" (DOCUMENT_WORD_UNAVAILABLE)
-MSG-NB-472: "Document template not found: &lt;code&gt;" (NOT_FOUND)
-MSG-NB-473: "Document template not found: &lt;version no&gt;" (NOT_FOUND)
-MSG-NB-474: "Word copy of document not found: &lt;D&gt;" (NOT_FOUND)
-MSG-NB-475: "Enter the template text" (TEMPLATE_BODY_REQUIRED)
-MSG-NB-476: "The Word file needs the title in its first paragraph and the text below it" (TEMPLATE_WORD_INVALID)
-MSG-NB-477: "The file is not a Word (.docx) document" (TEMPLATE_WORD_INVALID)</t>
+MSG-NB-469: "This document cannot be produced in Word" (DOCUMENT_WORD_UNAVAILABLE)
+MSG-NB-470: "Document template not found: &lt;code&gt;" (NOT_FOUND)
+MSG-NB-471: "Document template not found: &lt;version no&gt;" (NOT_FOUND)
+MSG-NB-472: "Word copy of document not found: &lt;D&gt;" (NOT_FOUND)
+MSG-NB-473: "Enter the template text" (TEMPLATE_BODY_REQUIRED)
+MSG-NB-474: "The Word file needs the title in its first paragraph and the text below it" (TEMPLATE_WORD_INVALID)
+MSG-NB-475: "The file is not a Word (.docx) document" (TEMPLATE_WORD_INVALID)</t>
         </is>
       </c>
       <c r="M473" s="12" t="inlineStr">
@@ -51171,10 +51171,10 @@
       <c r="L474" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-479: "Between 0 and 50 years"
-MSG-NB-480: "Between 1 and 50 years"
-MSG-NB-481: "Enter a description"
-MSG-NB-482: "Enter at least one status"</t>
+MSG-NB-477: "Between 0 and 50 years"
+MSG-NB-478: "Between 1 and 50 years"
+MSG-NB-479: "Enter a description"
+MSG-NB-480: "Enter at least one status"</t>
         </is>
       </c>
       <c r="M474" s="12" t="inlineStr">
@@ -51237,13 +51237,13 @@
       <c r="L475" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-487: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-NB-488: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-NB-489: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
-MSG-NB-490: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-NB-491: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
-MSG-NB-492: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
-MSG-NB-493: "Invalid request" (VALIDATION_FAILED)</t>
+MSG-NB-485: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-NB-486: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-NB-487: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
+MSG-NB-488: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-NB-489: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-NB-490: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
+MSG-NB-491: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
       </c>
       <c r="M475" s="12" t="inlineStr">
@@ -51318,8 +51318,8 @@
       <c r="L476" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-501: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
-MSG-NB-502: "&lt;Column&gt; is mandatory"</t>
+MSG-NB-499: "&lt;Column&gt; '&lt;value&gt;' is not a valid &lt;number, date (yyyy-mm-dd), Y/N value&gt;"
+MSG-NB-500: "&lt;Column&gt; is mandatory"</t>
         </is>
       </c>
       <c r="M476" s="12" t="inlineStr">
@@ -51394,7 +51394,7 @@
       <c r="L477" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-503: "&lt;quotation no&gt; is &lt;&gt;, not sent to the client"</t>
+MSG-NB-501: "&lt;quotation no&gt; is &lt;&gt;, not sent to the client"</t>
         </is>
       </c>
       <c r="M477" s="12" t="inlineStr">
@@ -51469,8 +51469,8 @@
       <c r="L478" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-504: "Account &lt;arn&gt; belongs to another company"
-MSG-NB-507: "The booking date &lt;date&gt; is in the future"</t>
+MSG-NB-502: "Account &lt;arn&gt; belongs to another company"
+MSG-NB-505: "The booking date &lt;date&gt; is in the future"</t>
         </is>
       </c>
       <c r="M478" s="12" t="inlineStr">
@@ -51545,9 +51545,9 @@
       <c r="L479" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-505: "Client Type must be INDIVIDUAL or CORPORATE"
-MSG-NB-506: "Client code &lt;code&gt; does not exist"
-MSG-NB-508: "The row matches several clients: &lt;details&gt;"</t>
+MSG-NB-503: "Client Type must be INDIVIDUAL or CORPORATE"
+MSG-NB-504: "Client code &lt;code&gt; does not exist"
+MSG-NB-506: "The row matches several clients: &lt;details&gt;"</t>
         </is>
       </c>
       <c r="M479" s="12" t="inlineStr">
@@ -51610,26 +51610,26 @@
       <c r="L480" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-NB-509: "Legacy policy &lt;legacy ref&gt; is already imported" (ACCOUNT_LEGACY_IMPORTED)
-MSG-NB-510: "Account &lt;arn&gt; was not imported from legacy" (ACCOUNT_NOT_MIGRATED)
-MSG-NB-511: "Client &lt;code&gt; was not migrated" (CLIENT_NOT_MIGRATED)
-MSG-NB-512: "A migrated client needs its source system and legacy code" (CLIENT_ORIGIN_REQUIRED)
-MSG-NB-513: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
-MSG-NB-514: "Account not found: &lt;account id&gt;" (NOT_FOUND)
-MSG-NB-515: "Account not found: &lt;arn&gt;" (NOT_FOUND)
-MSG-NB-516: "Account not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-517: "Batch run not found: &lt;run no&gt;" (NOT_FOUND)
-MSG-NB-518: "Booked invoice not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-519: "Booked invoice not found: &lt;invoice no&gt;" (NOT_FOUND)
-MSG-NB-520: "Client not found: &lt;client id&gt;" (NOT_FOUND)
-MSG-NB-521: "Company not found: &lt;company id&gt;" (NOT_FOUND)
-MSG-NB-522: "Legacy account header not found: &lt;account id&gt;" (NOT_FOUND)
-MSG-NB-523: "Notification not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-524: "Proposal request not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-525: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
-MSG-NB-526: "Quotation not found: &lt;key&gt;" (NOT_FOUND)
-MSG-NB-527: "Quotation version not found: &lt;version no&gt;" (NOT_FOUND)
-MSG-NB-528: "Work item not found: &lt;case id&gt;" (NOT_FOUND)</t>
+MSG-NB-507: "Legacy policy &lt;legacy ref&gt; is already imported" (ACCOUNT_LEGACY_IMPORTED)
+MSG-NB-508: "Account &lt;arn&gt; was not imported from legacy" (ACCOUNT_NOT_MIGRATED)
+MSG-NB-509: "Client &lt;code&gt; was not migrated" (CLIENT_NOT_MIGRATED)
+MSG-NB-510: "A migrated client needs its source system and legacy code" (CLIENT_ORIGIN_REQUIRED)
+MSG-NB-511: "&lt;entity type&gt; work item not found: &lt;entity id&gt;" (NOT_FOUND)
+MSG-NB-512: "Account not found: &lt;account id&gt;" (NOT_FOUND)
+MSG-NB-513: "Account not found: &lt;arn&gt;" (NOT_FOUND)
+MSG-NB-514: "Account not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-515: "Batch run not found: &lt;run no&gt;" (NOT_FOUND)
+MSG-NB-516: "Booked invoice not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-517: "Booked invoice not found: &lt;invoice no&gt;" (NOT_FOUND)
+MSG-NB-518: "Client not found: &lt;client id&gt;" (NOT_FOUND)
+MSG-NB-519: "Company not found: &lt;company id&gt;" (NOT_FOUND)
+MSG-NB-520: "Legacy account header not found: &lt;account id&gt;" (NOT_FOUND)
+MSG-NB-521: "Notification not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-522: "Proposal request not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-523: "Quotation not found: &lt;id&gt;" (NOT_FOUND)
+MSG-NB-524: "Quotation not found: &lt;key&gt;" (NOT_FOUND)
+MSG-NB-525: "Quotation version not found: &lt;version no&gt;" (NOT_FOUND)
+MSG-NB-526: "Work item not found: &lt;case id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M480" s="12" t="inlineStr">

</xml_diff>